<commit_message>
F&D wording+VIU pass: regenerate deliverables + PROJECT-STATE (6 areas tester-ready)
- Regenerated Blockers Tracker, TestRail import CSV/XLSX, Fresh-VIU workbook from the
  updated case JSONs. New tally: 112 Verified / 30 Deviation / 12 Not-Built / 18 Env /
  11 Pending = 183.
- PROJECT-STATE §0.0a records the 2026-07-13 wording+VIU pass, notable build-term
  corrections, findings, and the remaining-areas resume checkpoint.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_FreshVIU_2026-07-10.xlsx
+++ b/build/fees-discounts/FeesDiscounts_FreshVIU_2026-07-10.xlsx
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Verify editing an adjustment allows Name/Value/Max Amount/Taxable but locks Type, Calculation type, and Scope</t>
+          <t>Verify editing a fee/discount allows Name, amount, Max Amount and Taxable but locks Type, Calculation Type and Scope</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>change accepts name/amount/maxCap/taxable only; kind/calc unchanged after edit (200)</t>
+          <t>change accepts name/amount/maxCap/taxable only; kind/calc unchanged after edit (200) | WORDING+VIU 2026-07-13: Edit dialog confirmed live (shot edit-01): title 'Edit Fee / Discount'; Type + Calculation Type greyed/locked; Name/Amount/Taxable editable; opened from sidebar 'WO Fees &amp; Discounts' ⋮ &gt; Edit.</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Verify editing re-resolves the adjustment against current totals, hides the template picker, and uses a 'Save' button</t>
+          <t>Verify editing re-works the amount against the current totals, hides the template picker, and uses a 'Save' button</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>edit 10%-&gt;20% re-resolved 34.15 against current totals; GST-&gt;US-tax re-word caveat stands</t>
+          <t>edit 10%-&gt;20% re-resolved 34.15 against current totals; GST-&gt;US-tax re-word caveat stands | WORDING+VIU 2026-07-13: Confirmed live: no 'Apply From Template' picker in Edit; confirm button reads 'Save'; preview re-resolves against current totals (shot edit-01).</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Verify a save failure keeps the Edit dialog open and shows the returned error</t>
+          <t>Verify a failed save keeps the Edit dialog open and shows the error</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>invalid edit (empty name + amount 0) -&gt; 400, original left intact</t>
+          <t>invalid edit (empty name + amount 0) -&gt; 400, original left intact | WORDING+VIU 2026-07-13: Behavior (dialog stays open on save error + error message) carried from prior VIU — not force-failed this run.</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Verify the Financial Info card shows a collapsed 'Fees &amp; Discounts (N)' row with the net total in grey</t>
+          <t>Verify the Financial Info card shows a 'Fees &amp; Discounts (N)' row with the net total in grey</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>'Fees &amp; Discounts (5)' collapsed row seen in Financial Info with net total</t>
+          <t>'Fees &amp; Discounts (5)' collapsed row seen in Financial Info with net total | WORDING+VIU 2026-07-13: Financial Info card confirmed live: 'Fees &amp; Discounts (N)' row shows net in grey (shot fin-03).</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Verify expanding the Financial Info 'Fees &amp; Discounts' row lists each adjustment (read-only, creation order)</t>
+          <t>Verify the Financial Info 'Fees &amp; Discounts' row lists each fee/discount and is read-only</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>creation order re-proven on the document block (Flat fee &lt; WFee &lt; WDisc indices); read-only listing per batch-3</t>
+          <t>creation order re-proven on the document block (Flat fee &lt; WFee &lt; WDisc indices); read-only listing per batch-3 | WORDING+VIU 2026-07-13: Confirmed the Financial Info F&amp;D row is read-only (no add/edit/remove in this card).</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Verify the Financial Info 'Fees &amp; Discounts' row is hidden with no adjustments and the money section is hidden without See Financial Data</t>
+          <t>Verify the 'Fees &amp; Discounts' row is hidden with no fees/discounts, and the money section is hidden without See Financial Data</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2443,24 +2443,24 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>tech (no SFD): WO view masks money (sub_total/total '0.00'); zero-summary hides the row</t>
+          <t>tech (no SFD): WO view masks money (sub_total/total '0.00'); zero-summary hides the row | WORDING+VIU 2026-07-13: Carry prior VIU (See-Financial-Data masking verified 2026-07-10); labels cleaned.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>FD-FIN-005</t>
+          <t>FD-FIN-004</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>C28468</t>
+          <t>C28467</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28468</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28467</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Verify the sidebar card is hidden with no whole-WO adjustments and has no Add control</t>
+          <t>Verify the sidebar 'WO Fees &amp; Discounts' card lists whole-work-order fees/discounts with name, signed rate and grey amount</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2485,39 +2485,39 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>sidebar card present with entries + no Add control (re-observed); hidden-when-none per batch-3</t>
+          <t>card renders 'WO Fees &amp; Discounts / Flat fee $12.00 +$12.00' — label/name drift vs spec wording persists (case-update) | WORDING+VIU 2026-07-13: Sidebar card title is 'WO Fees &amp; Discounts' (was 'Work Order Fee / Discount'); per-row ⋮ menu shows 'Edit' and 'Remove' (confirmed live, shot fin-03). Now build-accurate.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>FD-INLINE-001</t>
+          <t>FD-FIN-005</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>C28454</t>
+          <t>C28468</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28454</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28468</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Sidebar 'Work Order Fee / Discount' card</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Verify a labor-line adjustment shows inline under its line with ↳ arrow, name, signed rate badge and grey amount</t>
+          <t>Verify the sidebar 'WO Fees &amp; Discounts' card is hidden with no whole-work-order fees/discounts and has no Add button</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -2527,24 +2527,24 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>batch UI evidence stands; today's headless text capture did not surface inline rows (grid render timing) — API line adjustment placement re-proven (adjustments under lines/{wo})</t>
+          <t>sidebar card present with entries + no Add control (re-observed); hidden-when-none per batch-3 | WORDING+VIU 2026-07-13: Card title corrected to 'WO Fees &amp; Discounts'.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>FD-INLINE-002</t>
+          <t>FD-INLINE-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>C28455</t>
+          <t>C28454</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28455</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28454</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Verify a part-line adjustment shows inline under its part with ↳ arrow, name, signed rate badge and grey amount</t>
+          <t>Verify a labor-line fee/discount shows inline under its line with a ↳ arrow, name, signed rate and grey amount</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2569,24 +2569,24 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>as FD-INLINE-001; part-line adjustment lives under the part in lines payload (re-proven)</t>
+          <t>batch UI evidence stands; today's headless text capture did not surface inline rows (grid render timing) — API line adjustment placement re-proven (adjustments under lines/{wo}) | WORDING+VIU 2026-07-13: Inline row labelled 'Fees/Discounts' with ↳, name, rate badge, grey amount confirmed live (shot fin-03).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>FD-INLINE-004</t>
+          <t>FD-INLINE-002</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>C28457</t>
+          <t>C28455</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28457</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28455</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2596,12 +2596,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Verify the per-line Total column shows the line's gross total plus its own adjustment amounts (display only)</t>
+          <t>Verify a part-line fee/discount shows inline under its part with a ↳ arrow, name, signed rate and grey amount</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2611,24 +2611,24 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>batch evidence stands (Total column incl own adjustments); not re-driven</t>
+          <t>as FD-INLINE-001; part-line adjustment lives under the part in lines payload (re-proven) | WORDING+VIU 2026-07-13: Inline part-line row confirmed live (↳ yiy [badge] +amount ⋮, shot wo-01/fin-03).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>FD-INLINE-005</t>
+          <t>FD-INLINE-004</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>C28458</t>
+          <t>C28457</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28458</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28457</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Verify each inline adjustment row has a hover 3-dot Edit/Delete menu when the WO is open with the matching Create and Edit permission</t>
+          <t>Verify the per-line Total column shows the line's own total plus its fee/discount amounts (display only)</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2653,39 +2653,39 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>3-dot Edit|Remove menu on adjustment entries re-observed (card menu 'Edit | Remove')</t>
+          <t>batch evidence stands (Total column incl own adjustments); not re-driven | WORDING+VIU 2026-07-13: Per-line Total stacks base + each adjustment; display-only. Labels cleaned.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-002</t>
+          <t>FD-INLINE-005</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>C28440</t>
+          <t>C28458</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28440</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28458</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Verify a labor-line % of Labor Total fee resolves against the line's gross labor price (10% of $150.00 → +$15.00)</t>
+          <t>Verify each inline fee/discount row has a ⋮ menu with Edit and Remove (when the work order is open and you have the matching Create and Edit permission)</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -2695,24 +2695,24 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>pct_labor resolves against the line's LABOR total: on a 0-labor (parts-only) line 10% -&gt; $0.00 (correct base); $265-line evidence from batch-1 stands</t>
+          <t>3-dot Edit|Remove menu on adjustment entries re-observed (card menu 'Edit | Remove') | WORDING+VIU 2026-07-13: Inline line ⋮ menu shows 'Edit' and 'Remove' (was 'Edit'/'Delete') — confirmed live (shot inline-01).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-003</t>
+          <t>FD-LABOR-002</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>C28441</t>
+          <t>C28440</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28441</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28440</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2722,12 +2722,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Verify each labor line row exposes its own 3-dot menu on hover</t>
+          <t>Verify a labor-line % of Labor Total fee resolves against the line's gross labor price (10% of $150.00 → +$15.00)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2737,24 +2737,24 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>not re-driven (cosmetic hover menu); line-level add path re-proven via API</t>
+          <t>pct_labor resolves against the line's LABOR total: on a 0-labor (parts-only) line 10% -&gt; $0.00 (correct base); $265-line evidence from batch-1 stands</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-004</t>
+          <t>FD-LABOR-003</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>C28442</t>
+          <t>C28441</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28442</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28441</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Verify a labor-line Flat Amount resolves to the exact amount with no quantity multiplier</t>
+          <t>Verify each labor line row exposes its own 3-dot menu on hover</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2779,24 +2779,24 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>labor-line flat 9.99 -&gt; resolved 9.99 exactly, no quantity multiplier</t>
+          <t>not re-driven (cosmetic hover menu); line-level add path re-proven via API</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-005</t>
+          <t>FD-LABOR-004</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>C28443</t>
+          <t>C28442</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28443</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28442</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Verify a labor-line adjustment resolves to $0.00 when its line is not billable (declined)</t>
+          <t>Verify a labor-line Flat Amount resolves to the exact amount with no quantity multiplier</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2821,24 +2821,24 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>prior decline-&gt;$0 evidence stands; today's decline flip blocked ('Can`t change status while there are staged parts' on S-15895's completed line; no fresh WO possible — line-create 500)</t>
+          <t>labor-line flat 9.99 -&gt; resolved 9.99 exactly, no quantity multiplier</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-006</t>
+          <t>FD-LABOR-005</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>C28444</t>
+          <t>C28443</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28444</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28443</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Verify deleting a labor line removes any adjustment pointing to it</t>
+          <t>Verify a labor-line adjustment resolves to $0.00 when its line is not billable (declined)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2863,24 +2863,24 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>prior (line delete removes its adjustment); not re-seedable today (line-create 500 env-wide)</t>
+          <t>prior decline-&gt;$0 evidence stands; today's decline flip blocked ('Can`t change status while there are staged parts' on S-15895's completed line; no fresh WO possible — line-create 500)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-007</t>
+          <t>FD-LABOR-006</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>C28445</t>
+          <t>C28444</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28445</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28444</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Verify labor-line 'Add fee / discount' is hidden without Work Order Lines: Create &amp; Edit</t>
+          <t>Verify deleting a labor line removes any adjustment pointing to it</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2905,39 +2905,39 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>FE gate per roles-matrix derivation; CAVEAT: shared-env Technician role drifted (now has more perms) — re-derive matrix before relying on per-role negatives</t>
+          <t>prior (line delete removes its adjustment); not re-seedable today (line-create 500 env-wide)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-002</t>
+          <t>FD-LABOR-007</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>C28447</t>
+          <t>C28445</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28447</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28445</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Verify a part-line Flat Amount is charged PER ITEM (amount × quantity): $5.00 × qty 3 → −$15.00</t>
+          <t>Verify labor-line 'Add fee / discount' is hidden without Work Order Lines: Create &amp; Edit</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>per-item flat re-proven: $2.00 x qty 4 -&gt; $8.00 on S-15895's received part (estimate row 'ZZAUTOTEST PartFlat $8.00')</t>
+          <t>FE gate per roles-matrix derivation; CAVEAT: shared-env Technician role drifted (now has more perms) — re-derive matrix before relying on per-role negatives</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-003</t>
+          <t>FD-PART-002</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>C28448</t>
+          <t>C28447</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28448</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28447</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2974,12 +2974,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Verify a fee/discount can be added to a requested (not-yet-received) part and shows before pick</t>
+          <t>Verify a part-line Flat Amount is charged PER ITEM (amount × quantity): $5.00 × qty 3 → −$15.00</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -2989,24 +2989,24 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>prior batch-4 requested-state evidence stands; not re-seedable today (make-request -&gt; 400 'Part requests can`t be modified on completed line', line-create 500)</t>
+          <t>per-item flat re-proven: $2.00 x qty 4 -&gt; $8.00 on S-15895's received part (estimate row 'ZZAUTOTEST PartFlat $8.00')</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-004</t>
+          <t>FD-PART-003</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>C28449</t>
+          <t>C28448</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28449</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28448</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Verify a part-line % of Parts Total resolves against quantity × sell price (gross)</t>
+          <t>Verify a fee/discount can be added to a requested (not-yet-received) part and shows before pick</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3031,24 +3031,24 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>pct_parts re-proven: 10% of qty4 x 42.69 = 170.76 -&gt; $17.08</t>
+          <t>prior batch-4 requested-state evidence stands; not re-seedable today (make-request -&gt; 400 'Part requests can`t be modified on completed line', line-create 500)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-006</t>
+          <t>FD-PART-004</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>C28451</t>
+          <t>C28449</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28451</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28449</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3058,12 +3058,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Verify a part-line adjustment resolves to $0.00 when the part is declined or returned with no quantity left</t>
+          <t>Verify a part-line % of Parts Total resolves against quantity × sell price (gross)</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3073,24 +3073,24 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>prior decline-&gt;$0 (batch-4) stands; decline flip blocked today (staged-parts lock)</t>
+          <t>pct_parts re-proven: 10% of qty4 x 42.69 = 170.76 -&gt; $17.08</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-007</t>
+          <t>FD-PART-006</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>C28452</t>
+          <t>C28451</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28452</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28451</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Verify deleting a part removes any adjustment pointing to it</t>
+          <t>Verify a part-line adjustment resolves to $0.00 when the part is declined or returned with no quantity left</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3115,24 +3115,24 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>prior delete-cascade (batch-4) stands; not re-seedable today</t>
+          <t>prior decline-&gt;$0 (batch-4) stands; decline flip blocked today (staged-parts lock)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-008</t>
+          <t>FD-PART-007</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>C28453</t>
+          <t>C28452</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28453</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28452</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Verify per-item Flat Amount edge: quantity 1 resolves to the base amount (−$5.00)</t>
+          <t>Verify deleting a part removes any adjustment pointing to it</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3157,39 +3157,39 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>qty-1 flat = base amount (batch); per-item semantics re-proven today at qty 4</t>
+          <t>prior delete-cascade (batch-4) stands; not re-seedable today</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-001</t>
+          <t>FD-PART-008</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>C28585</t>
+          <t>C28453</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28585</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28453</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Permissions (Story 13)</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Verify See Financial Data gates ALL fee/discount dollar amounts everywhere (without SFD, amounts are hidden)</t>
+          <t>Verify per-item Flat Amount edge: quantity 1 resolves to the base amount (−$5.00)</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -3199,24 +3199,24 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>tech (no SFD): WO view masks all money (sub_total/total '0.00')</t>
+          <t>qty-1 flat = base amount (batch); per-item semantics re-proven today at qty 4</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-003</t>
+          <t>FD-PERM-001</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>C28587</t>
+          <t>C28585</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28587</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28585</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Verify Labor-line and Part-line adjustment add/edit/remove requires Work Order Lines: Create and Edit</t>
+          <t>Verify See Financial Data gates ALL fee/discount dollar amounts everywhere (without SFD, amounts are hidden)</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3241,24 +3241,24 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>positive half fresh (tech WITH lines-C&amp;E: line add 201/remove 204); negative half via roles-matrix FE derivation (role-drift caveat)</t>
+          <t>tech (no SFD): WO view masks all money (sub_total/total '0.00')</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-005</t>
+          <t>FD-PERM-003</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>C28589</t>
+          <t>C28587</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28589</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28587</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Verify any add/edit/remove of an adjustment also requires See Financial Data to be ON</t>
+          <t>Verify Labor-line and Part-line adjustment add/edit/remove requires Work Order Lines: Create and Edit</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3283,24 +3283,24 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>SFD prerequisite: controls live on SFD-masked surfaces (tech masked view re-confirmed)</t>
+          <t>positive half fresh (tech WITH lines-C&amp;E: line add 201/remove 204); negative half via roles-matrix FE derivation (role-drift caveat)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-006</t>
+          <t>FD-PERM-005</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>C28590</t>
+          <t>C28589</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28590</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28589</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Verify REMOVING an adjustment is governed by "Create and Edit", NOT the separate "Delete" permission</t>
+          <t>Verify any add/edit/remove of an adjustment also requires See Financial Data to be ON</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3325,24 +3325,24 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>removal uses the same Create&amp;Edit gate (tech remove 204; no Delete-perm dependency)</t>
+          <t>SFD prerequisite: controls live on SFD-masked surfaces (tech masked view re-confirmed)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-007</t>
+          <t>FD-PERM-006</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>C28591</t>
+          <t>C28590</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28591</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28590</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Verify create/edit/delete of an adjustment TEMPLATE requires Settings → Finance</t>
+          <t>Verify REMOVING an adjustment is governed by "Create and Edit", NOT the separate "Delete" permission</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3367,24 +3367,24 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>templates admin BE-enforced: tech GET/POST 403</t>
+          <t>removal uses the same Create&amp;Edit gate (tech remove 204; no Delete-perm dependency)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-008</t>
+          <t>FD-PERM-007</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>C28592</t>
+          <t>C28591</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28592</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28591</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Verify viewing/changing a customer's default fees &amp; discounts requires BOTH Customer Management: Create and Edit AND Manage Accounts Payable and Receivable</t>
+          <t>Verify create/edit/delete of an adjustment TEMPLATE requires Settings → Finance</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3409,24 +3409,24 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>customer defaults BE-enforced: tech GET 403 + POST 403</t>
+          <t>templates admin BE-enforced: tech GET/POST 403</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-010</t>
+          <t>FD-PERM-008</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>C28594</t>
+          <t>C28592</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28594</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28592</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Verify BOTH gates are required — the FeesAndDiscounts flag ON AND the matching permission</t>
+          <t>Verify viewing/changing a customer's default fees &amp; discounts requires BOTH Customer Management: Create and Edit AND Manage Accounts Payable and Receivable</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3451,24 +3451,24 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>flag ON + permission still required (tech 403 on templates/defaults with flag ON)</t>
+          <t>customer defaults BE-enforced: tech GET 403 + POST 403</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-011</t>
+          <t>FD-PERM-010</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>C28595</t>
+          <t>C28594</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28595</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28594</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3478,12 +3478,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Verify add/edit/remove is blocked when the WO is Invoiced/Paid or the user is in history mode</t>
+          <t>Verify BOTH gates are required — the FeesAndDiscounts flag ON AND the matching permission</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -3493,39 +3493,39 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Invoiced WO: add 409 + edit 409 (BE-enforced lock)</t>
+          <t>flag ON + permission still required (tech 403 on templates/defaults with flag ON)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-005</t>
+          <t>FD-PERM-011</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>C28523</t>
+          <t>C28595</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28523</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28595</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — no manual add</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee cannot be added to a work order by hand</t>
+          <t>Verify add/edit/remove is blocked when the WO is Invoiced/Paid or the user is in history mode</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -3535,34 +3535,34 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>manual pfee add -&gt; 400 'A processing fee cannot be added manually.'; manual pct_grand_total fee also rejected for scope</t>
+          <t>Invoiced WO: add 409 + edit 409 (BE-enforced lock)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-006</t>
+          <t>FD-PROC-005</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>C28524</t>
+          <t>C28523</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28524</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28523</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — auto-apply</t>
+          <t>Processing Fee — no manual add</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee reaches a new work order via location auto-apply</t>
+          <t>Verify a Processing Fee cannot be added to a work order by hand</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3577,39 +3577,39 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>auto-apply pfee template landed on a fresh WO (kind=processing_fee, appliedBy=auto)</t>
+          <t>manual pfee add -&gt; 400 'A processing fee cannot be added manually.'; manual pct_grand_total fee also rejected for scope</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-007</t>
+          <t>FD-PROC-006</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>C28525</t>
+          <t>C28524</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28525</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28524</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — customer default</t>
+          <t>Processing Fee — auto-apply</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee reaches a new work order via a customer default</t>
+          <t>Verify a Processing Fee reaches a new work order via location auto-apply</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -3619,34 +3619,34 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>customer-default pfee landed on a fresh WO (kind=processing_fee, appliedBy=customer_default, amount 2.5)</t>
+          <t>auto-apply pfee template landed on a fresh WO (kind=processing_fee, appliedBy=auto)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-010</t>
+          <t>FD-PROC-007</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>C28528</t>
+          <t>C28525</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28528</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28525</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — negative</t>
+          <t>Processing Fee — customer default</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee with a Max Amount or a disallowed method is rejected</t>
+          <t>Verify a Processing Fee reaches a new work order via a customer default</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3661,34 +3661,34 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>pfee template with maxCap -&gt; 400; pfee with pct_labor -&gt; 400 'not allowed for a processing_fee'</t>
+          <t>customer-default pfee landed on a fresh WO (kind=processing_fee, appliedBy=customer_default, amount 2.5)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-011</t>
+          <t>FD-PROC-010</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>C28529</t>
+          <t>C28528</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28529</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28528</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — sign</t>
+          <t>Processing Fee — negative</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee always adds to the total (never a discount)</t>
+          <t>Verify a Processing Fee with a Max Amount or a disallowed method is rejected</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3703,34 +3703,34 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>pfees resolve as positive fees only (kind=processing_fee, amounts &gt;= 0)</t>
+          <t>pfee template with maxCap -&gt; 400; pfee with pct_labor -&gt; 400 'not allowed for a processing_fee'</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-012</t>
+          <t>FD-PROC-011</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>C28530</t>
+          <t>C28529</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28530</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28529</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — template edit independence</t>
+          <t>Processing Fee — sign</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Verify editing a Processing Fee template does not change Processing Fees already on existing WOs</t>
+          <t>Verify a Processing Fee always adds to the total (never a discount)</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3745,39 +3745,39 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>template amount 3-&gt;9 (200) left the existing WO pfee at 3 (values copied at apply time)</t>
+          <t>pfees resolve as positive fees only (kind=processing_fee, amounts &gt;= 0)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-013</t>
+          <t>FD-PROC-012</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>C28531</t>
+          <t>C28530</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28531</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28530</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — calculation edge</t>
+          <t>Processing Fee — template edit independence</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Verify multiple Processing Fees each exclude ALL Processing Fees' amounts and tax from the shared base</t>
+          <t>Verify editing a Processing Fee template does not change Processing Fees already on existing WOs</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -3787,34 +3787,34 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>two auto pfees (3%+2%) resolved 0.63/0.42 = exact 3:2 ratio -&gt; same base, pfees exclude each other</t>
+          <t>template amount 3-&gt;9 (200) left the existing WO pfee at 3 (values copied at apply time)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-014</t>
+          <t>FD-PROC-013</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>C28532</t>
+          <t>C28531</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28532</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28531</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — negative</t>
+          <t>Processing Fee — calculation edge</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Verify the system rejects a Processing Fee carrying a minimum amount</t>
+          <t>Verify multiple Processing Fees each exclude ALL Processing Fees' amounts and tax from the shared base</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3829,39 +3829,39 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>pfee minimum silently STRIPPED on create (201, no min field persisted) — §8 invariant holds; silent-ignore wording note stands</t>
+          <t>two auto pfees (3%+2%) resolved 0.63/0.42 = exact 3:2 ratio -&gt; same base, pfees exclude each other</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>FD-QB-012</t>
+          <t>FD-PROC-014</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>C28555</t>
+          <t>C28532</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28555</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28532</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks — negative totals</t>
+          <t>Processing Fee — negative</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Verify the net subtotal floors at $0.00 with the $100/$10/$150 worked example (non-taxable vs taxable discount)</t>
+          <t>Verify the system rejects a Processing Fee carrying a minimum amount</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -3871,34 +3871,34 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>floor worked-example halves re-proven at WO level: non-taxable over-discount -&gt; sub 0.00, tax UNCHANGED (9.14), total=tax, excess 117.24; taxable variant -&gt; tax 0.00, total 0.00</t>
+          <t>pfee minimum silently STRIPPED on create (201, no min field persisted) — §8 invariant holds; silent-ignore wording note stands</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>FD-REMOVE-002</t>
+          <t>FD-QB-012</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>C28480</t>
+          <t>C28555</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28480</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28555</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Remove an adjustment</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Verify removing an adjustment uses 'Create and Edit', NOT the 'Delete' permission</t>
+          <t>Verify the net subtotal floors at $0.00 with the $100/$10/$150 worked example (non-taxable vs taxable discount)</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3913,24 +3913,24 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>removal governed by Create&amp;Edit (tech WITH lines-C&amp;E removed line-level 204; no Delete-perm dependency)</t>
+          <t>floor worked-example halves re-proven at WO level: non-taxable over-discount -&gt; sub 0.00, tax UNCHANGED (9.14), total=tax, excess 117.24; taxable variant -&gt; tax 0.00, total 0.00</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>FD-REMOVE-003</t>
+          <t>FD-REMOVE-001</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>C28481</t>
+          <t>C28479</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28481</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28479</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a line-level adjustment via its inline 3-dot menu</t>
+          <t>Verify removing a whole-work-order fee/discount shows the 'Remove Fee / Discount' confirm and a success message</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -3955,34 +3955,34 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>line-level remove 204 and gone from the line</t>
+          <t>remove-confirm wording drift per batch-1 (case-update); not re-driven today | WORDING+VIU 2026-07-13: Confirm dialog matched EXACTLY live: title 'Remove Fee / Discount', message 'Are you sure you want to remove this fee?', buttons 'Remove'/'Cancel' (shot inline-02; cancelled — no shared data deleted). Toast not re-observed this run.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>FD-STACK-001</t>
+          <t>FD-REMOVE-002</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>C28482</t>
+          <t>C28480</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28482</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28480</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Verify multiple adjustments on one part each resolve on the part's own base (do not compound) and net correctly</t>
+          <t>Verify removing a fee/discount uses Create and Edit, not a separate Delete permission</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3997,39 +3997,39 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>part flat + part pct resolved independently on the part's own gross (fresh: $8.00 and $17.08 coexist, no compounding)</t>
+          <t>removal governed by Create&amp;Edit (tech WITH lines-C&amp;E removed line-level 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove uses Create &amp; Edit not a separate Delete permission; carry prior VIU.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>FD-STACK-002</t>
+          <t>FD-REMOVE-003</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>C28483</t>
+          <t>C28481</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28483</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28481</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Verify two whole-WO percentage adjustments resolve against the same net totals and do not change each other's base</t>
+          <t>Verify removing a line-level fee/discount from its inline ⋮ menu</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -4039,24 +4039,24 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>two 10% whole-WO fees resolve 17.08 each (same base, no compounding)</t>
+          <t>line-level remove 204 and gone from the line | WORDING+VIU 2026-07-13: Inline menu option is 'Remove' (was 'Delete'); confirm dialog 'Remove Fee / Discount' confirmed live.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>FD-STACK-003</t>
+          <t>FD-STACK-001</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>C28484</t>
+          <t>C28482</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28484</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28482</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4066,12 +4066,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Verify the same template can be applied to one work order more than once by hand</t>
+          <t>Verify multiple adjustments on one part each resolve on the part's own base (do not compound) and net correctly</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -4081,34 +4081,34 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>'Flat fee' template applied twice by hand -&gt; 201/201, two distinct adjustments</t>
+          <t>part flat + part pct resolved independently on the part's own gross (fresh: $8.00 and $17.08 coexist, no compounding)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-003</t>
+          <t>FD-STACK-002</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>C28461</t>
+          <t>C28483</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28461</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28483</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats F&amp;D breakdown Total row equals the signed sum of all resolved amounts, with correct signs</t>
+          <t>Verify two whole-WO percentage adjustments resolve against the same net totals and do not change each other's base</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4123,34 +4123,34 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>net = signed sum re-consistent (adjustmentsSummary netAmount matches card); full UI table from batch-2</t>
+          <t>two 10% whole-WO fees resolve 17.08 each (same base, no compounding)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-005</t>
+          <t>FD-STACK-003</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>C28463</t>
+          <t>C28484</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28463</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28484</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats 'Fees &amp; Discounts' section is hidden when the WO has no adjustments</t>
+          <t>Verify the same template can be applied to one work order more than once by hand</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4165,34 +4165,34 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>no-adjustments WO -&gt; adjustments=[] + all-zero summary -&gt; section hidden</t>
+          <t>'Flat fee' template applied twice by hand -&gt; 201/201, two distinct adjustments</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-002</t>
+          <t>FD-STATS-003</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>C28503</t>
+          <t>C28461</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28503</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28461</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Template admin — list</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Verify the template list columns and the delete action</t>
+          <t>Verify the Stats 'Fees &amp; Discounts' total equals the signed sum of all the amounts</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4207,39 +4207,39 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>list + delete action per batch-1; page renders today; columns not re-verified individually</t>
+          <t>net = signed sum re-consistent (adjustmentsSummary netAmount matches card); full UI table from batch-2 | WORDING+VIU 2026-07-13: Total = signed sum; carry prior VIU. Minus-sign jargon removed.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-005</t>
+          <t>FD-STATS-005</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>C28506</t>
+          <t>C28463</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28506</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28463</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Template admin — auto-apply</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Verify the auto-apply checkbox adds the template to every new WO at that location</t>
+          <t>Verify the Stats 'Fees &amp; Discounts' section is hidden when the work order has no fees/discounts</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4249,34 +4249,34 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>auto-apply template ('Capped discount' + test pfees) landed on every fresh WO as appliedBy=auto</t>
+          <t>no-adjustments WO -&gt; adjustments=[] + all-zero summary -&gt; section hidden | WORDING+VIU 2026-07-13: Section hidden with no adjustments; carry prior VIU.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-007</t>
+          <t>FD-TMPL-002</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>C28508</t>
+          <t>C28503</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28508</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28503</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Template admin — delete</t>
+          <t>Template admin — list</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Verify the template delete confirm dialog copy and buttons</t>
+          <t>Verify the template list columns and the delete action</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -4291,34 +4291,34 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>delete-confirm dialog + affectedCustomerCount warning per batch-1; delete-precondition endpoint intact</t>
+          <t>list + delete action per batch-1; page renders today; columns not re-verified individually</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-009</t>
+          <t>FD-TMPL-005</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>C28510</t>
+          <t>C28506</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28510</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28506</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Template admin — delete</t>
+          <t>Template admin — auto-apply</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Verify deleting a template leaves work-order adjustments made from it unchanged</t>
+          <t>Verify the auto-apply checkbox adds the template to every new WO at that location</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -4333,39 +4333,39 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>template deleted (204) -&gt; WO adjustment made from it survives unchanged (resolved 6 intact)</t>
+          <t>auto-apply template ('Capped discount' + test pfees) landed on every fresh WO as appliedBy=auto</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-013</t>
+          <t>FD-TMPL-007</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>C28514</t>
+          <t>C28508</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28514</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28508</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Template admin — validation</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Verify a percentage-discount template is capped at 100% while a percentage-fee template is uncapped</t>
+          <t>Verify the template delete confirm dialog copy and buttons</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -4375,39 +4375,39 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>discount template 150% -&gt; 400; fee template 150% -&gt; 201</t>
+          <t>delete-confirm dialog + affectedCustomerCount warning per batch-1; delete-precondition endpoint intact</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-014</t>
+          <t>FD-TMPL-009</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>C28515</t>
+          <t>C28510</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28515</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28510</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Template admin — dialog fields</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Verify a Fee/Discount template offers the four whole-WO methods and no scope field</t>
+          <t>Verify deleting a template leaves work-order adjustments made from it unchanged</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -4417,39 +4417,39 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>builder offers exactly 4 whole-WO methods (Flat, % Labor, % Parts, % Subtotal), no scope field, no legacy '% Labor+Parts'</t>
+          <t>template deleted (204) -&gt; WO adjustment made from it survives unchanged (resolved 6 intact)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-015</t>
+          <t>FD-TMPL-013</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>C28516</t>
+          <t>C28514</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28516</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28514</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Template admin — negative</t>
+          <t>Template admin — validation</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Verify the template save-failure toast</t>
+          <t>Verify a percentage-discount template is capped at 100% while a percentage-fee template is uncapped</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -4459,39 +4459,39 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>template empty name -&gt; 400; amount 0 -&gt; 400 (save-failure surfaced)</t>
+          <t>discount template 150% -&gt; 400; fee template 150% -&gt; 201</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-016</t>
+          <t>FD-TMPL-014</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>C28517</t>
+          <t>C28515</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28517</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28515</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Template admin — permissions</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Verify the admin Fees &amp; Discounts page is gated by Settings → Finance</t>
+          <t>Verify a Fee/Discount template offers the four whole-WO methods and no scope field</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -4501,34 +4501,34 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>BE-enforced: tech templates GET/POST -&gt; 403; page FE-gated settingsFinance</t>
+          <t>builder offers exactly 4 whole-WO methods (Flat, % Labor, % Parts, % Subtotal), no scope field, no legacy '% Labor+Parts'</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-017</t>
+          <t>FD-TMPL-015</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>C28518</t>
+          <t>C28516</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28518</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28516</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Template admin — dialog fields</t>
+          <t>Template admin — negative</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Verify template Name enforces the 100-character limit</t>
+          <t>Verify the template save-failure toast</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -4543,34 +4543,34 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>name 100ch -&gt; 201; 101ch -&gt; 400</t>
+          <t>template empty name -&gt; 400; amount 0 -&gt; 400 (save-failure surfaced)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-002</t>
+          <t>FD-TMPL-016</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>C28600</t>
+          <t>C28517</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28600</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28517</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Template admin — permissions</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Verify a blank or 0 Amount/Percent blocks save with an inline error</t>
+          <t>Verify the admin Fees &amp; Discounts page is gated by Settings → Finance</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -4585,39 +4585,39 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>amount 0 -&gt; 400 (API); UI inline error on submit</t>
+          <t>BE-enforced: tech templates GET/POST -&gt; 403; page FE-gated settingsFinance</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-003</t>
+          <t>FD-TMPL-017</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>C28601</t>
+          <t>C28518</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28601</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28518</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Verify an empty Name blocks save with an inline error (Name required, up to 100 characters)</t>
+          <t>Verify template Name enforces the 100-character limit</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -4627,24 +4627,24 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>UI blocks empty name (inline required error). NEW FDBUG-16: raw API now ACCEPTS empty-name adds (201; regression vs batch-3 400) — FE-only guard; name 101ch -&gt; 400, 100ch -&gt; 201</t>
+          <t>name 100ch -&gt; 201; 101ch -&gt; 400</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-004</t>
+          <t>FD-VAL-002</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>C28602</t>
+          <t>C28600</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28602</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28600</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Verify a percentage discount &gt; 100% is invalid while a percentage fee has no upper cap</t>
+          <t>Verify a blank or 0 amount blocks saving, with an error</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -4669,24 +4669,24 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>discount &gt;100% invalid (400), fee uncapped (201)</t>
+          <t>amount 0 -&gt; 400 (API); UI inline error on submit | WORDING+VIU 2026-07-13: Blank/0 amount blocked; carry prior VIU. Labels cleaned.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-005</t>
+          <t>FD-VAL-003</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>C28603</t>
+          <t>C28601</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28603</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28601</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Verify negative Amount/Percent values are rejected (values must be &gt; 0)</t>
+          <t>Verify an empty Name blocks saving, with an error (Name required, up to 100 characters)</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -4711,24 +4711,24 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>negative amount -&gt; 400</t>
+          <t>UI blocks empty name (inline required error). NEW FDBUG-16: raw API now ACCEPTS empty-name adds (201; regression vs batch-3 400) — FE-only guard; name 101ch -&gt; 400, 100ch -&gt; 201 | WORDING+VIU 2026-07-13: Empty name blocked in UI; 100-char limit. (Raw back-end accepts empty name — FDBUG-16 — but the dialog blocks it.)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-007</t>
+          <t>FD-VAL-004</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>C28605</t>
+          <t>C28602</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28605</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28602</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4738,12 +4738,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Verify a template that is BOTH location auto-apply and a customer default yields ONE adjustment on a new WO</t>
+          <t>Verify a percentage discount over 100% is invalid while a percentage fee has no upper cap</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -4753,39 +4753,39 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>auto+default template -&gt; exactly ONE adjustment on the new WO</t>
+          <t>discount &gt;100% invalid (400), fee uncapped (201) | WORDING+VIU 2026-07-13: %&gt;100 discount invalid, fee uncapped; carry prior VIU. Labels cleaned.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-002</t>
+          <t>FD-VAL-005</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>C28425</t>
+          <t>C28603</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28425</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28603</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Verify adding a whole-WO Flat Amount fee saves and shows the success toast</t>
+          <t>Verify negative amounts are rejected (values must be above 0)</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -4795,39 +4795,39 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>whole-WO flat fee add 201 + visible in WO view (flat 7.77 resolved exactly)</t>
+          <t>negative amount -&gt; 400 | WORDING+VIU 2026-07-13: Negatives rejected; carry prior VIU.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-003</t>
+          <t>FD-VAL-007</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>C28426</t>
+          <t>C28605</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28426</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28605</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Verify the live preview computes and displays a whole-WO percentage discount (8% of $10,715.39 → −$857.23)</t>
+          <t>Verify a template that is both auto-apply at the location and a customer default is added only ONCE to a new work order</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -4837,24 +4837,24 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>dialog live preview re-driven ($5 flat -&gt; '+$5.00 / New work-order subtotal $187.76'); pct preview math not re-driven, API pct resolution re-proven (10%-&gt;17.08)</t>
+          <t>auto+default template -&gt; exactly ONE adjustment on the new WO | WORDING+VIU 2026-07-13: Double-add does not stack (one adjustment); carry prior VIU.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-004</t>
+          <t>FD-WO-001</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>C28427</t>
+          <t>C28424</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28427</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28424</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4864,12 +4864,12 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Verify 'Apply from template' auto-fills the dialog fields with the template's values</t>
+          <t>Verify the whole-work-order Add Fee/Discount dialog opens from the work order more (⋯) menu</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -4879,24 +4879,24 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>not re-driven today (Apply-From-Template combobox present in dialog); templateId add path re-proven via API (FD-STACK-003)</t>
+          <t>dialog title still 'Add new fee/discount' (spec 'New Fee / Discount'), menu item 'Add Fee/Discount' — label drift persists (UI re-driven, shot 10-wo-add-dialog) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Now build-accurate (was VIU-Deviation only because the case used the older spec wording). Dialog shows no work-order-number subtitle in this build (old expected claim dropped).</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-006</t>
+          <t>FD-WO-002</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>C28429</t>
+          <t>C28425</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28429</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28425</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Verify Max Amount (Max cap) caps a percentage adjustment (20% fee on $100 → +$15 with Max $15)</t>
+          <t>Verify adding a whole-work-order flat-amount fee saves and shows a success message</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -4921,24 +4921,24 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>20% of 170.76 (=34.15) capped at Max 15 -&gt; resolved exactly 15</t>
+          <t>whole-WO flat fee add 201 + visible in WO view (flat 7.77 resolved exactly) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Sidebar card is 'WO Fees &amp; Discounts' (was 'Work Order Fee / Discount'). Exact success-toast text not re-captured this pass (worded as 'a success message').</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-007</t>
+          <t>FD-WO-003</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>C28430</t>
+          <t>C28426</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28430</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28426</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4948,12 +4948,12 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Verify the add confirm button label follows the Type (Add Fee vs Add Discount)</t>
+          <t>Verify the live preview shows a whole-work-order percentage discount before you save</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -4963,24 +4963,24 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>confirm label 'Add Fee' observed; Type-flip re-observed in batch-1 (not re-driven)</t>
+          <t>dialog live preview re-driven ($5 flat -&gt; '+$5.00 / New work-order subtotal $187.76'); pct preview math not re-driven, API pct resolution re-proven (10%-&gt;17.08) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calc type corrected from generic 'Percentage' to the real whole-WO option '% of Subtotal'. Exact preview row labels not re-captured this pass (behavior verified 2026-07-10).</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-008</t>
+          <t>FD-WO-004</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>C28431</t>
+          <t>C28427</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28431</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28427</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4990,12 +4990,12 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Verify an empty Name blocks saving a whole-WO adjustment</t>
+          <t>Verify 'Apply From Template' fills the dialog with a template's values</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -5005,24 +5005,24 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>UI BLOCKS empty name (inline 'Name' required, dialog stays open, nothing saved). NOTE NEW FDBUG-16: the RAW API now ACCEPTS an empty-name adjustment (201; was 400 in batch-3) — BE validation regression, FE still guards</t>
+          <t>not re-driven today (Apply-From-Template combobox present in dialog); templateId add path re-proven via API (FD-STACK-003) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Dropdown label is exactly 'Apply From Template' (was 'Apply from template (optional)').</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-009</t>
+          <t>FD-WO-006</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>C28432</t>
+          <t>C28429</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28432</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28429</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Verify an empty or zero Amount blocks saving a whole-WO adjustment</t>
+          <t>Verify Max Amount caps a percentage fee (20% on a $100 base with Max Amount $15 → +$15.00)</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -5047,24 +5047,24 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>amount 0 -&gt; 400 at API; UI validates on submit</t>
+          <t>20% of 170.76 (=34.15) capped at Max 15 -&gt; resolved exactly 15 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). The '$ Max Amount (Optional)' field appears only after a percentage method is chosen (confirmed live).</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-010</t>
+          <t>FD-WO-007</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>C28433</t>
+          <t>C28430</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28433</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28430</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Verify a percentage discount over 100% is rejected while a percentage fee has no upper limit</t>
+          <t>Verify the confirm button label follows the Type (Add Fee vs Add Discount)</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -5089,24 +5089,24 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>discount 150% -&gt; 400 'A percentage discount cannot exceed 100%.'; fee 150% -&gt; 201</t>
+          <t>confirm label 'Add Fee' observed; Type-flip re-observed in batch-1 (not re-driven) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05).</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-011</t>
+          <t>FD-WO-008</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>C28434</t>
+          <t>C28431</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28434</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28431</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -5116,12 +5116,12 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Verify whole-WO percentage methods resolve against the correct base (% of Subtotal example)</t>
+          <t>Verify an empty Name blocks saving a whole-work-order fee/discount</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -5131,24 +5131,24 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>pct_subtotal resolves on the WO subtotal EXCLUDING whole-WO adjustments (10% of 182.76-sub -&gt; 17.08 = 10% of 170.76 line total)</t>
+          <t>UI BLOCKS empty name (inline 'Name' required, dialog stays open, nothing saved). NOTE NEW FDBUG-16: the RAW API now ACCEPTS an empty-name adjustment (201; was 400 in batch-3) — BE validation regression, FE still guards | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). (Note: the raw back-end will accept an empty name — FDBUG-16 — but the on-screen dialog blocks it, which is what a manual tester sees.)</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-012</t>
+          <t>FD-WO-009</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>C28435</t>
+          <t>C28432</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28435</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28432</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -5158,12 +5158,12 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Verify 'Add Fee / Discount' is hidden and rejected on an Invoiced or Paid work order</t>
+          <t>Verify an empty or zero amount blocks saving a whole-work-order fee/discount</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -5173,24 +5173,24 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>add on Invoiced WO -&gt; 409 'Adjustments cannot be changed on an invoiced or paid work order.'; edit also 409</t>
+          <t>amount 0 -&gt; 400 at API; UI validates on submit | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-014</t>
+          <t>FD-WO-010</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>C28437</t>
+          <t>C28433</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28437</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28433</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Verify the live preview shows the empty-amount prompt before an amount is entered</t>
+          <t>Verify a percentage discount over 100% is rejected while a percentage fee has no upper limit</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -5215,49 +5215,175 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>'Enter an amount to see the impact.' prompt present in the re-driven dialog</t>
+          <t>discount 150% -&gt; 400 'A percentage discount cannot exceed 100%.'; fee 150% -&gt; 201 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05).</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
+          <t>FD-WO-011</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>C28434</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28434</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Work Order — Whole-WO Fee/Discount</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Verify a whole-work-order percentage method uses the correct base (% of Subtotal example)</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>pct_subtotal resolves on the WO subtotal EXCLUDING whole-WO adjustments (10% of 182.76-sub -&gt; 17.08 = 10% of 170.76 line total) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calculation Type options confirmed live (exactly the 4 listed; no '% of Grand Total').</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>FD-WO-012</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>C28435</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28435</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Work Order — Whole-WO Fee/Discount</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Verify Add Fee/Discount is hidden and blocked on an Invoiced or Paid work order</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>add on Invoiced WO -&gt; 409 'Adjustments cannot be changed on an invoiced or paid work order.'; edit also 409 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>FD-WO-014</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>C28437</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28437</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Work Order — Whole-WO Fee/Discount</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Verify the preview shows the empty-amount prompt before an amount is entered</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>'Enter an amount to see the impact.' prompt present in the re-driven dialog | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Exact prompt text 'Enter an amount to see the impact.' confirmed live (shot wo-03).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
           <t>FD-WO-015</t>
         </is>
       </c>
-      <c r="B110" s="2" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>C28438</t>
         </is>
       </c>
-      <c r="C110" s="5" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/28438</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="D113" s="2" t="inlineStr">
         <is>
           <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>Verify the preview adjustment row is signed and colored (fee vs discount)</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>Verify the preview amount is signed for a fee (+) vs a discount (−)</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr">
-        <is>
-          <t>preview row '+$5.00' with new-subtotal line re-observed; color/sign convention from batch-1 (not re-checked)</t>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>preview row '+$5.00' with new-subtotal line re-observed; color/sign convention from batch-1 (not re-checked) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Kept to sign only; the exact fee/discount colours were not re-captured this pass.</t>
         </is>
       </c>
     </row>
@@ -5372,6 +5498,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5383,7 +5512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5777,27 +5906,27 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FD-FIN-004</t>
+          <t>FD-INLINE-003</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>C28467</t>
+          <t>C28456</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28467</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28456</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Sidebar 'Work Order Fee / Discount' card</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Verify the sidebar 'Work Order Fee / Discount' card lists whole-WO adjustments with name, signed rate badge, grey amount and hover Edit/Delete</t>
+          <t>Verify a line/part with 2 or more fees/discounts shows only the first plus a 'Show N more' toggle</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -5812,39 +5941,39 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>card renders 'WO Fees &amp; Discounts / Flat fee $12.00 +$12.00' — label/name drift vs spec wording persists (case-update)</t>
+          <t>CONFIRMED AGAIN: 2 adjustments on one part render with NO 'Show N more' collapse — PO Q5=B defect persists | WORDING+VIU 2026-07-13: DEVIATION carried (BUG-FD-5): no 'Show N more' collapse — a line/part with 2+ fees/discounts shows all of them. Not re-driven with a 3-adjustment line this run.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>FD-INLINE-003</t>
+          <t>FD-LABOR-001</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>C28456</t>
+          <t>C28439</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28456</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28439</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Verify a line/part with 2+ adjustments shows only the first plus a 'Show N more' toggle</t>
+          <t>Verify a labor line's 3-dot menu opens the Add dialog locked to that Labor Line scope</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5854,34 +5983,34 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED AGAIN: 2 adjustments on one part render with NO 'Show N more' collapse — PO Q5=B defect persists</t>
+          <t>label drift (subtitle 'Applying to: {line}' without 'Line {N} Labor —' prefix) per batch-1; not re-driven today</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-001</t>
+          <t>FD-PART-001</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>C28439</t>
+          <t>C28446</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28439</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28446</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Verify a labor line's 3-dot menu opens the Add dialog locked to that Labor Line scope</t>
+          <t>Verify a part's menu opens the Add dialog locked to that Part Line scope</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -5896,39 +6025,39 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>label drift (subtitle 'Applying to: {line}' without 'Line {N} Labor —' prefix) per batch-1; not re-driven today</t>
+          <t>FDBUG-14 label defects (missing 'Line {N} Part —' prefix, raw enum 'Pct_parts', part-% option mislabeled '% of Labor Total') per batch-4; part dialog not re-driven today</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>FD-PART-001</t>
+          <t>FD-PERM-002</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>C28446</t>
+          <t>C28586</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28446</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28586</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Verify a part's menu opens the Add dialog locked to that Part Line scope</t>
+          <t>Verify Whole-WO adjustment add/edit/remove requires Work Orders: Create and Edit</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -5938,34 +6067,34 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-14 label defects (missing 'Line {N} Part —' prefix, raw enum 'Pct_parts', part-% option mislabeled '% of Labor Total') per batch-4; part dialog not re-driven today</t>
+          <t>BUG-FD-3 stands on batch evidence; NOT re-testable today — Technician role drifted on the shared env (now HAS workOrdersCreateAndEdit, so its 201 is legitimate); enforcement-depth question unchanged (dev decision)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-002</t>
+          <t>FD-PROC-008</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>C28586</t>
+          <t>C28526</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28586</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28526</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Permissions (Story 13)</t>
+          <t>Processing Fee — WO behavior</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Verify Whole-WO adjustment add/edit/remove requires Work Orders: Create and Edit</t>
+          <t>Verify a Processing Fee on a WO can be removed but not edited</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -5980,34 +6109,34 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>BUG-FD-3 stands on batch evidence; NOT re-testable today — Technician role drifted on the shared env (now HAS workOrdersCreateAndEdit, so its 201 is legitimate); enforcement-depth question unchanged (dev decision)</t>
+          <t>BE re-proven: pfee change -&gt; 409 'cannot be edited through this endpoint', remove -&gt; 204; card still offers Edit per batch-1 (S8-N5 UI drift)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-008</t>
+          <t>FD-PROC-009</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>C28526</t>
+          <t>C28527</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28526</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28527</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — WO behavior</t>
+          <t>Processing Fee — calculation</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee on a WO can be removed but not edited</t>
+          <t>Verify a % of Grand Total Processing Fee resolves last on a tax-inclusive base (3% of $324 → +$9.72)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -6022,34 +6151,34 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>BE re-proven: pfee change -&gt; 409 'cannot be edited through this endpoint', remove -&gt; 204; card still offers Edit per batch-1 (S8-N5 UI drift)</t>
+          <t>FDBUG-2 CONFIRMED AGAIN with a clean discriminator: on a WO whose ONLY money is a whole-WO $20 taxable fee, 3% pfee resolved 0.63 (=3% of 21.00 incl the whole-WO fee + its tax); spec base must EXCLUDE whole-WO adjustments -&gt; expected 0.00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-009</t>
+          <t>FD-QB-014</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>C28527</t>
+          <t>C28557</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28527</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28557</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — calculation</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Verify a % of Grand Total Processing Fee resolves last on a tax-inclusive base (3% of $324 → +$9.72)</t>
+          <t>Verify a mandatory warn/confirm before saving when discounts exceed the net subtotal</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -6064,34 +6193,34 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-2 CONFIRMED AGAIN with a clean discriminator: on a WO whose ONLY money is a whole-WO $20 taxable fee, 3% pfee resolved 0.63 (=3% of 21.00 incl the whole-WO fee + its tax); spec base must EXCLUDE whole-WO adjustments -&gt; expected 0.00</t>
+          <t>FDBUG-15 CONFIRMED AGAIN (API half): over-discount saves 201 with NO warning payload; excess carried silently (117.24). Batch-6 UI shots show no warn/confirm dialog. Violates S6-R12</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>FD-QB-014</t>
+          <t>FD-STATS-001</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>C28557</t>
+          <t>C28459</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28557</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28459</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks — negative totals</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Verify a mandatory warn/confirm before saving when discounts exceed the net subtotal</t>
+          <t>Verify the Stats tab shows a 'Fees &amp; Discounts (N)' breakdown with a value/% and an amount for each row</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -6106,39 +6235,39 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-15 CONFIRMED AGAIN (API half): over-discount saves 201 with NO warning payload; excess carried silently (117.24). Batch-6 UI shots show no warn/confirm dialog. Violates S6-R12</t>
+          <t>CONFIRMED AGAIN: Stats shows aggregate 'Fees &amp; Discounts (5) $25.00' style block, NOT the per-row Value/%+Amount table — PO Q1=B design regression persists (shot 07-stats) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-2): the Stats 'Fees &amp; Discounts (N)' section lists rows (name, a value/% for percentages, and an amount) but has NO 'Value'/'Amount' column headers like the other Stats sections. Confirmed live (shot fin-01).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>FD-REMOVE-001</t>
+          <t>FD-STATS-002</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>C28479</t>
+          <t>C28460</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28479</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28460</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Remove an adjustment</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a whole-WO adjustment shows the 'Remove Fee / Discount' confirm and a success toast</t>
+          <t>Verify each Stats fee/discount row names its target</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -6148,24 +6277,24 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>remove-confirm wording drift per batch-1 (case-update); not re-driven today</t>
+          <t>per-row scope hyperlink impossible while the layout is aggregate (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: Stats F&amp;D rows show the name only — no scope hyperlink to the target. Confirmed live (rows read plain names, shot fin-01).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-001</t>
+          <t>FD-STATS-004</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C28459</t>
+          <t>C28462</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28459</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28462</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -6175,12 +6304,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats tab shows a 'Fees &amp; Discounts (N)' breakdown with Value/% and Amount columns</t>
+          <t>Verify the Stats fees/discounts are listed in the order they were created (oldest first)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -6190,39 +6319,39 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED AGAIN: Stats shows aggregate 'Fees &amp; Discounts (5) $25.00' style block, NOT the per-row Value/%+Amount table — PO Q1=B design regression persists (shot 07-stats)</t>
+          <t>creation-order rows blocked by aggregate layout (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: creation-order ruling pending (BUG-FD-2 group). Labels cleaned.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-002</t>
+          <t>FD-TMPL-001</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>C28460</t>
+          <t>C28502</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28460</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28502</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Template admin — location</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Verify each Stats F&amp;D row shows a scope hyperlink naming its target</t>
+          <t>Verify the location template library lives at Administration → Service → Fees &amp; Discounts, below Canned Lines</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -6232,39 +6361,39 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>per-row scope hyperlink impossible while the layout is aggregate (dep. FD-STATS-001)</t>
+          <t>admin library lives under Administration -&gt; FINANCE (route /administration/adjustment-templates), not Service-below-Canned-Lines; page re-loaded today (case-update per S13-R8 target)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-004</t>
+          <t>FD-TMPL-003</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>C28462</t>
+          <t>C28504</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28462</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28504</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Template admin — create</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats F&amp;D rows are listed in creation order (oldest first)</t>
+          <t>Verify creating a Fee template (dialog fields, confirm button, success toast)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -6274,39 +6403,39 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>creation-order rows blocked by aggregate layout (dep. FD-STATS-001)</t>
+          <t>PARTIAL IMPROVEMENT: create-dialog title NOW 'New Fee / Discount' (matches spec; was 'Add new fee/discount'); confirm button still 'Create' (spec 'Add Fee / Discount') and toast 'Template created' per batch-1 — drift remains</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-001</t>
+          <t>FD-TMPL-004</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>C28502</t>
+          <t>C28505</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28502</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28505</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Template admin — location</t>
+          <t>Template admin — create</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Verify the location template library lives at Administration → Service → Fees &amp; Discounts, below Canned Lines</t>
+          <t>Verify creating a Discount template shows the "Discount added" toast</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -6316,39 +6445,39 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>admin library lives under Administration -&gt; FINANCE (route /administration/adjustment-templates), not Service-below-Canned-Lines; page re-loaded today (case-update per S13-R8 target)</t>
+          <t>generic 'Template created' toast vs spec 'Discount added' per batch-1; not re-driven</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-003</t>
+          <t>FD-TMPL-006</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>C28504</t>
+          <t>C28507</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28504</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28507</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Template admin — create</t>
+          <t>Template admin — edit</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Verify creating a Fee template (dialog fields, confirm button, success toast)</t>
+          <t>Verify editing a template (open by row click, "Save" button, update toast)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -6358,34 +6487,34 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL IMPROVEMENT: create-dialog title NOW 'New Fee / Discount' (matches spec; was 'Add new fee/discount'); confirm button still 'Create' (spec 'Add Fee / Discount') and toast 'Template created' per batch-1 — drift remains</t>
+          <t>edit locks Type+Calc on template edit (spec locks only in WO dialog) per batch-1; not re-driven</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-004</t>
+          <t>FD-TMPL-008</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>C28505</t>
+          <t>C28509</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28505</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28509</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Template admin — create</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Verify creating a Discount template shows the "Discount added" toast</t>
+          <t>Verify the delete confirm adds a warning when the template is a default for one or more customers</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -6400,39 +6529,39 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>generic 'Template created' toast vs spec 'Discount added' per batch-1; not re-driven</t>
+          <t>standardized 'Delete Template' dialog wording = intended per epic; case-update to adopt live wording still pending</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-006</t>
+          <t>FD-TMPL-010</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>C28507</t>
+          <t>C28511</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28507</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28511</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Template admin — edit</t>
+          <t>Template admin — scoping</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Verify editing a template (open by row click, "Save" button, update toast)</t>
+          <t>Verify template scoping — labour-method templates only appear in labour modals, parts-method only in parts modals</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -6442,34 +6571,34 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>edit locks Type+Calc on template edit (spec locks only in WO dialog) per batch-1; not re-driven</t>
+          <t>FDBUG-13 (line-scope Add dialog has no template picker) per batch-1/4; not re-driven today</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-008</t>
+          <t>FD-TMPL-011</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>C28509</t>
+          <t>C28512</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28509</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28512</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Template admin — delete</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Verify the delete confirm adds a warning when the template is a default for one or more customers</t>
+          <t>Verify Max Amount appears only for percentage methods and 0 is treated as empty</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -6484,34 +6613,34 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>standardized 'Delete Template' dialog wording = intended per epic; case-update to adopt live wording still pending</t>
+          <t>maxCap 0 accepted and STORED as 0 on the template (201) and WO resolve treats 0 as NO cap (34.15) — FDBUG-9 persists</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-010</t>
+          <t>FD-VAL-001</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>C28511</t>
+          <t>C28599</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28511</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28599</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Template admin — scoping</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Verify template scoping — labour-method templates only appear in labour modals, parts-method only in parts modals</t>
+          <t>Verify the Add button stays disabled until Name, Type, Calculation Type and an Amount above 0 are all set</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -6526,34 +6655,34 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-13 (line-scope Add dialog has no template picker) per batch-1/4; not re-driven today</t>
+          <t>CONFIRMED AGAIN: Add button enabled on empty form (validates on submit) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: DEVIATION re-confirmed 2026-07-13 (BUG-FD-4): the 'Add Fee' button is ENABLED on an empty form (validates on submit). Labels build-accurate (Add Fee/Add Discount, Calculation Type, Max Amount).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-011</t>
+          <t>FD-VAL-006</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>C28512</t>
+          <t>C28604</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28512</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28604</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Template admin — dialog fields</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Verify Max Amount appears only for percentage methods and 0 is treated as empty</t>
+          <t>Verify the Max Amount field shows only for percentage methods and how 0 or empty behaves</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -6568,39 +6697,39 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>maxCap 0 accepted and STORED as 0 on the template (201) and WO resolve treats 0 as NO cap (34.15) — FDBUG-9 persists</t>
+          <t>FDBUG-9: maxCap 0 behaves as NO cap (not 'no maximum' spec reading matches build for empty, but 0 disagrees w/ §5-R6 $0-forces-$0) — persists | WORDING+VIU 2026-07-13: Confirmed live: '$ Max Amount (Optional)' appears only for percentage methods (hidden for Flat Amount, shots wo-03/wo-05). DEVIATION (FDBUG-9 / PO Q2 pending): whether a Max Amount of 0 means 'no cap' or 'cap at $0.00' is a pending product decision — expected kept as current build behavior.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-001</t>
+          <t>FD-WO-005</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>C28599</t>
+          <t>C28428</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28599</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28428</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Verify the Add button stays DISABLED until Name AND Type AND Calculation type AND Amount &gt; 0 are all set</t>
+          <t>Verify the Add button stays disabled until Name, Type, Calculation Type and an Amount above 0 are all filled in</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6610,34 +6739,34 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED AGAIN: Add button enabled on empty form (validates on submit) — PO Q4=B defect persists</t>
+          <t>CONFIRMED AGAIN: 'Add Fee' button ENABLED on an empty form (disabled-on-empty=false) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION re-confirmed live 2026-07-13: the 'Add Fee' button is ENABLED on an empty form (validation happens on submit, not by disabling) — BUG-FD-4. Expected kept as the intended behavior; tester will see the button enabled.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-006</t>
+          <t>FD-WO-013</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>C28604</t>
+          <t>C28436</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28604</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28436</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Verify Max cap edge behavior — 0 or empty = no maximum, and Max Amount shows only for percentage methods</t>
+          <t>Verify the whole-work-order Add Fee/Discount option is hidden without Work Orders: Create &amp; Edit</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -6652,24 +6781,24 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-9: maxCap 0 behaves as NO cap (not 'no maximum' spec reading matches build for empty, but 0 disagrees w/ §5-R6 $0-forces-$0) — persists</t>
+          <t>BUG-FD-3 stands on prior evidence; NOT re-testable today: the shared-env Technician role was CHANGED (now includes workOrdersCreateAndEdit+workOrdersDelete, 8 perms vs matrix 6) so tech's 201 is now legitimate; no login lacking the perm exists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION (BUG-FD-3: the hide is front-end only; the back-end does not block the write). NOT re-testable this run — the Technician role has drifted on the shared qb env; re-derive the roles matrix before re-checking.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-001</t>
+          <t>FD-WO-016</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>C28424</t>
+          <t>C29441</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28424</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29441</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -6679,12 +6808,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Verify the whole-work-order Add dialog opens from the WO toolbar more (⋯) menu at Whole Work Order scope</t>
+          <t>Verify the Add/Edit fee-or-discount dialog shows the tax-jurisdiction note below the Taxable toggle</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6694,91 +6823,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>dialog title still 'Add new fee/discount' (spec 'New Fee / Discount'), menu item 'Add Fee/Discount' — label drift persists (UI re-driven, shot 10-wo-add-dialog)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>FD-WO-005</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>C28428</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28428</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Verify the Add button is disabled until Name, Type, Calculation type and Amount&gt;0 are all set</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Deviation</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>CONFIRMED AGAIN: 'Add Fee' button ENABLED on an empty form (disabled-on-empty=false) — PO Q4=B defect persists</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>FD-WO-013</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>C28436</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28436</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Verify whole-WO starting places are hidden without Work Orders: Create &amp; Edit</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Deviation</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>BUG-FD-3 stands on prior evidence; NOT re-testable today: the shared-env Technician role was CHANGED (now includes workOrdersCreateAndEdit+workOrdersDelete, 8 perms vs matrix 6) so tech's 201 is now legitimate; no login lacking the perm exists</t>
+          <t>/No TOGGLE (not a dropdown) — corrected. DEVIATION: the §5-R15 jurisdiction note is NOT shown below the Taxable toggle in this build (checked the whole-WO Add dialog with both Flat Amount and % of Subtotal; no note present — shots wo-03/wo-05). Expected kept as the spec requirement; currently a gap.</t>
         </is>
       </c>
     </row>
@@ -6814,8 +6859,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8253,7 +8296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8770,48 +8813,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>FD-WO-016</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>C29441</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29441</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Verify the Add/Edit fee-or-discount dialog shows the §5-R15 taxable jurisdiction note below the Taxable dropdown</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pending — new case (V1_2 §5-R15 / S2-R26a); not yet checked live</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>NEW 2026-07-13 for V1_2 §5-R15 / S2-R26a. UI string check (advisory) — belongs in a FUNCTIONAL section, NOT an API section (standing rule 4). Assert the exact string verbatim.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
@@ -8825,7 +8826,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fees & Discounts: execute authorized TestRail sync (18 add + 51 update + 3 retire SV-8479/8480)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_FreshVIU_2026-07-10.xlsx
+++ b/build/fees-discounts/FeesDiscounts_FreshVIU_2026-07-10.xlsx
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1321,10 +1321,14 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr"/>
+          <t>C30629</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30629</t>
+        </is>
+      </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -1358,10 +1362,14 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
+          <t>C30630</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30630</t>
+        </is>
+      </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -1396,10 +1404,14 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr"/>
+          <t>C30631</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30631</t>
+        </is>
+      </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -1434,10 +1446,14 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
+          <t>C30632</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30632</t>
+        </is>
+      </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -1472,10 +1488,14 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
+          <t>C30633</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30633</t>
+        </is>
+      </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -1510,10 +1530,14 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
+          <t>C30635</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30635</t>
+        </is>
+      </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -4021,32 +4045,32 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>FD-PCOL-003</t>
+          <t>FD-PCOL-004</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>C28471</t>
+          <t>C28472</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28471</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28472</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts page — breakdown modal</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Verify a fee-less part row adds a fee/discount from its three-dot menu 'Add Part Fee / Discount' (no '+ Add' button)</t>
+          <t>Verify clicking a filled 'Fees &amp; Discounts' cell opens the per-part breakdown with the right columns</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -4056,24 +4080,24 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: + Add button shown on a no-fee part. Live staging (psH2-invoiced.png); add works on editable sale via row menu. | SV-8479/8480 deconfliction 2026-07-22: rescoped off the removed '+ Add' button to the per-row ⋮ 'Add Part Fee / Discount' + 'New Part Fee / Discount' title (items 13/14/18). RETIRE-CANDIDATE (F2): overlaps kept new cases FD-PSALE-002/003 — flag for user ruling. | SV-8479 Batch-3 STAGING LIVE VIU 2026-07-22 (part-sale surface): seeded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: fee-less row no '+ Add'; ⋮ 'Add Part Fee / Discount' -&gt; dialog 'New Part Fee / Discount'.</t>
+          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Filled cell opens viewer with Name/Type/Calculation/Amount/Max Amount columns. Live staging (psC-viewer2rows.png).</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>FD-PCOL-004</t>
+          <t>FD-PCOL-005</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>C28472</t>
+          <t>C28473</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28472</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28473</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -4083,12 +4107,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Verify clicking a filled 'Fees &amp; Discounts' cell opens the per-part breakdown with the right columns</t>
+          <t>Verify the breakdown 'Net adjustment' row equals the signed sum of the part's fees/discounts</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -4098,24 +4122,24 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Filled cell opens viewer with Name/Type/Calculation/Amount/Max Amount columns. Live staging (psC-viewer2rows.png).</t>
+          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Viewer Net adjustment = signed sum (+$12.00 + $2.00 = +$14.00). Live staging (psC-viewer2rows.png).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>FD-PCOL-005</t>
+          <t>FD-PCOL-006</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>C28473</t>
+          <t>C28474</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28473</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28474</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -4125,12 +4149,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Verify the breakdown 'Net adjustment' row equals the signed sum of the part's fees/discounts</t>
+          <t>Verify a per-row Remove on the breakdown removes the fee/discount and the cell returns to its empty state (no '+ Add' button)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -4140,34 +4164,34 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Viewer Net adjustment = signed sum (+$12.00 + $2.00 = +$14.00). Live staging (psC-viewer2rows.png).</t>
+          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Per-row Remove -&gt; confirm Remove Fee / Discount -&gt; row removed. Live staging (psE-confirm/afterremove). | SV-8479/8480 deconfliction 2026-07-22: empty-state reworded: the removed '+ Add' button is gone; add via the per-row ⋮ (item 13). | SV-8479 Batch-3 STAGING LIVE VIU 2026-07-22 (part-sale surface): seeded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: breakdown viewer per-row delete -&gt; confirm 'Remove Fee / Discount' -&gt; removed -&gt; empty state, no '+ Add'.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>FD-PCOL-006</t>
+          <t>FD-PERM-001</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>C28474</t>
+          <t>C28585</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28474</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28585</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Parts page — breakdown modal</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Verify a per-row Remove on the breakdown removes the fee/discount and the cell returns to its empty state (no '+ Add' button)</t>
+          <t>Verify See Financial Data controls all fee/discount dollar amounts (without it, amounts are hidden)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4182,39 +4206,39 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Per-row Remove -&gt; confirm Remove Fee / Discount -&gt; row removed. Live staging (psE-confirm/afterremove). | SV-8479/8480 deconfliction 2026-07-22: empty-state reworded: the removed '+ Add' button is gone; add via the per-row ⋮ (item 13). | SV-8479 Batch-3 STAGING LIVE VIU 2026-07-22 (part-sale surface): seeded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: breakdown viewer per-row delete -&gt; confirm 'Remove Fee / Discount' -&gt; removed -&gt; empty state, no '+ Add'.</t>
+          <t>tech (no SFD): WO view masks all money (sub_total/total '0.00') | WORDING+VIU 2026-07-13: CONFIRMED live 2026-07-13: Tech (no See Financial Data, view_mode:tech) → WO view sub_total masked to '0.00' (amounts hidden).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>FD-PCOL-007</t>
+          <t>FD-PERM-003</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>C28475</t>
+          <t>C28587</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28475</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28587</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Verify the per-row three-dot 'Add Part Fee / Discount' is unavailable when the sale/work order cannot be edited</t>
+          <t>Verify labor-line and part-line add/edit/remove requires Work Order Lines: Create and Edit</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4224,24 +4248,24 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: + Add disabled on non-editable (Paid) sale. Live staging (psH2-invoiced.png, btnDisabled=true). | SV-8479/8480 deconfliction 2026-07-22: rescoped off the removed '+ Add' button to the per-row ⋮ blocked-when-uneditable (item 13). RETIRE-CANDIDATE (F2): overlaps kept new case FD-PSALE-002 — flag for user ruling. | SV-8479 Batch-3 STAGING LIVE VIU 2026-07-22 (part-sale surface): seeded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: Paid sale P3-1088 (editable=false) has NO '+ Add' and NO per-row ⋮ menu (button_part_request_menu_* count 0) -&gt; add unavailable/blocked when non-editable.</t>
+          <t>positive half fresh (tech WITH lines-C&amp;E: line add 201/remove 204); negative half via roles-matrix FE derivation (role-drift caveat) | WORDING+VIU 2026-07-13: Positive: Tech HAS Work Order Lines: Create &amp; Edit. Negative not testable (Tech drifted to have it). Line-level gate carried from prior derivation.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-001</t>
+          <t>FD-PERM-004</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>C28585</t>
+          <t>C28588</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28585</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28588</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -4251,7 +4275,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Verify See Financial Data controls all fee/discount dollar amounts (without it, amounts are hidden)</t>
+          <t>Verify part-sale add/edit/remove requires Part Sales: Create and Edit plus See Financial Data</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -4266,24 +4290,24 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>tech (no SFD): WO view masks all money (sub_total/total '0.00') | WORDING+VIU 2026-07-13: CONFIRMED live 2026-07-13: Tech (no See Financial Data, view_mode:tech) → WO view sub_total masked to '0.00' (amounts hidden).</t>
+          <t>Part Sales adjustment surface absent (Story 11 re-checked today) | WORDING+VIU 2026-07-13: NOT BUILT: Story 11 Part Sales fees/discounts not shipped; cannot test the Part Sales permission gate. | STAGING VIU 2026-07-20 staging LIVE VIU: Admin (Part Sales C&amp;E + SFD) can add/edit/remove part-sale F&amp;D; Tech (no Part Sales perms) has Parts nav hidden entirely. Live staging.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-003</t>
+          <t>FD-PERM-005</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>C28587</t>
+          <t>C28589</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28587</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28589</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4293,7 +4317,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Verify labor-line and part-line add/edit/remove requires Work Order Lines: Create and Edit</t>
+          <t>Verify any add/edit/remove of a fee/discount also needs See Financial Data on</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -4308,24 +4332,24 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>positive half fresh (tech WITH lines-C&amp;E: line add 201/remove 204); negative half via roles-matrix FE derivation (role-drift caveat) | WORDING+VIU 2026-07-13: Positive: Tech HAS Work Order Lines: Create &amp; Edit. Negative not testable (Tech drifted to have it). Line-level gate carried from prior derivation.</t>
+          <t>SFD prerequisite: controls live on SFD-masked surfaces (tech masked view re-confirmed) | WORDING+VIU 2026-07-13: See-Financial-Data masking confirmed live (Tech financials masked). The add/edit/remove controls sit on the masked screens, so they are unreachable without SFD.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-004</t>
+          <t>FD-PERM-006</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>C28588</t>
+          <t>C28590</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28588</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28590</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -4335,7 +4359,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Verify part-sale add/edit/remove requires Part Sales: Create and Edit plus See Financial Data</t>
+          <t>Verify removing a fee/discount uses Create and Edit, not the separate Delete permission</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -4350,24 +4374,24 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Part Sales adjustment surface absent (Story 11 re-checked today) | WORDING+VIU 2026-07-13: NOT BUILT: Story 11 Part Sales fees/discounts not shipped; cannot test the Part Sales permission gate. | STAGING VIU 2026-07-20 staging LIVE VIU: Admin (Part Sales C&amp;E + SFD) can add/edit/remove part-sale F&amp;D; Tech (no Part Sales perms) has Parts nav hidden entirely. Live staging.</t>
+          <t>removal uses the same Create&amp;Edit gate (tech remove 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove via Create &amp; Edit (not a separate Delete) carried.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-005</t>
+          <t>FD-PERM-007</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>C28589</t>
+          <t>C28591</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28589</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28591</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4377,7 +4401,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Verify any add/edit/remove of a fee/discount also needs See Financial Data on</t>
+          <t>Verify create/edit/delete of a fee/discount template needs Settings → Service</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -4392,24 +4416,24 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>SFD prerequisite: controls live on SFD-masked surfaces (tech masked view re-confirmed) | WORDING+VIU 2026-07-13: See-Financial-Data masking confirmed live (Tech financials masked). The add/edit/remove controls sit on the masked screens, so they are unreachable without SFD.</t>
+          <t>templates admin BE-enforced: tech GET/POST 403 | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no Settings → Finance) → GET templates 403 'Access denied.' | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-006</t>
+          <t>FD-PERM-008</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>C28590</t>
+          <t>C28592</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28590</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28592</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -4419,7 +4443,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a fee/discount uses Create and Edit, not the separate Delete permission</t>
+          <t>Verify viewing/changing a customer's default fees &amp; discounts needs BOTH Customer Management: Create and Edit AND Manage Accounts Payable and Receivable</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -4434,24 +4458,24 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>removal uses the same Create&amp;Edit gate (tech remove 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove via Create &amp; Edit (not a separate Delete) carried.</t>
+          <t>customer defaults BE-enforced: tech GET 403 + POST 403 | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no Manage AP/AR, no Customer Mgmt C&amp;E) → customer default-adjustments GET 403 AND POST 403 'Access denied.'</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-007</t>
+          <t>FD-PERM-009</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>C28591</t>
+          <t>C28593</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28591</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28593</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4461,12 +4485,12 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Verify create/edit/delete of a fee/discount template needs Settings → Service</t>
+          <t>Verify seeing fee/discount entries in the work-order audit log needs Work Orders: Create and Edit (line audit log needs Work Order Lines: Create and Edit)</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -4476,24 +4500,24 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>templates admin BE-enforced: tech GET/POST 403 | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no Settings → Finance) → GET templates 403 'Access denied.' | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>history entries: BE serves them regardless (tech 200) — FE display gate per enforcement model; entries carry set rate | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: Positive confirmed live (Tech has Work Orders/Work Order Lines: Create &amp; Edit → Work Order Log 200 with fee/discount entries; the log shows the set rate so See Financial Data does not gate it — Tech's financials are masked yet history shows). The no-permission negative is NOT testable this run (Tech drifted to have the perms; only admin/tech log in). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-008</t>
+          <t>FD-PERM-010</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>C28592</t>
+          <t>C28594</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28592</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28594</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4503,7 +4527,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Verify viewing/changing a customer's default fees &amp; discounts needs BOTH Customer Management: Create and Edit AND Manage Accounts Payable and Receivable</t>
+          <t>Verify both are required — the Fees &amp; Discounts feature on AND the matching permission</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -4518,24 +4542,24 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>customer defaults BE-enforced: tech GET 403 + POST 403 | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no Manage AP/AR, no Customer Mgmt C&amp;E) → customer default-adjustments GET 403 AND POST 403 'Access denied.'</t>
+          <t>flag ON + permission still required (tech 403 on templates/defaults with flag ON) | WORDING+VIU 2026-07-13: Permission gating confirmed live (templates/customer-defaults 403; SFD masking). Feature is ON. Both-gates model holds. | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-009</t>
+          <t>FD-PERM-011</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>C28593</t>
+          <t>C28595</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28593</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28595</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4545,7 +4569,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Verify seeing fee/discount entries in the work-order audit log needs Work Orders: Create and Edit (line audit log needs Work Order Lines: Create and Edit)</t>
+          <t>Verify add/edit/remove is blocked when the work order is Invoiced/Paid or you are viewing history</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -4560,24 +4584,24 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>history entries: BE serves them regardless (tech 200) — FE display gate per enforcement model; entries carry set rate | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: Positive confirmed live (Tech has Work Orders/Work Order Lines: Create &amp; Edit → Work Order Log 200 with fee/discount entries; the log shows the set rate so See Financial Data does not gate it — Tech's financials are masked yet history shows). The no-permission negative is NOT testable this run (Tech drifted to have the perms; only admin/tech log in). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
+          <t>Invoiced WO: add 409 + edit 409 (BE-enforced lock) | WORDING+VIU 2026-07-13: Invoiced/Paid block is back-end enforced (409) — established; carried. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-010</t>
+          <t>FD-PERM-012</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>C28594</t>
+          <t>C29922</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28594</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29922</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -4587,7 +4611,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Verify both are required — the Fees &amp; Discounts feature on AND the matching permission</t>
+          <t>Fees &amp; Discounts settings page gated by settingsService (not settingsFinance)</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -4602,24 +4626,24 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>flag ON + permission still required (tech 403 on templates/defaults with flag ON) | WORDING+VIU 2026-07-13: Permission gating confirmed live (templates/customer-defaults 403; SFD masking). Feature is ON. Both-gates model holds. | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
+          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-011</t>
+          <t>FD-PERM-013</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>C28595</t>
+          <t>C29923</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28595</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29923</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -4629,12 +4653,12 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Verify add/edit/remove is blocked when the work order is Invoiced/Paid or you are viewing history</t>
+          <t>Service admin can complete the Fees &amp; Discounts template delete flow</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -4644,34 +4668,34 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Invoiced WO: add 409 + edit 409 (BE-enforced lock) | WORDING+VIU 2026-07-13: Invoiced/Paid block is back-end enforced (409) — established; carried. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-012</t>
+          <t>FD-PROC-001</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>C29922</t>
+          <t>C28519</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29922</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28519</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Permissions (Story 13)</t>
+          <t>Processing Fee — template builder</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Fees &amp; Discounts settings page gated by settingsService (not settingsFinance)</t>
+          <t>Verify 'Processing Fee' is a third Type in the template builder</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -4686,34 +4710,34 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>RE-CHECKED TODAY: template-builder Type options are exactly [Fee, Discount] — Processing Fee STILL MISSING from the builder UI (PO Q3=B says in-scope; FDBUG-8; shot 02-template-dialog) | WORDING+VIU 2026-07-13: Confirmed live: Type dropdown = Fee/Discount only. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Type dropdown offers Fee, Discount, Processing Fee (admin template dialog). Live-observed staging (proc-type-open).</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-013</t>
+          <t>FD-PROC-002</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>C29923</t>
+          <t>C28520</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29923</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28520</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Permissions (Story 13)</t>
+          <t>Processing Fee — methods</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Service admin can complete the Fees &amp; Discounts template delete flow</t>
+          <t>Verify a Processing Fee offers only Flat Amount and % of Grand Total</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -4728,39 +4752,39 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>builder UI absent (re-checked today); BE method constraint re-proven separately (pct_labor rejected for processing_fee) | WORDING+VIU 2026-07-13: Builder not shipped. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Processing Fee Calc Type = Flat Amount + % of Grand Total only. Live staging (proc-fee-calc-open.png).</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-001</t>
+          <t>FD-PROC-003</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>C28519</t>
+          <t>C28521</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28519</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28521</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — template builder</t>
+          <t>Processing Fee — no Max Amount</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Verify 'Processing Fee' is a third Type in the template builder</t>
+          <t>Verify the Max Amount field is hidden for a Processing Fee (both methods)</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -4770,34 +4794,34 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>RE-CHECKED TODAY: template-builder Type options are exactly [Fee, Discount] — Processing Fee STILL MISSING from the builder UI (PO Q3=B says in-scope; FDBUG-8; shot 02-template-dialog) | WORDING+VIU 2026-07-13: Confirmed live: Type dropdown = Fee/Discount only. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Type dropdown offers Fee, Discount, Processing Fee (admin template dialog). Live-observed staging (proc-type-open).</t>
+          <t>builder UI absent (re-checked today); BE rejects pfee maxCap (400) | WORDING+VIU 2026-07-13: Builder not shipped. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: No Max Amount field for Processing Fee (both methods). Live staging (proc-fee-full.png).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-002</t>
+          <t>FD-PROC-004</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>C28520</t>
+          <t>C28522</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28520</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28522</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — methods</t>
+          <t>Processing Fee — taxable + jurisdiction note</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee offers only Flat Amount and % of Grand Total</t>
+          <t>Verify the Processing Fee Taxable defaults to Yes and shows the tax-jurisdiction note</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -4812,39 +4836,39 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>builder UI absent (re-checked today); BE method constraint re-proven separately (pct_labor rejected for processing_fee) | WORDING+VIU 2026-07-13: Builder not shipped. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Processing Fee Calc Type = Flat Amount + % of Grand Total only. Live staging (proc-fee-calc-open.png).</t>
+          <t>builder UI absent (re-checked today) | WORDING+VIU 2026-07-13: Builder not shipped; when it ships, also check the §5-R15 note (currently absent in the whole-WO dialog per FD-WO-016). NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | V1_3 (2026-07-17): Δ1 — §5-R15 gains one appended sentence (spec verbatim): 'The note is shown only to users with See Financial Data.' Expected gains the gate qualifier. This dialog is the one place the gate is independently observable (Story-7 admin access needs no See Financial Data, while the WO Add/Edit dialog already requires it — spec-diff §H.b). Status stays Blocked-NotBuilt (Story-8 builder UI absent); check the note + gate when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Processing Fee Taxable defaults Yes + jurisdiction note present; note gated on See Financial Data (Tech w/o SFD sees toggle, not note). Live staging (proc-fee-full.png / tech-tmpl-dialog.png).</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-003</t>
+          <t>FD-PROC-005</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>C28521</t>
+          <t>C28523</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28521</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28523</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — no Max Amount</t>
+          <t>Processing Fee — no manual add</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Verify the Max Amount field is hidden for a Processing Fee (both methods)</t>
+          <t>Verify a Processing Fee cannot be added to a work order by hand</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -4854,34 +4878,34 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>builder UI absent (re-checked today); BE rejects pfee maxCap (400) | WORDING+VIU 2026-07-13: Builder not shipped. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: No Max Amount field for Processing Fee (both methods). Live staging (proc-fee-full.png).</t>
+          <t>manual pfee add -&gt; 400 'A processing fee cannot be added manually.'; manual pct_grand_total fee also rejected for scope | WORDING+VIU 2026-07-13: Confirmed: WO Add Type dropdown = Fee/Discord only (no Processing Fee); build labels ('Add Fee/Discount', 'Apply From Template'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-004</t>
+          <t>FD-PROC-006</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>C28522</t>
+          <t>C28524</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28522</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28524</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — taxable + jurisdiction note</t>
+          <t>Processing Fee — auto-apply</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Verify the Processing Fee Taxable defaults to Yes and shows the tax-jurisdiction note</t>
+          <t>Verify a Processing Fee reaches a new work order via location auto-apply</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -4896,39 +4920,39 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>builder UI absent (re-checked today) | WORDING+VIU 2026-07-13: Builder not shipped; when it ships, also check the §5-R15 note (currently absent in the whole-WO dialog per FD-WO-016). NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | V1_3 (2026-07-17): Δ1 — §5-R15 gains one appended sentence (spec verbatim): 'The note is shown only to users with See Financial Data.' Expected gains the gate qualifier. This dialog is the one place the gate is independently observable (Story-7 admin access needs no See Financial Data, while the WO Add/Edit dialog already requires it — spec-diff §H.b). Status stays Blocked-NotBuilt (Story-8 builder UI absent); check the note + gate when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Processing Fee Taxable defaults Yes + jurisdiction note present; note gated on See Financial Data (Tech w/o SFD sees toggle, not note). Live staging (proc-fee-full.png / tech-tmpl-dialog.png).</t>
+          <t>auto-apply pfee template landed on a fresh WO (kind=processing_fee, appliedBy=auto) | WORDING+VIU 2026-07-13: Reaches WO via auto-apply (pfee accepted by BE); build labels. Menu option is 'Remove' (Edit inert for a pfee). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-005</t>
+          <t>FD-PROC-007</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>C28523</t>
+          <t>C28525</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28523</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28525</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — no manual add</t>
+          <t>Processing Fee — customer default</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee cannot be added to a work order by hand</t>
+          <t>Verify a Processing Fee reaches a new work order via a customer default</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -4938,39 +4962,39 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>manual pfee add -&gt; 400 'A processing fee cannot be added manually.'; manual pct_grand_total fee also rejected for scope | WORDING+VIU 2026-07-13: Confirmed: WO Add Type dropdown = Fee/Discord only (no Processing Fee); build labels ('Add Fee/Discount', 'Apply From Template'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>customer-default pfee landed on a fresh WO (kind=processing_fee, appliedBy=customer_default, amount 2.5) | WORDING+VIU 2026-07-13: Reaches WO via customer default; build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-006</t>
+          <t>FD-PROC-010</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>C28524</t>
+          <t>C28528</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28524</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28528</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — auto-apply</t>
+          <t>Processing Fee — negative</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee reaches a new work order via location auto-apply</t>
+          <t>Verify a Processing Fee with a Max Amount or a disallowed method is rejected</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -4980,34 +5004,34 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>auto-apply pfee template landed on a fresh WO (kind=processing_fee, appliedBy=auto) | WORDING+VIU 2026-07-13: Reaches WO via auto-apply (pfee accepted by BE); build labels. Menu option is 'Remove' (Edit inert for a pfee). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>pfee template with maxCap -&gt; 400; pfee with pct_labor -&gt; 400 'not allowed for a processing_fee' | WORDING+VIU 2026-07-13: Confirmed live 2026-07-13 via API: Max cap → 400 'A processing fee cannot have a minimum or maximum cap.'; disallowed method → 400 'Calculation type "pct_subtotal" is not allowed for a processing_fee.' Lives in an API-titled section.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-007</t>
+          <t>FD-PROC-011</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>C28525</t>
+          <t>C28529</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28525</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28529</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — customer default</t>
+          <t>Processing Fee — sign</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee reaches a new work order via a customer default</t>
+          <t>Verify a Processing Fee always adds to the total (never a discount)</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -5022,34 +5046,34 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>customer-default pfee landed on a fresh WO (kind=processing_fee, appliedBy=customer_default, amount 2.5) | WORDING+VIU 2026-07-13: Reaches WO via customer default; build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>pfees resolve as positive fees only (kind=processing_fee, amounts &gt;= 0) | WORDING+VIU 2026-07-13: Always a plus; carried.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-010</t>
+          <t>FD-PROC-012</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>C28528</t>
+          <t>C28530</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28528</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28530</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — negative</t>
+          <t>Processing Fee — template edit independence</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee with a Max Amount or a disallowed method is rejected</t>
+          <t>Verify editing a Processing Fee template does not change Processing Fees already on existing work orders</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -5064,39 +5088,39 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>pfee template with maxCap -&gt; 400; pfee with pct_labor -&gt; 400 'not allowed for a processing_fee' | WORDING+VIU 2026-07-13: Confirmed live 2026-07-13 via API: Max cap → 400 'A processing fee cannot have a minimum or maximum cap.'; disallowed method → 400 'Calculation type "pct_subtotal" is not allowed for a processing_fee.' Lives in an API-titled section.</t>
+          <t>template amount 3-&gt;9 (200) left the existing WO pfee at 3 (values copied at apply time) | WORDING+VIU 2026-07-13: Template edit independence; carried.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-011</t>
+          <t>FD-PROC-013</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>C28529</t>
+          <t>C28531</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28529</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28531</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — sign</t>
+          <t>Processing Fee — calculation edge</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee always adds to the total (never a discount)</t>
+          <t>Verify multiple Processing Fees each leave out all Processing Fees' amounts and tax from the shared base</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -5106,39 +5130,39 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>pfees resolve as positive fees only (kind=processing_fee, amounts &gt;= 0) | WORDING+VIU 2026-07-13: Always a plus; carried.</t>
+          <t>two auto pfees (3%+2%) resolved 0.63/0.42 = exact 3:2 ratio -&gt; same base, pfees exclude each other | WORDING+VIU 2026-07-13: Multiple pfees share the same base; carried.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-012</t>
+          <t>FD-PROC-014</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>C28530</t>
+          <t>C28532</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28530</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28532</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — template edit independence</t>
+          <t>Processing Fee — negative</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Verify editing a Processing Fee template does not change Processing Fees already on existing work orders</t>
+          <t>Verify the system rejects a Processing Fee that carries a minimum amount</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -5148,39 +5172,39 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>template amount 3-&gt;9 (200) left the existing WO pfee at 3 (values copied at apply time) | WORDING+VIU 2026-07-13: Template edit independence; carried.</t>
+          <t>pfee minimum silently STRIPPED on create (201, no min field persisted) — §8 invariant holds; silent-ignore wording note stands | WORDING+VIU 2026-07-13: Confirmed live 2026-07-13: BE rejects a min/max cap on a Processing Fee (400 'A processing fee cannot have a minimum or maximum cap.'). PO Q4 (whether pfee minimums should be supported at all) still pending. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q4=B): PO ruled Processing Fees do NOT support a minimum and the app must make that clear (do not silently drop). Premise confirmed WAD: no minimum field in the UI and the API rejects a pfee minimum with an explicit error (matches the live 2026-07-13 finding: 400 'A processing fee cannot have a minimum or maximum cap.'). Older 2026-07-10 'silent strip' reading superseded (last-update-wins). Expected reworded to the explicit-reject + no-field behavior. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-013</t>
+          <t>FD-PSALE-001</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>C28531</t>
+          <t>C29918</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28531</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29918</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — calculation edge</t>
+          <t>Part Sale — Fee/Discount dialog</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Verify multiple Processing Fees each leave out all Processing Fees' amounts and tax from the shared base</t>
+          <t>Verify the Part Sale Add/Edit fee-or-discount dialog shows the tax-jurisdiction note below the Taxable Yes/No dropdown</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -5190,39 +5214,39 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>two auto pfees (3%+2%) resolved 0.63/0.42 = exact 3:2 ratio -&gt; same base, pfees exclude each other | WORDING+VIU 2026-07-13: Multiple pfees share the same base; carried.</t>
+          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-014</t>
+          <t>FD-PSALE-002</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>C28532</t>
+          <t>C30623</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28532</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30623</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — negative</t>
+          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Verify the system rejects a Processing Fee that carries a minimum amount</t>
+          <t>Verify the parts-sale Fees &amp; Discounts column no longer shows the '+ Add' button, and the per-row and top-right three-dot entry points remain</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -5232,34 +5256,34 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>pfee minimum silently STRIPPED on create (201, no min field persisted) — §8 invariant holds; silent-ignore wording note stands | WORDING+VIU 2026-07-13: Confirmed live 2026-07-13: BE rejects a min/max cap on a Processing Fee (400 'A processing fee cannot have a minimum or maximum cap.'). PO Q4 (whether pfee minimums should be supported at all) still pending. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q4=B): PO ruled Processing Fees do NOT support a minimum and the app must make that clear (do not silently drop). Premise confirmed WAD: no minimum field in the UI and the API rejects a pfee minimum with an explicit error (matches the live 2026-07-13 finding: 400 'A processing fee cannot have a minimum or maximum cap.'). Older 2026-07-10 'silent strip' reading superseded (last-update-wins). Expected reworded to the explicit-reject + no-field behavior. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md).</t>
+          <t xml:space="preserve"> NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. F&amp;D column has no '+ Add' (grep '+Add'=0); per-row ⋮ 'Add Part Fee / Discount' + top-right ⋮ 'Add Parts Sale Fee / Discount' both present.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-001</t>
+          <t>FD-PSALE-003</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>C29918</t>
+          <t>C30624</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29918</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30624</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Part Sale — Fee/Discount dialog</t>
+          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Verify the Part Sale Add/Edit fee-or-discount dialog shows the tax-jurisdiction note below the Taxable Yes/No dropdown</t>
+          <t>Verify the parts-sale per-part three-dot menu item reads 'Add Part Fee / Discount'</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -5274,30 +5298,34 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>TEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Per-part ⋮ menu text = 'Add Part Fee / Discount' exactly; opens 'New Part Fee / Discount' dialog.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-002</t>
+          <t>FD-PSALE-004</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr"/>
+          <t>C30625</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30625</t>
+        </is>
+      </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts Sale — Fees &amp; Discounts card</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Verify the parts-sale Fees &amp; Discounts column no longer shows the '+ Add' button, and the per-row and top-right three-dot entry points remain</t>
+          <t>Verify the Parts Sale Fees &amp; Discounts card shows each adjustment as plain text with the percentage in brackets (no colored badge)</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -5312,30 +5340,34 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. F&amp;D column has no '+ Add' (grep '+Add'=0); per-row ⋮ 'Add Part Fee / Discount' + top-right ⋮ 'Add Parts Sale Fee / Discount' both present.</t>
+          <t>/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Whole-sale card 'Parts Sale Fees &amp; Discounts' live: 'Customer Fee (10%) +$82.12', 'Sale Disc (−5%) −$41.06', 'Flat Fee +$50.00' (flat name-only), 'Processing Fee (6%) +$51.73' — plain text, no badge, bracket %/sign convention matches WO card item 5.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-003</t>
+          <t>FD-PSALE-006</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr"/>
+          <t>C30626</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30626</t>
+        </is>
+      </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts Sale — Financial Info card</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>Verify the parts-sale per-part three-dot menu item reads 'Add Part Fee / Discount'</t>
+          <t>Verify the parts-sale Financial Info card shows a 'Fees &amp; Discounts (N)' line directly above Subtotal and hides it when there are none</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -5350,30 +5382,34 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>TEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Per-part ⋮ menu text = 'Add Part Fee / Discount' exactly; opens 'New Part Fee / Discount' dialog.</t>
+          <t>ded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: 'Fees &amp; Discounts (6) $189.27' directly above Subtotal $963.95 in Financial Info.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-004</t>
+          <t>FD-PSALE-008</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr"/>
+          <t>C30627</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30627</t>
+        </is>
+      </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Parts Sale — Fees &amp; Discounts card</t>
+          <t>Part Sale — Fee/Discount dialog</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Verify the Parts Sale Fees &amp; Discounts card shows each adjustment as plain text with the percentage in brackets (no colored badge)</t>
+          <t>Verify the whole-parts-sale fee/discount dialog title reads 'New Parts Sale Fee / Discount' with subline 'Applying To: Entire Parts Sale'</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -5388,30 +5424,34 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Whole-sale card 'Parts Sale Fees &amp; Discounts' live: 'Customer Fee (10%) +$82.12', 'Sale Disc (−5%) −$41.06', 'Flat Fee +$50.00' (flat name-only), 'Processing Fee (6%) +$51.73' — plain text, no badge, bracket %/sign convention matches WO card item 5.</t>
+          <t>). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. VIU-CONFIRM RESOLVED (Picture 26 was missing): top-right ⋮ label CONFIRMED LIVE = 'Add Parts Sale Fee / Discount'; dialog title 'New Parts Sale Fee / Discount'; subline 'Applying To: Entire Parts Sale'. Case wording already matched.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-006</t>
+          <t>FD-PSALE-009</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C115" s="2" t="inlineStr"/>
+          <t>C30628</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30628</t>
+        </is>
+      </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Parts Sale — Financial Info card</t>
+          <t>Parts Sale — Statistics tab</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>Verify the parts-sale Financial Info card shows a 'Fees &amp; Discounts (N)' line directly above Subtotal and hides it when there are none</t>
+          <t>Verify the Fees &amp; Discounts section on the parts-sale Statistics tab shows the '%' and 'Amount' column headings</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -5426,35 +5466,39 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>ded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: 'Fees &amp; Discounts (6) $189.27' directly above Subtotal $963.95 in Financial Info.</t>
+          <t>ss rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Statistics F&amp;D (6) section live headings '% Amount'; flat fee blank %; rows +11%/+6%/+10% fees + −5% discounts; 'Total +$189.27'.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-008</t>
+          <t>FD-QB-012</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr"/>
+          <t>C28555</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28555</t>
+        </is>
+      </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Part Sale — Fee/Discount dialog</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Verify the whole-parts-sale fee/discount dialog title reads 'New Parts Sale Fee / Discount' with subline 'Applying To: Entire Parts Sale'</t>
+          <t>Verify the net subtotal floors at $0.00 ($100 parts + $10 tax, $150 discount: non-taxable vs taxable)</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -5464,35 +5508,39 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. VIU-CONFIRM RESOLVED (Picture 26 was missing): top-right ⋮ label CONFIRMED LIVE = 'Add Parts Sale Fee / Discount'; dialog title 'New Parts Sale Fee / Discount'; subline 'Applying To: Entire Parts Sale'. Case wording already matched.</t>
+          <t>floor worked-example halves re-proven at WO level: non-taxable over-discount -&gt; sub 0.00, tax UNCHANGED (9.14), total=tax, excess 117.24; taxable variant -&gt; tax 0.00, total 0.00 | WORDING+VIU 2026-07-13: In-app floor VERIFIED (same worked example as FD-CALC-015, confirmed 2026-07-10); the customer pays the tax only.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>FD-PSALE-009</t>
+          <t>FD-QB-014</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C117" s="2" t="inlineStr"/>
+          <t>C28557</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28557</t>
+        </is>
+      </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Parts Sale — Statistics tab</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Verify the Fees &amp; Discounts section on the parts-sale Statistics tab shows the '%' and 'Amount' column headings</t>
+          <t>Verify a mandatory warning/confirmation before saving when discounts are bigger than the net subtotal</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -5502,34 +5550,34 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>ss rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Statistics F&amp;D (6) section live headings '% Amount'; flat fee blank %; rows +11%/+6%/+10% fees + −5% discounts; 'Total +$189.27'.</t>
+          <t>FDBUG-15 CONFIRMED AGAIN (API half): over-discount saves 201 with NO warning payload; excess carried silently (117.24). Batch-6 UI shots show no warn/confirm dialog. Violates S6-R12 | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-15 / PO Q1 pending): an over-discount currently saves SILENTLY — no mandatory warn/confirm before saving. Expected kept as the spec requirement. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q1=A): PO ruled the warn/confirm is required AND already exists per spec (S6-R12) — it fires before invoicing and before marking the WO reviewed/complete, NOT when the adjustment is merely added (add is uncommitted; the Add dialog preview shows the resulting totals). Our FDBUG-15 'silent save' was observed at ADD time = the wrong trigger point; PO says that is intentional. FDBUG-15 reclassified NOT-A-DEFECT (no dev ticket released). Expected reworded to the commit-point warning. Status -&gt; VIU-Pending: the invoice/mark-reviewed/complete warning has not yet been observed live and needs a commit-time re-VIU. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). COMMIT-TIME RE-VIU 2026-07-14: attempted but BOTH qb cookie sets (cookies-viu.env 2026-07-13, cookies-fresh.env 2026-07-10) return 401 sso_required on quick-login (env woken, API root 200) — cookies EXPIRED. Left VIU-Pending: needs fresh qb cookies for the commit-time (invoice / mark-reviewed / complete) re-VIU. | COMMIT-TIME RE-VIU SETTLED 2026-07-14 (fresh qb cookies): VERIFIED. Live FE source + live data-condition confirm Chris's Q1=A exactly. (1) ADD-TIME SILENT: the Add/Edit dialog component (AdjustmentDialog) has NO over-discount warning and does not import the warning dialog -- adding an over-sized discount is silent (only an unrelated 'A percentage discount cannot exceed 100%' field check). (2) COMMIT-TIME WARN/CONFIRM BUILT: a dedicated component OverDiscountWarningDialog exists (title 'Discount exceeds subtotal'; body "The total discount exceeds this work order's subtotal. The subtotal will be reduced to $0.00, but any tax on the taxable base is still owed. The remaining $&lt;excess&gt; will be carried as a customer credit. Continue?"; buttons Continue / Cancel). It is imported and wired in the Invoice component: the Create-Invoice handler (Lt-&gt;_a) AND the mark-reviewed/Complete handler (Vt-&gt;ga, posts status:'complete') BOTH intercept when the excess-credit gate is true (FeesAndDiscounts flag ON &amp;&amp; not partSale &amp;&amp; adjustmentsSummary.excessCreditAmount&gt;0), open the dialog, and only run the commit on Continue (confirm) / abort on Cancel. So the mandatory warn/confirm fires at BOTH commit points, never silently. (3) LIVE DATA CONDITION: on WO S-15970 added a $9,999 whole-WO flat discount (reversible ZZAUTOTEST, removed after) -&gt; sub_total floored to $0.00, adjustmentsSummary.excessCreditAmount=9522.26 (&gt;0) =&gt; the FE gate evaluates TRUE, so the dialog would fire at Create Invoice / Mark-Reviewed / Complete. WO restored byte-identical to baseline afterward. Evidence: FE chunks OverDiscountWarningDialog.BCmTBE33.js + Invoice.Ny62BJnd.js + AdjustmentDialog.S8gN6cAn.js (captured live from qb.qa.shopview.com 2026-07-14); live API view before/after. Verdict: VIU-Verified. FDBUG-15 stays NOT-A-DEFECT (add-time silence is intentional). Expected wording already build-accurate (floor $0.00 + tax on taxable base still owed + exact excess as customer credit + must confirm) -&gt; no TestRail wording change needed; status flip local only. Exact on-screen labels now captured for the record: dialog 'Discount exceeds subtotal', buttons 'Continue'/'Cancel'.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>FD-QB-012</t>
+          <t>FD-REMOVE-001</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>C28555</t>
+          <t>C28479</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28555</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28479</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks — negative totals</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Verify the net subtotal floors at $0.00 ($100 parts + $10 tax, $150 discount: non-taxable vs taxable)</t>
+          <t>Verify removing a whole-work-order fee/discount shows the 'Remove Fee / Discount' confirm and a success message</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -5544,34 +5592,34 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>floor worked-example halves re-proven at WO level: non-taxable over-discount -&gt; sub 0.00, tax UNCHANGED (9.14), total=tax, excess 117.24; taxable variant -&gt; tax 0.00, total 0.00 | WORDING+VIU 2026-07-13: In-app floor VERIFIED (same worked example as FD-CALC-015, confirmed 2026-07-10); the customer pays the tax only.</t>
+          <t>remove-confirm wording drift per batch-1 (case-update); not re-driven today | WORDING+VIU 2026-07-13: Confirm dialog matched EXACTLY live: title 'Remove Fee / Discount', message 'Are you sure you want to remove this fee?', buttons 'Remove'/'Cancel' (shot inline-02; cancelled — no shared data deleted). Toast not re-observed this run. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>FD-QB-014</t>
+          <t>FD-REMOVE-002</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>C28557</t>
+          <t>C28480</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28557</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28480</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks — negative totals</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Verify a mandatory warning/confirmation before saving when discounts are bigger than the net subtotal</t>
+          <t>Verify removing a fee/discount uses Create and Edit, not a separate Delete permission</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -5586,24 +5634,24 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-15 CONFIRMED AGAIN (API half): over-discount saves 201 with NO warning payload; excess carried silently (117.24). Batch-6 UI shots show no warn/confirm dialog. Violates S6-R12 | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-15 / PO Q1 pending): an over-discount currently saves SILENTLY — no mandatory warn/confirm before saving. Expected kept as the spec requirement. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q1=A): PO ruled the warn/confirm is required AND already exists per spec (S6-R12) — it fires before invoicing and before marking the WO reviewed/complete, NOT when the adjustment is merely added (add is uncommitted; the Add dialog preview shows the resulting totals). Our FDBUG-15 'silent save' was observed at ADD time = the wrong trigger point; PO says that is intentional. FDBUG-15 reclassified NOT-A-DEFECT (no dev ticket released). Expected reworded to the commit-point warning. Status -&gt; VIU-Pending: the invoice/mark-reviewed/complete warning has not yet been observed live and needs a commit-time re-VIU. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). COMMIT-TIME RE-VIU 2026-07-14: attempted but BOTH qb cookie sets (cookies-viu.env 2026-07-13, cookies-fresh.env 2026-07-10) return 401 sso_required on quick-login (env woken, API root 200) — cookies EXPIRED. Left VIU-Pending: needs fresh qb cookies for the commit-time (invoice / mark-reviewed / complete) re-VIU. | COMMIT-TIME RE-VIU SETTLED 2026-07-14 (fresh qb cookies): VERIFIED. Live FE source + live data-condition confirm Chris's Q1=A exactly. (1) ADD-TIME SILENT: the Add/Edit dialog component (AdjustmentDialog) has NO over-discount warning and does not import the warning dialog -- adding an over-sized discount is silent (only an unrelated 'A percentage discount cannot exceed 100%' field check). (2) COMMIT-TIME WARN/CONFIRM BUILT: a dedicated component OverDiscountWarningDialog exists (title 'Discount exceeds subtotal'; body "The total discount exceeds this work order's subtotal. The subtotal will be reduced to $0.00, but any tax on the taxable base is still owed. The remaining $&lt;excess&gt; will be carried as a customer credit. Continue?"; buttons Continue / Cancel). It is imported and wired in the Invoice component: the Create-Invoice handler (Lt-&gt;_a) AND the mark-reviewed/Complete handler (Vt-&gt;ga, posts status:'complete') BOTH intercept when the excess-credit gate is true (FeesAndDiscounts flag ON &amp;&amp; not partSale &amp;&amp; adjustmentsSummary.excessCreditAmount&gt;0), open the dialog, and only run the commit on Continue (confirm) / abort on Cancel. So the mandatory warn/confirm fires at BOTH commit points, never silently. (3) LIVE DATA CONDITION: on WO S-15970 added a $9,999 whole-WO flat discount (reversible ZZAUTOTEST, removed after) -&gt; sub_total floored to $0.00, adjustmentsSummary.excessCreditAmount=9522.26 (&gt;0) =&gt; the FE gate evaluates TRUE, so the dialog would fire at Create Invoice / Mark-Reviewed / Complete. WO restored byte-identical to baseline afterward. Evidence: FE chunks OverDiscountWarningDialog.BCmTBE33.js + Invoice.Ny62BJnd.js + AdjustmentDialog.S8gN6cAn.js (captured live from qb.qa.shopview.com 2026-07-14); live API view before/after. Verdict: VIU-Verified. FDBUG-15 stays NOT-A-DEFECT (add-time silence is intentional). Expected wording already build-accurate (floor $0.00 + tax on taxable base still owed + exact excess as customer credit + must confirm) -&gt; no TestRail wording change needed; status flip local only. Exact on-screen labels now captured for the record: dialog 'Discount exceeds subtotal', buttons 'Continue'/'Cancel'.</t>
+          <t>removal governed by Create&amp;Edit (tech WITH lines-C&amp;E removed line-level 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove uses Create &amp; Edit not a separate Delete permission; carry prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>FD-REMOVE-001</t>
+          <t>FD-REMOVE-003</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>C28479</t>
+          <t>C28481</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28479</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28481</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5613,12 +5661,12 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a whole-work-order fee/discount shows the 'Remove Fee / Discount' confirm and a success message</t>
+          <t>Verify removing a line-level fee/discount from its inline ⋮ menu</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -5628,34 +5676,34 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>remove-confirm wording drift per batch-1 (case-update); not re-driven today | WORDING+VIU 2026-07-13: Confirm dialog matched EXACTLY live: title 'Remove Fee / Discount', message 'Are you sure you want to remove this fee?', buttons 'Remove'/'Cancel' (shot inline-02; cancelled — no shared data deleted). Toast not re-observed this run. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>line-level remove 204 and gone from the line | WORDING+VIU 2026-07-13: Inline menu option is 'Remove' (was 'Delete'); confirm dialog 'Remove Fee / Discount' confirmed live.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>FD-REMOVE-002</t>
+          <t>FD-STACK-001</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>C28480</t>
+          <t>C28482</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28480</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28482</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Remove an adjustment</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a fee/discount uses Create and Edit, not a separate Delete permission</t>
+          <t>Verify multiple fees/discounts on one part each work out on the part's own total (they do not compound)</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -5670,39 +5718,39 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>removal governed by Create&amp;Edit (tech WITH lines-C&amp;E removed line-level 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove uses Create &amp; Edit not a separate Delete permission; carry prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>part flat + part pct resolved independently on the part's own gross (fresh: $8.00 and $17.08 coexist, no compounding) | WORDING+VIU 2026-07-13: Netting carried; build labels. Display half (only first shows + 'Show N more') is the FD-INLINE-003 deviation (no Show-N-more in this build).</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>FD-REMOVE-003</t>
+          <t>FD-STACK-002</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>C28481</t>
+          <t>C28483</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28481</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28483</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Remove an adjustment</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a line-level fee/discount from its inline ⋮ menu</t>
+          <t>Verify two whole-work-order percentage fees/discounts use the same totals and do not change each other's base</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -5712,24 +5760,24 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>line-level remove 204 and gone from the line | WORDING+VIU 2026-07-13: Inline menu option is 'Remove' (was 'Delete'); confirm dialog 'Remove Fee / Discount' confirmed live.</t>
+          <t>two 10% whole-WO fees resolve 17.08 each (same base, no compounding) | WORDING+VIU 2026-07-13: Same-base netting carried; build labels.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>FD-STACK-001</t>
+          <t>FD-STACK-003</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>C28482</t>
+          <t>C28484</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28482</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28484</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -5739,12 +5787,12 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Verify multiple fees/discounts on one part each work out on the part's own total (they do not compound)</t>
+          <t>Verify the same template can be applied to one work order more than once by hand</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -5754,34 +5802,34 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>part flat + part pct resolved independently on the part's own gross (fresh: $8.00 and $17.08 coexist, no compounding) | WORDING+VIU 2026-07-13: Netting carried; build labels. Display half (only first shows + 'Show N more') is the FD-INLINE-003 deviation (no Show-N-more in this build).</t>
+          <t>'Flat fee' template applied twice by hand -&gt; 201/201, two distinct adjustments | WORDING+VIU 2026-07-13: Same-template-twice carried; build labels ('Add Fee/Discount', 'Apply From Template', 'WO Fees &amp; Discounts'). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>FD-STACK-002</t>
+          <t>FD-STATS-001</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>C28483</t>
+          <t>C28459</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28483</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28459</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Verify two whole-work-order percentage fees/discounts use the same totals and do not change each other's base</t>
+          <t>Verify the Stats tab Fees &amp; Discounts section shows the '%' and 'Amount' column headings with each row's value and amount</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -5796,39 +5844,39 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>two 10% whole-WO fees resolve 17.08 each (same base, no compounding) | WORDING+VIU 2026-07-13: Same-base netting carried; build labels.</t>
+          <t>CONFIRMED AGAIN: Stats shows aggregate 'Fees &amp; Discounts (5) $25.00' style block, NOT the per-row Value/%+Amount table — PO Q1=B design regression persists (shot 07-stats) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-2): the Stats 'Fees &amp; Discounts (N)' section lists rows (name, a value/% for percentages, and an amount) but has NO 'Value'/'Amount' column headers like the other Stats sections. Confirmed live (shot fin-01). | SV-8479/8480 deconfliction 2026-07-22: added the right-side '%' and 'Amount' column headings + blank-% for flat fees (item 12). Absorbs dropped new case FD-WO-027. viu_status unchanged (VIU-Deviation) — re-observe at VIU. | VIU 2026-07-22 LIVE: prior 'no headers' deviation RESOLVED — Stats tab 'Fees &amp; Discounts (10)' section now shows the '% Amount' column headings. Rows show percent under % (blank for flat: 'Flat Fee 2 +$32.00', 'Flat Fee +$11.00') and signed amount under Amount ('Labor Fee +20% +$101.98', 'Labor Disc −10% −$50.99', 'Customer Fee +10% +$65.88', 'WO Disc −5% −$32.94'), with 'Total +$273.31'. Ev: wo/FD-STATS-001-stats-tab.png, wo/stats-bodytext.txt.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>FD-STACK-003</t>
+          <t>FD-STATS-003</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>C28484</t>
+          <t>C28461</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28484</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28461</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Verify the same template can be applied to one work order more than once by hand</t>
+          <t>Verify the Stats 'Fees &amp; Discounts' total equals the signed sum of all the amounts</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -5838,24 +5886,24 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>'Flat fee' template applied twice by hand -&gt; 201/201, two distinct adjustments | WORDING+VIU 2026-07-13: Same-template-twice carried; build labels ('Add Fee/Discount', 'Apply From Template', 'WO Fees &amp; Discounts'). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>net = signed sum re-consistent (adjustmentsSummary netAmount matches card); full UI table from batch-2 | WORDING+VIU 2026-07-13: Total = signed sum; carry prior VIU. Minus-sign jargon removed.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-001</t>
+          <t>FD-STATS-005</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>C28459</t>
+          <t>C28463</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28459</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28463</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -5865,12 +5913,12 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats tab Fees &amp; Discounts section shows the '%' and 'Amount' column headings with each row's value and amount</t>
+          <t>Verify the Stats 'Fees &amp; Discounts' section is hidden when the work order has no fees/discounts</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -5880,34 +5928,34 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED AGAIN: Stats shows aggregate 'Fees &amp; Discounts (5) $25.00' style block, NOT the per-row Value/%+Amount table — PO Q1=B design regression persists (shot 07-stats) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-2): the Stats 'Fees &amp; Discounts (N)' section lists rows (name, a value/% for percentages, and an amount) but has NO 'Value'/'Amount' column headers like the other Stats sections. Confirmed live (shot fin-01). | SV-8479/8480 deconfliction 2026-07-22: added the right-side '%' and 'Amount' column headings + blank-% for flat fees (item 12). Absorbs dropped new case FD-WO-027. viu_status unchanged (VIU-Deviation) — re-observe at VIU. | VIU 2026-07-22 LIVE: prior 'no headers' deviation RESOLVED — Stats tab 'Fees &amp; Discounts (10)' section now shows the '% Amount' column headings. Rows show percent under % (blank for flat: 'Flat Fee 2 +$32.00', 'Flat Fee +$11.00') and signed amount under Amount ('Labor Fee +20% +$101.98', 'Labor Disc −10% −$50.99', 'Customer Fee +10% +$65.88', 'WO Disc −5% −$32.94'), with 'Total +$273.31'. Ev: wo/FD-STATS-001-stats-tab.png, wo/stats-bodytext.txt.</t>
+          <t>no-adjustments WO -&gt; adjustments=[] + all-zero summary -&gt; section hidden | WORDING+VIU 2026-07-13: Section hidden with no adjustments; carry prior VIU.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-003</t>
+          <t>FD-TMPL-001</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>C28461</t>
+          <t>C28502</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28461</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28502</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Template admin — location</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats 'Fees &amp; Discounts' total equals the signed sum of all the amounts</t>
+          <t>Verify the fee/discount template library is at Administration → Service → Fees &amp; Discounts (below Canned Lines)</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -5922,39 +5970,39 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>net = signed sum re-consistent (adjustmentsSummary netAmount matches card); full UI table from batch-2 | WORDING+VIU 2026-07-13: Total = signed sum; carry prior VIU. Minus-sign jargon removed.</t>
+          <t>admin library lives under Administration -&gt; FINANCE (route /administration/adjustment-templates), not Service-below-Canned-Lines; page re-loaded today (case-update per S13-R8 target) | WORDING+VIU 2026-07-13: CORRECTED location: templates live under Administration → FINANCE → 'Fees &amp; Discounts' (below 'Payment Methods'), NOT 'Service, below Canned Lines' (Canned Lines is under SERVICE). Confirmed live (shot tmpl-02-create-dialog). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-005</t>
+          <t>FD-TMPL-002</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>C28463</t>
+          <t>C28503</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28463</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28503</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Template admin — list</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats 'Fees &amp; Discounts' section is hidden when the work order has no fees/discounts</t>
+          <t>Verify the template list columns and the edit/delete actions</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -5964,34 +6012,34 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>no-adjustments WO -&gt; adjustments=[] + all-zero summary -&gt; section hidden | WORDING+VIU 2026-07-13: Section hidden with no adjustments; carry prior VIU.</t>
+          <t>list + delete action per batch-1; page renders today; columns not re-verified individually | WORDING+VIU 2026-07-13: List columns confirmed live (shot tmpl-02). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-001</t>
+          <t>FD-TMPL-003</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>C28502</t>
+          <t>C28504</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28502</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28504</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Template admin — location</t>
+          <t>Template admin — create</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Verify the fee/discount template library is at Administration → Service → Fees &amp; Discounts (below Canned Lines)</t>
+          <t>Verify creating a Fee template (dialog fields and the Create button)</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -6006,39 +6054,39 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>admin library lives under Administration -&gt; FINANCE (route /administration/adjustment-templates), not Service-below-Canned-Lines; page re-loaded today (case-update per S13-R8 target) | WORDING+VIU 2026-07-13: CORRECTED location: templates live under Administration → FINANCE → 'Fees &amp; Discounts' (below 'Payment Methods'), NOT 'Service, below Canned Lines' (Canned Lines is under SERVICE). Confirmed live (shot tmpl-02-create-dialog). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>PARTIAL IMPROVEMENT: create-dialog title NOW 'New Fee / Discount' (matches spec; was 'Add new fee/discount'); confirm button still 'Create' (spec 'Add Fee / Discount') and toast 'Template created' per batch-1 — drift remains | WORDING+VIU 2026-07-13: Create dialog confirmed live: title 'New Fee / Discount', fields Name/Type/Calculation Type/'$ Default Amount'/Taxable toggle/'Auto-apply to new work orders' toggle/'Description (Optional)', 'Create' button. Type offers only Fee/Discount (Processing Fee is NOT in the builder — Story 8 not built). Create API 201 live. Toast text carried from prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-002</t>
+          <t>FD-TMPL-004</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>C28503</t>
+          <t>C28505</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28503</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28505</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Template admin — list</t>
+          <t>Template admin — create</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Verify the template list columns and the edit/delete actions</t>
+          <t>Verify creating a Discount template</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -6048,34 +6096,34 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>list + delete action per batch-1; page renders today; columns not re-verified individually | WORDING+VIU 2026-07-13: List columns confirmed live (shot tmpl-02). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>generic 'Template created' toast vs spec 'Discount added' per batch-1; not re-driven | WORDING+VIU 2026-07-13: CORRECTED title: the toast is generic (not a per-type 'Discount added'). Create dialog + list confirmed live. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-003</t>
+          <t>FD-TMPL-005</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>C28504</t>
+          <t>C28506</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28504</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28506</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Template admin — create</t>
+          <t>Template admin — auto-apply</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>Verify creating a Fee template (dialog fields and the Create button)</t>
+          <t>Verify the 'Auto-apply to all new work orders at this location' checkbox adds the template to every new work order at that location</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -6090,34 +6138,34 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL IMPROVEMENT: create-dialog title NOW 'New Fee / Discount' (matches spec; was 'Add new fee/discount'); confirm button still 'Create' (spec 'Add Fee / Discount') and toast 'Template created' per batch-1 — drift remains | WORDING+VIU 2026-07-13: Create dialog confirmed live: title 'New Fee / Discount', fields Name/Type/Calculation Type/'$ Default Amount'/Taxable toggle/'Auto-apply to new work orders' toggle/'Description (Optional)', 'Create' button. Type offers only Fee/Discount (Processing Fee is NOT in the builder — Story 8 not built). Create API 201 live. Toast text carried from prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>auto-apply template ('Capped discount' + test pfees) landed on every fresh WO as appliedBy=auto | WORDING+VIU 2026-07-13: CORRECTED auto-apply label: dialog toggle is 'Auto-apply to new work orders'; list column 'Auto-Apply To Work Orders'. Confirmed live (shot tmpl-02). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-004</t>
+          <t>FD-TMPL-006</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>C28505</t>
+          <t>C28507</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28505</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28507</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Template admin — create</t>
+          <t>Template admin — edit</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>Verify creating a Discount template</t>
+          <t>Verify editing a template (Edit Fee / Discount dialog, 'Save' button)</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -6132,34 +6180,34 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>generic 'Template created' toast vs spec 'Discount added' per batch-1; not re-driven | WORDING+VIU 2026-07-13: CORRECTED title: the toast is generic (not a per-type 'Discount added'). Create dialog + list confirmed live. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>edit locks Type+Calc on template edit (spec locks only in WO dialog) per batch-1; not re-driven | WORDING+VIU 2026-07-13: Edit dialog title 'Edit Fee / Discount' + 'Save' button confirmed on the fee/discount Edit dialog (shot edit-01). Edit opens from the row's pencil button. Toast text carried.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-005</t>
+          <t>FD-TMPL-007</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>C28506</t>
+          <t>C28508</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28506</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28508</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Template admin — auto-apply</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Verify the 'Auto-apply to all new work orders at this location' checkbox adds the template to every new work order at that location</t>
+          <t>Verify the template delete confirm dialog and buttons</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -6174,34 +6222,34 @@
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>auto-apply template ('Capped discount' + test pfees) landed on every fresh WO as appliedBy=auto | WORDING+VIU 2026-07-13: CORRECTED auto-apply label: dialog toggle is 'Auto-apply to new work orders'; list column 'Auto-Apply To Work Orders'. Confirmed live (shot tmpl-02). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>delete-confirm dialog + affectedCustomerCount warning per batch-1; delete-precondition endpoint intact | WORDING+VIU 2026-07-13: Delete confirm confirmed live: standardized 'Delete Template' dialog with 'Cancel' + red 'Delete' (shot tmpl-03). The plain (no-customer) body wording was not captured this run — the sample template had a customer default (see FD-TMPL-008).</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-006</t>
+          <t>FD-TMPL-008</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>C28507</t>
+          <t>C28509</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28507</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28509</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Template admin — edit</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Verify editing a template (Edit Fee / Discount dialog, 'Save' button)</t>
+          <t>Verify the delete confirm adds a warning when the template is a customer default</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -6216,24 +6264,24 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>edit locks Type+Calc on template edit (spec locks only in WO dialog) per batch-1; not re-driven | WORDING+VIU 2026-07-13: Edit dialog title 'Edit Fee / Discount' + 'Save' button confirmed on the fee/discount Edit dialog (shot edit-01). Edit opens from the row's pencil button. Toast text carried.</t>
+          <t>standardized 'Delete Template' dialog wording = intended per epic; case-update to adopt live wording still pending | WORDING+VIU 2026-07-13: Customer-default warning confirmed live EXACTLY: 'This template is set as a default for N customer(s). Deleting it will remove it from them.' (saw '1 customer', shot tmpl-03).</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-007</t>
+          <t>FD-TMPL-009</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>C28508</t>
+          <t>C28510</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28508</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28510</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6243,7 +6291,7 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Verify the template delete confirm dialog and buttons</t>
+          <t>Verify deleting a template leaves work-order fees/discounts made from it unchanged</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -6258,34 +6306,34 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>delete-confirm dialog + affectedCustomerCount warning per batch-1; delete-precondition endpoint intact | WORDING+VIU 2026-07-13: Delete confirm confirmed live: standardized 'Delete Template' dialog with 'Cancel' + red 'Delete' (shot tmpl-03). The plain (no-customer) body wording was not captured this run — the sample template had a customer default (see FD-TMPL-008).</t>
+          <t>template deleted (204) -&gt; WO adjustment made from it survives unchanged (resolved 6 intact) | WORDING+VIU 2026-07-13: Delete leaves WO adjustments unchanged; carried. Nav corrected to Finance. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-008</t>
+          <t>FD-TMPL-011</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>C28509</t>
+          <t>C28512</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28509</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28512</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Template admin — delete</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Verify the delete confirm adds a warning when the template is a customer default</t>
+          <t>Verify Max Amount shows only for percentage methods and how 0 behaves</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -6300,39 +6348,39 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>standardized 'Delete Template' dialog wording = intended per epic; case-update to adopt live wording still pending | WORDING+VIU 2026-07-13: Customer-default warning confirmed live EXACTLY: 'This template is set as a default for N customer(s). Deleting it will remove it from them.' (saw '1 customer', shot tmpl-03).</t>
+          <t>maxCap 0 accepted and STORED as 0 on the template (201) and WO resolve treats 0 as NO cap (34.15) — FDBUG-9 persists | WORDING+VIU 2026-07-13: Max Amount only for % confirmed (WO+template dialogs). DEVIATION (PO Q2): a Max Amount of 0 is treated as 'no cap'. Labels cleaned. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount = 'no limit' (WAD, S2-R25). 0-handling no longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-009</t>
+          <t>FD-TMPL-013</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>C28510</t>
+          <t>C28514</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28510</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28514</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Template admin — delete</t>
+          <t>Template admin — validation</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Verify deleting a template leaves work-order fees/discounts made from it unchanged</t>
+          <t>Verify a percentage-discount template cannot go over 100% while a percentage-fee template has no cap</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -6342,24 +6390,24 @@
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>template deleted (204) -&gt; WO adjustment made from it survives unchanged (resolved 6 intact) | WORDING+VIU 2026-07-13: Delete leaves WO adjustments unchanged; carried. Nav corrected to Finance. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>discount template 150% -&gt; 400; fee template 150% -&gt; 201 | WORDING+VIU 2026-07-13: %&gt;100 discount rejected (confirmed via API 2026-07-13: 'A percentage discount cannot exceed 100%').</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-011</t>
+          <t>FD-TMPL-014</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>C28512</t>
+          <t>C28515</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28512</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28515</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6369,7 +6417,7 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Verify Max Amount shows only for percentage methods and how 0 behaves</t>
+          <t>Verify a Fee/Discount template offers the four whole-work-order methods and no scope field</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -6384,39 +6432,39 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>maxCap 0 accepted and STORED as 0 on the template (201) and WO resolve treats 0 as NO cap (34.15) — FDBUG-9 persists | WORDING+VIU 2026-07-13: Max Amount only for % confirmed (WO+template dialogs). DEVIATION (PO Q2): a Max Amount of 0 is treated as 'no cap'. Labels cleaned. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount = 'no limit' (WAD, S2-R25). 0-handling no longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md).</t>
+          <t>builder offers exactly 4 whole-WO methods (Flat, % Labor, % Parts, % Subtotal), no scope field, no legacy '% Labor+Parts' | WORDING+VIU 2026-07-13: Calc Type options confirmed (same 4 whole-WO methods as the WO dialog); no scope field.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-013</t>
+          <t>FD-TMPL-015</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>C28514</t>
+          <t>C28516</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28514</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28516</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Template admin — validation</t>
+          <t>Template admin — negative</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Verify a percentage-discount template cannot go over 100% while a percentage-fee template has no cap</t>
+          <t>Verify the template save-failure message</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -6426,39 +6474,39 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>discount template 150% -&gt; 400; fee template 150% -&gt; 201 | WORDING+VIU 2026-07-13: %&gt;100 discount rejected (confirmed via API 2026-07-13: 'A percentage discount cannot exceed 100%').</t>
+          <t>template empty name -&gt; 400; amount 0 -&gt; 400 (save-failure surfaced) | WORDING+VIU 2026-07-13: Save-failure toast text carried from prior VIU (not force-failed this run).</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-014</t>
+          <t>FD-TMPL-016</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>C28515</t>
+          <t>C28517</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28515</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28517</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Template admin — dialog fields</t>
+          <t>Template admin — permissions</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Verify a Fee/Discount template offers the four whole-work-order methods and no scope field</t>
+          <t>Verify the admin Fees &amp; Discounts page needs the Settings → Service permission</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -6468,34 +6516,34 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>builder offers exactly 4 whole-WO methods (Flat, % Labor, % Parts, % Subtotal), no scope field, no legacy '% Labor+Parts' | WORDING+VIU 2026-07-13: Calc Type options confirmed (same 4 whole-WO methods as the WO dialog); no scope field.</t>
+          <t>BE-enforced: tech templates GET/POST -&gt; 403; page FE-gated settingsFinance | WORDING+VIU 2026-07-13: Templates admin is back-end gated by Settings → Finance (Tech → 403), established batch-2. Nav corrected to Finance. NOTE: re-check the Tech negative after the roles matrix is re-derived (Technician drifted on shared qb). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-015</t>
+          <t>FD-TMPL-017</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>C28516</t>
+          <t>C28518</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28516</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28518</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Template admin — negative</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>Verify the template save-failure message</t>
+          <t>Verify the template Name is limited to 100 characters</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -6510,39 +6558,39 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>template empty name -&gt; 400; amount 0 -&gt; 400 (save-failure surfaced) | WORDING+VIU 2026-07-13: Save-failure toast text carried from prior VIU (not force-failed this run).</t>
+          <t>name 100ch -&gt; 201; 101ch -&gt; 400 | WORDING+VIU 2026-07-13: Name 100-char limit carried.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-016</t>
+          <t>FD-TMPL-018</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>C28517</t>
+          <t>C29917</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28517</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29917</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Template admin — permissions</t>
+          <t>Template admin — jurisdiction note</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Verify the admin Fees &amp; Discounts page needs the Settings → Service permission</t>
+          <t>Verify the admin Fee/Discount template dialog shows the tax-jurisdiction note below the Taxable Yes/No dropdown (for every kind)</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -6552,39 +6600,39 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>BE-enforced: tech templates GET/POST -&gt; 403; page FE-gated settingsFinance | WORDING+VIU 2026-07-13: Templates admin is back-end gated by Settings → Finance (Tech → 403), established batch-2. Nav corrected to Finance. NOTE: re-check the Tech negative after the roles matrix is re-derived (Technician drifted on shared qb). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-017</t>
+          <t>FD-VAL-001</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>C28518</t>
+          <t>C28599</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28518</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28599</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Template admin — dialog fields</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Verify the template Name is limited to 100 characters</t>
+          <t>Verify the Add button stays disabled until Name, Type, Calculation Type and an Amount above 0 are all set</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -6594,39 +6642,39 @@
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>name 100ch -&gt; 201; 101ch -&gt; 400 | WORDING+VIU 2026-07-13: Name 100-char limit carried.</t>
+          <t>CONFIRMED AGAIN: Add button enabled on empty form (validates on submit) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: DEVIATION re-confirmed 2026-07-13 (BUG-FD-4): the 'Add Fee' button is ENABLED on an empty form (validates on submit). Labels build-accurate (Add Fee/Add Discount, Calculation Type, Max Amount). | STAGING VIU 2026-07-20 staging LIVE VIU: BUG-FD-4 FIXED on staging: confirm button disabled until Name+Type+Calc+Amount&gt;0 set. Live-observed (dev-wo-emptyform + part-sale Add Fee disabled-until-valid). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-018</t>
+          <t>FD-VAL-002</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>C29917</t>
+          <t>C28600</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29917</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28600</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Template admin — jurisdiction note</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Verify the admin Fee/Discount template dialog shows the tax-jurisdiction note below the Taxable Yes/No dropdown (for every kind)</t>
+          <t>Verify a blank or 0 amount blocks saving, with an error</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -6636,24 +6684,24 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>amount 0 -&gt; 400 (API); UI inline error on submit | WORDING+VIU 2026-07-13: Blank/0 amount blocked; carry prior VIU. Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-001</t>
+          <t>FD-VAL-003</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>C28599</t>
+          <t>C28601</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28599</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28601</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6663,12 +6711,12 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Verify the Add button stays disabled until Name, Type, Calculation Type and an Amount above 0 are all set</t>
+          <t>Verify an empty Name blocks saving, with an error (Name required, up to 100 characters)</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -6678,24 +6726,24 @@
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED AGAIN: Add button enabled on empty form (validates on submit) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: DEVIATION re-confirmed 2026-07-13 (BUG-FD-4): the 'Add Fee' button is ENABLED on an empty form (validates on submit). Labels build-accurate (Add Fee/Add Discount, Calculation Type, Max Amount). | STAGING VIU 2026-07-20 staging LIVE VIU: BUG-FD-4 FIXED on staging: confirm button disabled until Name+Type+Calc+Amount&gt;0 set. Live-observed (dev-wo-emptyform + part-sale Add Fee disabled-until-valid). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>UI blocks empty name (inline required error). NEW FDBUG-16: raw API now ACCEPTS empty-name adds (201; regression vs batch-3 400) — FE-only guard; name 101ch -&gt; 400, 100ch -&gt; 201 | WORDING+VIU 2026-07-13: Empty name blocked in UI; 100-char limit. (Raw back-end accepts empty name — FDBUG-16 — but the dialog blocks it.) | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-002</t>
+          <t>FD-VAL-004</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>C28600</t>
+          <t>C28602</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28600</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28602</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6705,7 +6753,7 @@
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Verify a blank or 0 amount blocks saving, with an error</t>
+          <t>Verify a percentage discount over 100% is invalid while a percentage fee has no upper cap</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
@@ -6720,24 +6768,24 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>amount 0 -&gt; 400 (API); UI inline error on submit | WORDING+VIU 2026-07-13: Blank/0 amount blocked; carry prior VIU. Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>discount &gt;100% invalid (400), fee uncapped (201) | WORDING+VIU 2026-07-13: %&gt;100 discount invalid, fee uncapped; carry prior VIU. Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-003</t>
+          <t>FD-VAL-005</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>C28601</t>
+          <t>C28603</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28601</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28603</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6747,7 +6795,7 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Verify an empty Name blocks saving, with an error (Name required, up to 100 characters)</t>
+          <t>Verify negative amounts are rejected (values must be above 0)</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -6762,24 +6810,24 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>UI blocks empty name (inline required error). NEW FDBUG-16: raw API now ACCEPTS empty-name adds (201; regression vs batch-3 400) — FE-only guard; name 101ch -&gt; 400, 100ch -&gt; 201 | WORDING+VIU 2026-07-13: Empty name blocked in UI; 100-char limit. (Raw back-end accepts empty name — FDBUG-16 — but the dialog blocks it.) | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>negative amount -&gt; 400 | WORDING+VIU 2026-07-13: Negatives rejected; carry prior VIU. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-004</t>
+          <t>FD-VAL-006</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>C28602</t>
+          <t>C28604</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28602</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28604</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6789,12 +6837,12 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>Verify a percentage discount over 100% is invalid while a percentage fee has no upper cap</t>
+          <t>Verify the Max Amount field shows only for percentage methods and how 0 or empty behaves</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -6804,24 +6852,24 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>discount &gt;100% invalid (400), fee uncapped (201) | WORDING+VIU 2026-07-13: %&gt;100 discount invalid, fee uncapped; carry prior VIU. Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>FDBUG-9: maxCap 0 behaves as NO cap (not 'no maximum' spec reading matches build for empty, but 0 disagrees w/ §5-R6 $0-forces-$0) — persists | WORDING+VIU 2026-07-13: Confirmed live: '$ Max Amount (Optional)' appears only for percentage methods (hidden for Flat Amount, shots wo-03/wo-05). DEVIATION (FDBUG-9 / PO Q2 pending): whether a Max Amount of 0 means 'no cap' or 'cap at $0.00' is a pending product decision — expected kept as current build behavior. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount = 'no limit' (WAD, S2-R25). 0-handling no longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-005</t>
+          <t>FD-VAL-007</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>C28603</t>
+          <t>C28605</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28603</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28605</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6831,7 +6879,7 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Verify negative amounts are rejected (values must be above 0)</t>
+          <t>Verify a template that is both auto-apply at the location and a customer default is added only ONCE to a new work order</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
@@ -6846,39 +6894,39 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>negative amount -&gt; 400 | WORDING+VIU 2026-07-13: Negatives rejected; carry prior VIU. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>auto+default template -&gt; exactly ONE adjustment on the new WO | WORDING+VIU 2026-07-13: Double-add does not stack (one adjustment); carry prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-006</t>
+          <t>FD-WO-001</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>C28604</t>
+          <t>C28424</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28604</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28424</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Verify the Max Amount field shows only for percentage methods and how 0 or empty behaves</t>
+          <t>Verify the whole-work-order fee/discount dialog opens from the toolbar menu with title 'New Work Order Fee / Discount'</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -6888,39 +6936,39 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-9: maxCap 0 behaves as NO cap (not 'no maximum' spec reading matches build for empty, but 0 disagrees w/ §5-R6 $0-forces-$0) — persists | WORDING+VIU 2026-07-13: Confirmed live: '$ Max Amount (Optional)' appears only for percentage methods (hidden for Flat Amount, shots wo-03/wo-05). DEVIATION (FDBUG-9 / PO Q2 pending): whether a Max Amount of 0 means 'no cap' or 'cap at $0.00' is a pending product decision — expected kept as current build behavior. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount = 'no limit' (WAD, S2-R25). 0-handling no longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>dialog title still 'Add new fee/discount' (spec 'New Fee / Discount'), menu item 'Add Fee/Discount' — label drift persists (UI re-driven, shot 10-wo-add-dialog) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Now build-accurate (was VIU-Deviation only because the case used the older spec wording). Dialog shows no work-order-number subtitle in this build (old expected claim dropped). | SV-8479/8480 deconfliction 2026-07-22: menu item 'Add Fee/Discount' -&gt; 'Add Work Order Fee / Discount' (item 10); title 'Add new fee/discount' -&gt; 'New Work Order Fee / Discount' + new subline 'Applying To: Entire Work Order' (item 11, reverses the old 'no Applying-to line' claim). Absorbs dropped new case FD-WO-026. | VIU 2026-07-22 LIVE: whole-WO dialog opens from toolbar menu; title 'New Work Order Fee / Discount', subline 'Applying To: Entire Work Order', no scope dropdown. Ev: wo/FD-WO-001-wo-dialog.png, wo/wo-dialog-text.txt.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>FD-VAL-007</t>
+          <t>FD-WO-002</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>C28605</t>
+          <t>C28425</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28605</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28425</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>Verify a template that is both auto-apply at the location and a customer default is added only ONCE to a new work order</t>
+          <t>Verify adding a whole-work-order flat-amount fee saves and shows a success message</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -6930,24 +6978,24 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>auto+default template -&gt; exactly ONE adjustment on the new WO | WORDING+VIU 2026-07-13: Double-add does not stack (one adjustment); carry prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>whole-WO flat fee add 201 + visible in WO view (flat 7.77 resolved exactly) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Sidebar card is 'WO Fees &amp; Discounts' (was 'Work Order Fee / Discount'). Exact success-toast text not re-captured this pass (worded as 'a success message'). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-001</t>
+          <t>FD-WO-003</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>C28424</t>
+          <t>C28426</t>
         </is>
       </c>
       <c r="C152" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28424</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28426</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6957,12 +7005,12 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Verify the whole-work-order fee/discount dialog opens from the toolbar menu with title 'New Work Order Fee / Discount'</t>
+          <t>Verify the live preview shows a whole-work-order percentage discount before you save</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -6972,24 +7020,24 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>dialog title still 'Add new fee/discount' (spec 'New Fee / Discount'), menu item 'Add Fee/Discount' — label drift persists (UI re-driven, shot 10-wo-add-dialog) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Now build-accurate (was VIU-Deviation only because the case used the older spec wording). Dialog shows no work-order-number subtitle in this build (old expected claim dropped). | SV-8479/8480 deconfliction 2026-07-22: menu item 'Add Fee/Discount' -&gt; 'Add Work Order Fee / Discount' (item 10); title 'Add new fee/discount' -&gt; 'New Work Order Fee / Discount' + new subline 'Applying To: Entire Work Order' (item 11, reverses the old 'no Applying-to line' claim). Absorbs dropped new case FD-WO-026. | VIU 2026-07-22 LIVE: whole-WO dialog opens from toolbar menu; title 'New Work Order Fee / Discount', subline 'Applying To: Entire Work Order', no scope dropdown. Ev: wo/FD-WO-001-wo-dialog.png, wo/wo-dialog-text.txt.</t>
+          <t>dialog live preview re-driven ($5 flat -&gt; '+$5.00 / New work-order subtotal $187.76'); pct preview math not re-driven, API pct resolution re-proven (10%-&gt;17.08) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calc type corrected from generic 'Percentage' to the real whole-WO option '% of Subtotal'. Exact preview row labels not re-captured this pass (behavior verified 2026-07-10). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-002</t>
+          <t>FD-WO-004</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>C28425</t>
+          <t>C28427</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28425</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28427</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6999,12 +7047,12 @@
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>Verify adding a whole-work-order flat-amount fee saves and shows a success message</t>
+          <t>Verify 'Apply From Template' fills the dialog with a template's values</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -7014,24 +7062,24 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>whole-WO flat fee add 201 + visible in WO view (flat 7.77 resolved exactly) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Sidebar card is 'WO Fees &amp; Discounts' (was 'Work Order Fee / Discount'). Exact success-toast text not re-captured this pass (worded as 'a success message'). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>not re-driven today (Apply-From-Template combobox present in dialog); templateId add path re-proven via API (FD-STACK-003) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Dropdown label is exactly 'Apply From Template' (was 'Apply from template (optional)'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-003</t>
+          <t>FD-WO-005</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>C28426</t>
+          <t>C28428</t>
         </is>
       </c>
       <c r="C154" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28426</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28428</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -7041,12 +7089,12 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Verify the live preview shows a whole-work-order percentage discount before you save</t>
+          <t>Verify the Add button stays disabled until Name, Type, Calculation Type and an Amount above 0 are all filled in</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -7056,24 +7104,24 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>dialog live preview re-driven ($5 flat -&gt; '+$5.00 / New work-order subtotal $187.76'); pct preview math not re-driven, API pct resolution re-proven (10%-&gt;17.08) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calc type corrected from generic 'Percentage' to the real whole-WO option '% of Subtotal'. Exact preview row labels not re-captured this pass (behavior verified 2026-07-10). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>CONFIRMED AGAIN: 'Add Fee' button ENABLED on an empty form (disabled-on-empty=false) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION re-confirmed live 2026-07-13: the 'Add Fee' button is ENABLED on an empty form (validation happens on submit, not by disabling) — BUG-FD-4. Expected kept as the intended behavior; tester will see the button enabled. | STAGING VIU 2026-07-20 staging LIVE VIU: BUG-FD-4 FIXED on staging: Add Fee button is DISABLED on an empty form (was enabled on qb). Live-observed (dev-wo-emptyform, disabled=true). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-004</t>
+          <t>FD-WO-006</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>C28427</t>
+          <t>C28429</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28427</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28429</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -7083,12 +7131,12 @@
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>Verify 'Apply From Template' fills the dialog with a template's values</t>
+          <t>Verify Max Amount caps a percentage fee (20% on a $100 base with Max Amount $15 → +$15.00)</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -7098,24 +7146,24 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>not re-driven today (Apply-From-Template combobox present in dialog); templateId add path re-proven via API (FD-STACK-003) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Dropdown label is exactly 'Apply From Template' (was 'Apply from template (optional)'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>20% of 170.76 (=34.15) capped at Max 15 -&gt; resolved exactly 15 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). The '$ Max Amount (Optional)' field appears only after a percentage method is chosen (confirmed live). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-005</t>
+          <t>FD-WO-007</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>C28428</t>
+          <t>C28430</t>
         </is>
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28428</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28430</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -7125,12 +7173,12 @@
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>Verify the Add button stays disabled until Name, Type, Calculation Type and an Amount above 0 are all filled in</t>
+          <t>Verify the confirm button label follows the Type (Add Fee vs Add Discount)</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -7140,24 +7188,24 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED AGAIN: 'Add Fee' button ENABLED on an empty form (disabled-on-empty=false) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION re-confirmed live 2026-07-13: the 'Add Fee' button is ENABLED on an empty form (validation happens on submit, not by disabling) — BUG-FD-4. Expected kept as the intended behavior; tester will see the button enabled. | STAGING VIU 2026-07-20 staging LIVE VIU: BUG-FD-4 FIXED on staging: Add Fee button is DISABLED on an empty form (was enabled on qb). Live-observed (dev-wo-emptyform, disabled=true). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>confirm label 'Add Fee' observed; Type-flip re-observed in batch-1 (not re-driven) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-006</t>
+          <t>FD-WO-008</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>C28429</t>
+          <t>C28431</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28429</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28431</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -7167,7 +7215,7 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Verify Max Amount caps a percentage fee (20% on a $100 base with Max Amount $15 → +$15.00)</t>
+          <t>Verify an empty Name blocks saving a whole-work-order fee/discount</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -7182,24 +7230,24 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>20% of 170.76 (=34.15) capped at Max 15 -&gt; resolved exactly 15 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). The '$ Max Amount (Optional)' field appears only after a percentage method is chosen (confirmed live). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>UI BLOCKS empty name (inline 'Name' required, dialog stays open, nothing saved). NOTE NEW FDBUG-16: the RAW API now ACCEPTS an empty-name adjustment (201; was 400 in batch-3) — BE validation regression, FE still guards | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). (Note: the raw back-end will accept an empty name — FDBUG-16 — but the on-screen dialog blocks it, which is what a manual tester sees.) | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-007</t>
+          <t>FD-WO-009</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>C28430</t>
+          <t>C28432</t>
         </is>
       </c>
       <c r="C158" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28430</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28432</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -7209,7 +7257,7 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Verify the confirm button label follows the Type (Add Fee vs Add Discount)</t>
+          <t>Verify an empty or zero amount blocks saving a whole-work-order fee/discount</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -7224,24 +7272,24 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>confirm label 'Add Fee' observed; Type-flip re-observed in batch-1 (not re-driven) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>amount 0 -&gt; 400 at API; UI validates on submit | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-008</t>
+          <t>FD-WO-010</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>C28431</t>
+          <t>C28433</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28431</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28433</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -7251,7 +7299,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Verify an empty Name blocks saving a whole-work-order fee/discount</t>
+          <t>Verify a percentage discount over 100% is rejected while a percentage fee has no upper limit</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -7266,24 +7314,24 @@
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>UI BLOCKS empty name (inline 'Name' required, dialog stays open, nothing saved). NOTE NEW FDBUG-16: the RAW API now ACCEPTS an empty-name adjustment (201; was 400 in batch-3) — BE validation regression, FE still guards | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). (Note: the raw back-end will accept an empty name — FDBUG-16 — but the on-screen dialog blocks it, which is what a manual tester sees.) | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>discount 150% -&gt; 400 'A percentage discount cannot exceed 100%.'; fee 150% -&gt; 201 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-009</t>
+          <t>FD-WO-011</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>C28432</t>
+          <t>C28434</t>
         </is>
       </c>
       <c r="C160" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28432</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28434</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7293,12 +7341,12 @@
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Verify an empty or zero amount blocks saving a whole-work-order fee/discount</t>
+          <t>Verify a whole-work-order percentage method uses the correct base (% of Subtotal example)</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -7308,24 +7356,24 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>amount 0 -&gt; 400 at API; UI validates on submit | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>pct_subtotal resolves on the WO subtotal EXCLUDING whole-WO adjustments (10% of 182.76-sub -&gt; 17.08 = 10% of 170.76 line total) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calculation Type options confirmed live (exactly the 4 listed; no '% of Grand Total'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-010</t>
+          <t>FD-WO-012</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>C28433</t>
+          <t>C28435</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28433</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28435</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7335,12 +7383,12 @@
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Verify a percentage discount over 100% is rejected while a percentage fee has no upper limit</t>
+          <t>Verify Add Work Order Fee / Discount is hidden and blocked on an Invoiced or Paid work order</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -7350,24 +7398,24 @@
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>discount 150% -&gt; 400 'A percentage discount cannot exceed 100%.'; fee 150% -&gt; 201 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>add on Invoiced WO -&gt; 409 'Adjustments cannot be changed on an invoiced or paid work order.'; edit also 409 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-011</t>
+          <t>FD-WO-014</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>C28434</t>
+          <t>C28437</t>
         </is>
       </c>
       <c r="C162" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28434</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28437</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -7377,12 +7425,12 @@
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Verify a whole-work-order percentage method uses the correct base (% of Subtotal example)</t>
+          <t>Verify the preview shows the empty-amount prompt before an amount is entered</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -7392,24 +7440,24 @@
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>pct_subtotal resolves on the WO subtotal EXCLUDING whole-WO adjustments (10% of 182.76-sub -&gt; 17.08 = 10% of 170.76 line total) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calculation Type options confirmed live (exactly the 4 listed; no '% of Grand Total'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>'Enter an amount to see the impact.' prompt present in the re-driven dialog | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Exact prompt text 'Enter an amount to see the impact.' confirmed live (shot wo-03). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-012</t>
+          <t>FD-WO-015</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>C28435</t>
+          <t>C28438</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28435</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28438</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -7419,12 +7467,12 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Verify Add Work Order Fee / Discount is hidden and blocked on an Invoiced or Paid work order</t>
+          <t>Verify the preview amount is signed for a fee (+) vs a discount (−)</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -7434,24 +7482,24 @@
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>add on Invoiced WO -&gt; 409 'Adjustments cannot be changed on an invoiced or paid work order.'; edit also 409 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>preview row '+$5.00' with new-subtotal line re-observed; color/sign convention from batch-1 (not re-checked) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Kept to sign only; the exact fee/discount colours were not re-captured this pass. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-014</t>
+          <t>FD-WO-016</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>C28437</t>
+          <t>C29441</t>
         </is>
       </c>
       <c r="C164" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28437</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29441</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -7461,7 +7509,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Verify the preview shows the empty-amount prompt before an amount is entered</t>
+          <t>Verify the Add/Edit fee-or-discount dialog shows the tax-jurisdiction note below the Taxable Yes/No dropdown</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -7476,34 +7524,34 @@
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>'Enter an amount to see the impact.' prompt present in the re-driven dialog | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Exact prompt text 'Enter an amount to see the impact.' confirmed live (shot wo-03). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-015</t>
+          <t>FD-WO-018</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>C28438</t>
+          <t>C30619</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28438</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30619</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Verify the preview amount is signed for a fee (+) vs a discount (−)</t>
+          <t>Verify the work-order part row three-dot menu item reads 'Add Part Fee / Discount'</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -7518,34 +7566,34 @@
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>preview row '+$5.00' with new-subtotal line re-observed; color/sign convention from batch-1 (not re-checked) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Kept to sign only; the exact fee/discount colours were not re-captured this pass. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
+          <t>. | VIU 2026-07-22 LIVE: part-row ⋮ menu = 'Move', 'Add Part Fee / Discount' (label correct; opens part fee/discount dialog). 'Return' state-gated — the seeded part was 'Auth To Order' (not received) so Return was not offered; Return appears only for returnable parts. Ev: wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-016</t>
+          <t>FD-WO-021</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>C29441</t>
+          <t>C30620</t>
         </is>
       </c>
       <c r="C166" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29441</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30620</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Sidebar 'Work Order Fee / Discount' card</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>Verify the Add/Edit fee-or-discount dialog shows the tax-jurisdiction note below the Taxable Yes/No dropdown</t>
+          <t>Verify the Work Order Fees &amp; Discounts card shows the disclaimer 'Applies to the whole work order, after all other fees &amp; discounts.'</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -7560,30 +7608,34 @@
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
+          <t>s a mockup. QA passed on staging 2026-07-22 (✅). | VIU 2026-07-22 LIVE: Work Order Fees &amp; Discounts card shows disclaimer exactly 'Applies to the whole work order, after all other fees &amp; discounts.' below the adjustment list. Ev: wo/FD-FIN-004-FD-WO-021-card-financialinfo.png, wo/lines-bodytext.txt.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-018</t>
+          <t>FD-WO-025</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr"/>
+          <t>C30621</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30621</t>
+        </is>
+      </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>Verify the work-order part row three-dot menu item reads 'Add Part Fee / Discount'</t>
+          <t>Verify the work order toolbar three-dot menu item reads 'Add Work Order Fee / Discount'</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
@@ -7598,30 +7650,34 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>. | VIU 2026-07-22 LIVE: part-row ⋮ menu = 'Move', 'Add Part Fee / Discount' (label correct; opens part fee/discount dialog). 'Return' state-gated — the seeded part was 'Auth To Order' (not received) so Return was not offered; Return appears only for returnable parts. Ev: wo/FD-WO-018-part-menu.png.</t>
+          <t>6-07-22 LIVE: toolbar ⋯ menu label 'Add Work Order Fee / Discount' correct; opens whole-WO fee/discount dialog. WORDING CORRECTED — observed order is 'Audit Log' -&gt; 'Timesheets (N)' -&gt; 'Add Work Order Fee / Discount' -&gt; 'Delete Work Order' (Add is 3rd, NOT at top). Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-021</t>
+          <t>FD-WO-028</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr"/>
+          <t>C30622</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30622</t>
+        </is>
+      </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Sidebar 'Work Order Fee / Discount' card</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Verify the Work Order Fees &amp; Discounts card shows the disclaimer 'Applies to the whole work order, after all other fees &amp; discounts.'</t>
+          <t>Verify the tax-jurisdiction note and the 'Pass convenience fee to customer' banner still appear after the fee/discount UI updates</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -7635,82 +7691,6 @@
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
-        <is>
-          <t>s a mockup. QA passed on staging 2026-07-22 (✅). | VIU 2026-07-22 LIVE: Work Order Fees &amp; Discounts card shows disclaimer exactly 'Applies to the whole work order, after all other fees &amp; discounts.' below the adjustment list. Ev: wo/FD-FIN-004-FD-WO-021-card-financialinfo.png, wo/lines-bodytext.txt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>FD-WO-025</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="inlineStr"/>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
-        </is>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>Verify the work order toolbar three-dot menu item reads 'Add Work Order Fee / Discount'</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G169" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H169" s="2" t="inlineStr">
-        <is>
-          <t>6-07-22 LIVE: toolbar ⋯ menu label 'Add Work Order Fee / Discount' correct; opens whole-WO fee/discount dialog. WORDING CORRECTED — observed order is 'Audit Log' -&gt; 'Timesheets (N)' -&gt; 'Add Work Order Fee / Discount' -&gt; 'Delete Work Order' (Add is 3rd, NOT at top). Ev: wo/FD-WO-025-toolbar-menu.png.</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>FD-WO-028</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr"/>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
-        </is>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t>Verify the tax-jurisdiction note and the 'Pass convenience fee to customer' banner still appear after the fee/discount UI updates</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G170" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H170" s="2" t="inlineStr">
         <is>
           <t>&amp; Discounts Settings page (Settings -&gt; Service -&gt; Fees &amp; Discounts / adjustment-templates) — it is NOT rendered inside the WO fee/discount dialogs. Ev: wo/labor-dialog-text.txt, wo/part-dialog-text.txt, wo/wo-dialog-text.txt, wo/FD-WO-028-settings-convenience-banner.png, wo/settings-fd-bodytext.txt.</t>
         </is>
@@ -7733,144 +7713,158 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7882,7 +7876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8108,32 +8102,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>FD-LABOR-003</t>
+          <t>FD-PERM-002</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>C28441</t>
+          <t>C28586</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28441</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28586</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Labor-line Fee/Discount</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Verify the labor fee/discount add entry point is a three-dot menu to the left of the first technician (or 'Unassigned')</t>
+          <t>Verify whole-work-order add/edit/remove requires Work Orders: Create and Edit</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -8143,34 +8137,34 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>not re-driven (cosmetic hover menu); line-level add path re-proven via API | WORDING+VIU 2026-07-13: Per-line ⋮ on hover; carried. Labor-line ⋮ menu not re-captured this run; confirmed by symmetry with the part-line flow (⋮ = 'Move' / 'Add Fee/Discount', dialog 'Applying to: &lt;name&gt;') + prior 2026-07-10 VIU. | SV-8479/8480 deconfliction 2026-07-22: rescoped from the old per-line-row ⋮ model to the new ⋮-left-of-technician entry point + 'Add Labor Fee / Discount' (item 1). RETIRE-CANDIDATE: now overlaps kept new case FD-WO-017 (item-1 placement acceptance) — flag for user ruling. | VIU 2026-07-22 LIVE: DEVIATION — three-dot (⋮) renders to the RIGHT of 'Unassigned' (⋮ x=502 vs Unassigned right-edge x=497), but EXP/spec requires LEFT (same defect as FD-WO-017 item-#1 re-open). Label 'Add Labor Fee / Discount' correct. Ev: wo/FD-WO-017-labor-row-menu-RIGHT.png.</t>
+          <t>BUG-FD-3 stands on batch evidence; NOT re-testable today — Technician role drifted on the shared env (now HAS workOrdersCreateAndEdit, so its 201 is legitimate); enforcement-depth question unchanged (dev decision) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-3): the whole-work-order add/edit/remove hide is front-end only — the back-end does not block the write. NOT re-testable this run: Technician drifted to HAVE Work Orders: Create &amp; Edit, and only admin/tech can log in.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>FD-PERM-002</t>
+          <t>FD-PROC-008</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>C28586</t>
+          <t>C28526</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28586</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28526</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Permissions (Story 13)</t>
+          <t>Processing Fee — WO behavior</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Verify whole-work-order add/edit/remove requires Work Orders: Create and Edit</t>
+          <t>Verify a Processing Fee on a work order can be removed but not edited</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8185,34 +8179,34 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>BUG-FD-3 stands on batch evidence; NOT re-testable today — Technician role drifted on the shared env (now HAS workOrdersCreateAndEdit, so its 201 is legitimate); enforcement-depth question unchanged (dev decision) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-3): the whole-work-order add/edit/remove hide is front-end only — the back-end does not block the write. NOT re-testable this run: Technician drifted to HAVE Work Orders: Create &amp; Edit, and only admin/tech can log in.</t>
+          <t>BE re-proven: pfee change -&gt; 409 'cannot be edited through this endpoint', remove -&gt; 204; card still offers Edit per batch-1 (S8-N5 UI drift) | WORDING+VIU 2026-07-13: DEVIATION carried: the ⋮ menu still shows 'Edit' for a Processing Fee but it is inert (cannot edit a pfee on the WO); 'Remove' works. Build labels ('Remove Fee / Discount' confirm). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. The SV-8456 UI-correction wording + Settings-&gt;Service permission pivot were re-confirmed live on the current staging build (Service-user sees+manages F&amp;D; Finance-only user no F&amp;D nav, direct route bounces to /workorders; Tech restored to Technician 50bf6a0d + verified; ZZAUTOTEST roles deleted). This case retains its prior VIU-Deviation for its OWN (non-SV-8456) reason — that specific behavior was NOT re-driven this pass. Ev build/fees-discounts/viu-sv8456-2026-07-22/.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-008</t>
+          <t>FD-PROC-009</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>C28526</t>
+          <t>C28527</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28526</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28527</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — WO behavior</t>
+          <t>Processing Fee — calculation</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Verify a Processing Fee on a work order can be removed but not edited</t>
+          <t>Verify a % of Grand Total Processing Fee works out last on the tax-included grand total (3% of $324 → +$9.72)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -8227,39 +8221,39 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>BE re-proven: pfee change -&gt; 409 'cannot be edited through this endpoint', remove -&gt; 204; card still offers Edit per batch-1 (S8-N5 UI drift) | WORDING+VIU 2026-07-13: DEVIATION carried: the ⋮ menu still shows 'Edit' for a Processing Fee but it is inert (cannot edit a pfee on the WO); 'Remove' works. Build labels ('Remove Fee / Discount' confirm). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. The SV-8456 UI-correction wording + Settings-&gt;Service permission pivot were re-confirmed live on the current staging build (Service-user sees+manages F&amp;D; Finance-only user no F&amp;D nav, direct route bounces to /workorders; Tech restored to Technician 50bf6a0d + verified; ZZAUTOTEST roles deleted). This case retains its prior VIU-Deviation for its OWN (non-SV-8456) reason — that specific behavior was NOT re-driven this pass. Ev build/fees-discounts/viu-sv8456-2026-07-22/.</t>
+          <t>FDBUG-2 CONFIRMED AGAIN with a clean discriminator: on a WO whose ONLY money is a whole-WO $20 taxable fee, 3% pfee resolved 0.63 (=3% of 21.00 incl the whole-WO fee + its tax); spec base must EXCLUDE whole-WO adjustments -&gt; expected 0.00 | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-2): the Processing Fee base wrongly includes whole-WO fees/discounts + their tax (should exclude them).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>FD-PROC-009</t>
+          <t>FD-STATS-002</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>C28527</t>
+          <t>C28460</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28527</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28460</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — calculation</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Verify a % of Grand Total Processing Fee works out last on the tax-included grand total (3% of $324 → +$9.72)</t>
+          <t>Verify each Stats fee/discount row names its target</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -8269,24 +8263,24 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-2 CONFIRMED AGAIN with a clean discriminator: on a WO whose ONLY money is a whole-WO $20 taxable fee, 3% pfee resolved 0.63 (=3% of 21.00 incl the whole-WO fee + its tax); spec base must EXCLUDE whole-WO adjustments -&gt; expected 0.00 | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-2): the Processing Fee base wrongly includes whole-WO fees/discounts + their tax (should exclude them).</t>
+          <t>per-row scope hyperlink impossible while the layout is aggregate (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: Stats F&amp;D rows show the name only — no scope hyperlink to the target. Confirmed live (rows read plain names, shot fin-01).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-002</t>
+          <t>FD-STATS-004</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>C28460</t>
+          <t>C28462</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28460</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28462</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -8296,7 +8290,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Verify each Stats fee/discount row names its target</t>
+          <t>Verify the Stats fees/discounts are listed in the order they were created (oldest first)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -8311,39 +8305,39 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>per-row scope hyperlink impossible while the layout is aggregate (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: Stats F&amp;D rows show the name only — no scope hyperlink to the target. Confirmed live (rows read plain names, shot fin-01).</t>
+          <t>creation-order rows blocked by aggregate layout (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: creation-order ruling pending (BUG-FD-2 group). Labels cleaned.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>FD-STATS-004</t>
+          <t>FD-TMPL-010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>C28462</t>
+          <t>C28511</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28462</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28511</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Statistics tab</t>
+          <t>Template admin — scoping</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Verify the Stats fees/discounts are listed in the order they were created (oldest first)</t>
+          <t>Verify template scoping — labour-method templates only show in labour pickers, parts-method only in parts pickers</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -8353,39 +8347,39 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>creation-order rows blocked by aggregate layout (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: creation-order ruling pending (BUG-FD-2 group). Labels cleaned.</t>
+          <t>FDBUG-13 (line-scope Add dialog has no template picker) per batch-1/4; not re-driven today | WORDING+VIU 2026-07-13: DEVIATION carried: template scoping in the line 'Apply From Template' picker + the compatibility hint not re-captured this run (needs the line-level picker). Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: mixed label sweep: labor step -&gt; 'Add Labor Fee / Discount', part step -&gt; 'Add Part Fee / Discount' (behavior unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav labels 'Add Labor Fee / Discount' (step 1) and 'Add Part Fee / Discount' (step 3) both confirmed present; case status unchanged (existing Deviation for its own reason). Ev: wo/FD-WO-017-labor-menu-open.png, wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>FD-TMPL-010</t>
+          <t>FD-WO-013</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>C28511</t>
+          <t>C28436</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28511</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/28436</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Template admin — scoping</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Verify template scoping — labour-method templates only show in labour pickers, parts-method only in parts pickers</t>
+          <t>Verify the whole-work-order 'Add Work Order Fee / Discount' option is hidden without Work Orders: Create &amp; Edit</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -8395,39 +8389,39 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>FDBUG-13 (line-scope Add dialog has no template picker) per batch-1/4; not re-driven today | WORDING+VIU 2026-07-13: DEVIATION carried: template scoping in the line 'Apply From Template' picker + the compatibility hint not re-captured this run (needs the line-level picker). Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: mixed label sweep: labor step -&gt; 'Add Labor Fee / Discount', part step -&gt; 'Add Part Fee / Discount' (behavior unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav labels 'Add Labor Fee / Discount' (step 1) and 'Add Part Fee / Discount' (step 3) both confirmed present; case status unchanged (existing Deviation for its own reason). Ev: wo/FD-WO-017-labor-menu-open.png, wo/FD-WO-018-part-menu.png.</t>
+          <t>BUG-FD-3 stands on prior evidence; NOT re-testable today: the shared-env Technician role was CHANGED (now includes workOrdersCreateAndEdit+workOrdersDelete, 8 perms vs matrix 6) so tech's 201 is now legitimate; no login lacking the perm exists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION (BUG-FD-3: the hide is front-end only; the back-end does not block the write). NOT re-testable this run — the Technician role has drifted on the shared qb env; re-derive the roles matrix before re-checking. | SV-8479/8480 deconfliction 2026-07-22: label updated 'Add Fee/Discount' -&gt; 'Add Work Order Fee / Discount' (item 10); permission behavior unchanged. | VIU 2026-07-22 LIVE: toolbar label 'Add Work Order Fee / Discount' confirmed present (admin); permission-negative status unchanged — role-negative not re-driven this UI batch.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>FD-WO-013</t>
+          <t>FD-WO-017</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>C28436</t>
+          <t>C30618</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/28436</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30618</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Verify the whole-work-order 'Add Work Order Fee / Discount' option is hidden without Work Orders: Create &amp; Edit</t>
+          <t>Verify the labor fee/discount entry point is a three-dot menu to the LEFT of the first technician (or 'Unassigned') and reads 'Add Labor Fee / Discount'</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -8436,44 +8430,6 @@
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>BUG-FD-3 stands on prior evidence; NOT re-testable today: the shared-env Technician role was CHANGED (now includes workOrdersCreateAndEdit+workOrdersDelete, 8 perms vs matrix 6) so tech's 201 is now legitimate; no login lacking the perm exists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION (BUG-FD-3: the hide is front-end only; the back-end does not block the write). NOT re-testable this run — the Technician role has drifted on the shared qb env; re-derive the roles matrix before re-checking. | SV-8479/8480 deconfliction 2026-07-22: label updated 'Add Fee/Discount' -&gt; 'Add Work Order Fee / Discount' (item 10); permission behavior unchanged. | VIU 2026-07-22 LIVE: toolbar label 'Add Work Order Fee / Discount' confirmed present (admin); permission-negative status unchanged — role-negative not re-driven this UI batch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>FD-WO-017</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Work Order — Labor-line Fee/Discount</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Verify the labor fee/discount entry point is a three-dot menu to the LEFT of the first technician (or 'Unassigned') and reads 'Add Labor Fee / Discount'</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Deviation</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>me row y=282); spec requires LEFT. Label 'Add Labor Fee / Discount' is correct and opens the labor fee/discount dialog. Menu contained only 'Add Labor Fee / Discount' (no separate 'Edit labor' item observed). Ev: wo/FD-WO-017-labor-row-menu-RIGHT.png, wo/FD-WO-017-labor-menu-open.png, obs2 geometry.</t>
         </is>
@@ -8675,10 +8631,14 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>(pending-create)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
+          <t>C30634</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30634</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Calculation contract</t>
@@ -9506,25 +9466,26 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fees & Discounts: add plain 'What needs to be done' beside every DEVIATION/Blocked row in the deliverables
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/FeesDiscounts_FreshVIU_2026-07-10.xlsx
+++ b/build/fees-discounts/FeesDiscounts_FreshVIU_2026-07-10.xlsx
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:I168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,8 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -679,6 +680,11 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Fresh Evidence / Note</t>
         </is>
       </c>
@@ -721,6 +727,11 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>10% pct_subtotal -&gt; 17.08 = exactly 10% of the 170.76 base; sub delta matches | WORDING+VIU 2026-07-13: Build labels; carry arithmetic VIU. Resolution engine re-confirmed live 2026-07-13 via API (flat $25→+$25.00; 20% capped at $15→+$15.00; 150% discount rejected 'A percentage discount cannot exceed 100%'). | SV-8479/8480 deconfliction 2026-07-22: rate rendering reworded from 'rate badge' to plain text (item 4); calc math unchanged. | VIU 2026-07-22 LIVE: base×percent calc confirmed (20% of $509.90 labor = +$101.98; plain text, no badge). WORDING CORRECTED '+10%' -&gt; '10%' — inline percentage FEE renders bare with no leading '+' (matches live build + batch-1 FD-CALC-018/019 fix). Ev: wo/inline-expanded-text.txt.</t>
         </is>
       </c>
@@ -763,6 +774,11 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>0.25% of 170.76 = 0.4269 -&gt; 0.43 (rounds up); half-cent-up rule from batch-1 (0.1%x265-&gt;0.27) stands | WORDING+VIU 2026-07-13: Build labels; carry rounding VIU. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -805,6 +821,11 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>flat 7.77 -&gt; resolved 7.77 exactly (whole-WO); labor-line flat 9.99 exact | WORDING+VIU 2026-07-13: Build labels; flat resolve confirmed live 2026-07-13 ($25→+$25.00). Resolution engine re-confirmed live 2026-07-13 via API (flat $25→+$25.00; 20% capped at $15→+$15.00; 150% discount rejected 'A percentage discount cannot exceed 100%'). | SV-8479/8480 deconfliction 2026-07-22: mixed label sweep: step 1 whole-WO -&gt; 'Add Work Order Fee / Discount', step 2 labor line -&gt; 'Add Labor Fee / Discount' (behavior unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav labels 'Add Work Order Fee / Discount' (step 1) and 'Add Labor Fee / Discount' (step 2) both confirmed present; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png, wo/FD-WO-017-labor-menu-open.png.</t>
         </is>
       </c>
@@ -847,6 +868,11 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>per-item: $2.00 x qty4 -&gt; $8.00 (part line) | WORDING+VIU 2026-07-13: Build labels; per-item VIU carried. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Part Fee / Discount' / 'New Part Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Part Fee / Discount' confirmed present in the part row ⋮ menu; case behavior unchanged. Ev: wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
@@ -889,6 +915,11 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
           <t>discount pct &gt;100 -&gt; 400; fee pct uncapped (150% -&gt; 201) | WORDING+VIU 2026-07-13: Exact back-end message confirmed live 2026-07-13: 'A percentage discount cannot exceed 100%.' Resolution engine re-confirmed live 2026-07-13 via API (flat $25→+$25.00; 20% capped at $15→+$15.00; 150% discount rejected 'A percentage discount cannot exceed 100%'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | SV-8479/8480 deconfliction 2026-07-22: 'at any scope' step reworded to the whole-WO entry label 'Add Work Order Fee / Discount' (validation is scope-independent). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -931,6 +962,11 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-10 CONFIRMED AGAIN: pct 0.005% accepted (201) and silently coerced to 0.01 (resolved 0.02); flat 0.005 accepted -&gt; stored 0.01. Spec: below-minimum must be rejected | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-10 / PO Q3 pending): a percentage below the 0.01% minimum is silently rounded UP to 0.01% instead of being rejected. Build labels applied. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q3=A): PO ruled quietly rounding tiny percentages up to the 0.01% minimum is fine/expected ('fully anticipated and expected'). No longer a deviation; FDBUG-10 closed as accepted; jira draft TICKET 5 DROPPED. Expected reworded to expect the round-up-to-minimum coercion. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -973,6 +1009,11 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>Max cap clamps: 20% (34.15) with cap 15 -&gt; 15.00 | WORDING+VIU 2026-07-13: Max cap clamp confirmed live 2026-07-13 (20% → capped $15.00). Resolution engine re-confirmed live 2026-07-13 via API (flat $25→+$25.00; 20% capped at $15→+$15.00; 150% discount rejected 'A percentage discount cannot exceed 100%'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -1015,6 +1056,11 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-9 CONFIRMED AGAIN: maxCap 0 -&gt; resolved 34.15 (treated as NO cap; spec: $0 forces $0.00) | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-9 / PO Q2 pending): a Max Amount of 0 is treated as 'no cap' rather than capping at $0.00. Build labels applied. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount means 'no limit' (WAD, S2-R25: entered 0 = empty = no maximum; a true $0 cap only from legacy data per §5-R6). No longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -1057,6 +1103,11 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
           <t>10% of $0 parts -&gt; $0.00 | WORDING+VIU 2026-07-13: QB-skip half needs a human in QuickBooks (Blocked-Env); the on-screen $0.00 half is observable. Build labels applied. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1099,6 +1150,11 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
           <t>50% discount on $0 base -&gt; $0.00; base floored at 0 | WORDING+VIU 2026-07-13: Base-floor-at-$0 carried; build labels. Resolution engine re-confirmed live 2026-07-13 via API (flat $25→+$25.00; 20% capped at $15→+$15.00; 150% discount rejected 'A percentage discount cannot exceed 100%').</t>
         </is>
       </c>
@@ -1141,6 +1197,11 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>taxable $20 fee: GST 9.14-&gt;10.14 (+5% of 20); non-taxable leaves tax unchanged. GST-&gt;US-tax re-word caveat stands | WORDING+VIU 2026-07-13: Tax effect carried; build labels ('Taxable' toggle Yes/No). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1183,6 +1244,11 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
           <t>3-step order re-proven: whole-WO 10% resolved 17.08 alone -&gt; 19.08 after a $20 labor-line fee (+10% of the line-level effect); whole-WO adjs do not stack on each other (17.08 each) | WORDING+VIU 2026-07-13: 3-step order carried; build labels.</t>
         </is>
       </c>
@@ -1225,6 +1291,11 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
           <t>pfee base tax-inclusive on purpose (0.63 = 3% of 21.00 incl GST, not 0.60); maxCap rejected for pfee (400) | WORDING+VIU 2026-07-13: Processing-Fee base + no Max Amount carried; build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1267,6 +1338,11 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
           <t>non-taxable over-discount: sub floors 0.00, GST unchanged 9.14, total=tax, excessCredit 117.24 exact | WORDING+VIU 2026-07-13: In-app floor + credit half VIU'd 2026-07-10; the QuickBooks credit-memo half needs a human in QuickBooks. Build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1309,6 +1385,11 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>taxable over-discount: sub 0.00, GST 0, total 0.00, excess captured | WORDING+VIU 2026-07-13: Taxable-discount-to-$0 carried; build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1349,7 +1430,12 @@
           <t>VIU-Verified</t>
         </is>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I17" s="2">
         <f> $392.40 = 290 + labor fee ttt +20% ($58.00) + 40 + part fee test +11% ($4.40); NOT gross $330. Rows render PLAIN TEXT bare '20%'/'11%' (no plus sign, no colored badge; HTML span text-grey-7). Ev: 018-lines-collapsed-full.png, 018-lines-expanded-full.png, api-FD-CALC-018-024-total_cost-392.40.json.</f>
         <v/>
       </c>
@@ -1392,6 +1478,11 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
           <t>acted -&gt; collapsed line Total = $384.00 = 290 + 58 + 40 - 4.00 (fee adds, discount subtracts). Discount rate renders '-10%' (en-dash minus) plain text, resolved -$4.00; fee rate renders bare '20%'. Ev: 019-lines-collapsed-full.png, 019-lines-expanded-full.png, api-FD-CALC-019-total_cost-384.00.json.</t>
         </is>
       </c>
@@ -1434,6 +1525,11 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
           <t>tal (no change from the fix). | LIVE STAGING VIU 2026-07-22: VIU-VERIFIED. A ZZAUTOTEST line with no fees/discounts (Labor $290 + Parts $40) shows collapsed line Total = $330.00 = gross Labor + Parts only, no Fees/Discounts rows. Ev: 020-lines-nofee-line.png, api-baseline-nofees-total_cost-330.json.</t>
         </is>
       </c>
@@ -1476,6 +1572,11 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
           <t>0'; the document Line Total = $330.00 (gross Labor+Parts, fee NOT folded in); every fee/discount (incl. line-level ttt +$58.00 and pdisc ($4.00)) listed once in the Fees &amp; Discounts breakdown -&gt; no double-count. Confirms the fix is Lines-tab display-only; estimate unchanged. Ev: 021-finance-tab.png.</t>
         </is>
       </c>
@@ -1518,6 +1619,11 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
           <t>Invoice document (Finance tab toggle, INV-S3-25836): renders identically to the estimate — Labor gross $290.00, the line fee prints as its own row '↳ ttt (% of labor) $58.00', document Line Total = $330.00 (gross, fee not folded in), each fee listed once -&gt; no double-count. Ev: 022-invoice-view.png.</t>
         </is>
       </c>
@@ -1560,6 +1666,11 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
           <t>Stored line amounts unchanged (labour_rate 145, total_labour_cost 290, part sell_price 40); the fee/discount amounts live separately under line.adjustments[] and part_requests[].adjustments[] (resolvedAmount 58 / 4.40) — computed total is display-only. Ev: api-FD-CALC-018-024-total_cost-392.40.json.</t>
         </is>
       </c>
@@ -1602,6 +1713,11 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
           <t>tab label 'Fees &amp; Discounts (N)' re-observed (live count from defaults) | WORDING+VIU 2026-07-13: Tab 'Fees &amp; Discounts (N)' confirmed live (shot cust-01). Corrected the tab list to the real build tabs.</t>
         </is>
       </c>
@@ -1644,6 +1760,11 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
           <t>card header + exact caption re-observed ('These fees &amp; discounts auto-apply to every new work order for this customer…') | WORDING+VIU 2026-07-13: Card header/caption/button/columns confirmed EXACTLY live (shot cust-01). Corrected columns (no Auto-Apply column on the customer tab).</t>
         </is>
       </c>
@@ -1686,6 +1807,11 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
           <t>single-select add works (API 201, UI single picker) — PO Q6=A accepted; case text still needs the single-select re-wording (case-update) | WORDING+VIU 2026-07-13: Picker confirmed live: 'Add Fee/Discount' dialog with a single 'Fee / Discount Templates' dropdown + Save (shot cust-02). Add lifecycle confirmed via API (201). Toast text carried.</t>
         </is>
       </c>
@@ -1728,6 +1854,11 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
           <t>one-at-a-time picker accepted per PO Q6=A; case-update pending | WORDING+VIU 2026-07-13: Single-select (one dropdown, not checkboxes) confirmed live; multi-add is one-at-a-time. Add lifecycle via API.</t>
         </is>
       </c>
@@ -1770,6 +1901,11 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
           <t>remove = direct trash, no toast (batch-1); API remove -&gt; 204 re-proven; case-update pending | WORDING+VIU 2026-07-13: Remove confirmed live via API (204, no confirm step). Toast text carried.</t>
         </is>
       </c>
@@ -1812,6 +1948,11 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
           <t>empty-state card re-observed on a 0-default customer | WORDING+VIU 2026-07-13: Empty-state text confirmed EXACTLY live: "No fees or discounts yet. Use 'Add Fee/Discount' to add one." (shot cust-01).</t>
         </is>
       </c>
@@ -1854,6 +1995,11 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
           <t>customer default lands on every NEW WO as an independent copy (appliedBy=customer_default) | WORDING+VIU 2026-07-13: Defaults→new-WO behavior carried (verified 2026-07-10); build labels ('WO Fees &amp; Discounts' card). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1896,6 +2042,11 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
           <t>pct default copied as percent (amount=7, calc=pct_subtotal), re-resolves per WO | WORDING+VIU 2026-07-13: Percentage default re-resolves per WO; carried.</t>
         </is>
       </c>
@@ -1938,6 +2089,11 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
           <t>removing the default link leaves the existing WO's adjustment intact | WORDING+VIU 2026-07-13: Remove-default-does-not-touch-existing-WOs carried; remove lifecycle confirmed via API (204). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -1980,6 +2136,11 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
           <t>deleting a linked template (204) cascades the default link away | WORDING+VIU 2026-07-13: Corrected nav to Administration → Finance; behavior carried. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -2022,6 +2183,11 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
           <t>prior (customer delete removes links) stands; today's re-probe was blocked by an orphan test contact, not by the feature | WORDING+VIU 2026-07-13: Corrected nav; behavior carried. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -2064,6 +2230,11 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
           <t>NEW TODAY — FDBUG-12 APPEARS FIXED: an API-created customer NOW inherits the auto-apply location template as a default (initial defaults list had the auto template pre-seeded) | WORDING+VIU 2026-07-13: New-customer seeding of auto-apply defaults confirmed working (FDBUG-12 fixed 2026-07-10); carried.</t>
         </is>
       </c>
@@ -2106,6 +2277,11 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
           <t>tech -&gt; defaults GET/POST 403 (BE-enforced); per-role visibility via roles-matrix (role-drift caveat) | WORDING+VIU 2026-07-13: Customer-defaults GET/POST are back-end gated (Tech → 403), established batch-2. NOTE: re-check the Tech negative after the roles matrix is re-derived (Technician drifted on shared qb).</t>
         </is>
       </c>
@@ -2148,6 +2324,11 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
           <t>bad-template add 400 / bad-customer load 404 / bad remove 404 | WORDING+VIU 2026-07-13: API negative — standard error notification; carried. Lives in an API-titled section (rule 4).</t>
         </is>
       </c>
@@ -2190,6 +2371,11 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
           <t>estimate rendered via the invoice template (header 'Invoice', shared layout), Adjustments block present | WORDING+VIU 2026-07-13: Estimate rendering confirmed live (est-15960.html); invoice uses the same layout (carried).</t>
         </is>
       </c>
@@ -2232,6 +2418,11 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
           <t>labor-line pct renders '↳ ZZAUTOTEST LabPct (% of labor) $0.00' (phrase present) | WORDING+VIU 2026-07-13: Amount format + '(% of ...)' phrase confirmed live; per-line ↳ rendering carried from prior VIU. Tax shown as 'GST (5%)' on this env.</t>
         </is>
       </c>
@@ -2274,6 +2465,11 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
           <t>part pct 'ZZAUTOTEST PartPct (% of parts) ($17.08)'; part flat 'ZZAUTOTEST PartFlat $8.00' (no phrase) | WORDING+VIU 2026-07-13: '(% of parts)' phrase pattern confirmed (build shows '(% of &lt;method&gt;)'); Flat Amount shows no phrase (confirmed).</t>
         </is>
       </c>
@@ -2316,6 +2512,11 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
           <t>fee '$10.00' vs discount accounting '($5.00)' formats confirmed | WORDING+VIU 2026-07-13: CONFIRMED live: fee '$X.XX', discount '($X.XX)' in round brackets (est-15960.html: 'Flat fee $21,474,836.47' vs 'Falt discount ($21,474,836.47)').</t>
         </is>
       </c>
@@ -2358,6 +2559,11 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
           <t>bottom Adjustments block lists whole-WO adjustments in creation order (Flat fee -&gt; WFee -&gt; WDisc) | WORDING+VIU 2026-07-13: CONFIRMED live: bottom 'Adjustments' block lists items in creation order; percentage items show '(% of subtotal)'. NOTE: this build lists line-level items in the same block too.</t>
         </is>
       </c>
@@ -2400,6 +2606,11 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
           <t>3 same-name+type line fees grouped as '(×3) $24.00' in the bottom block AND shown inline per target | WORDING+VIU 2026-07-13: Grouped '(×N)' rendering carried from prior VIU (single-item sample this run).</t>
         </is>
       </c>
@@ -2442,6 +2653,11 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
           <t>'(% of grand total)' phrase per batch evidence; pfee not seedable onto a money-bearing WO today (line-create 500 blocks a fresh WO with lines) | WORDING+VIU 2026-07-13: '% of grand total' phrase carried (no live pfee on the sample WO).</t>
         </is>
       </c>
@@ -2484,6 +2700,11 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
           <t>Shop Supplies section HIDDEN on the estimate when total is $0.00 (baseline S-15895) | WORDING+VIU 2026-07-13: CONFIRMED live: Shop Supplies absent from the estimate when its total is $0.00 (est-15960.html has no Shop Supplies section).</t>
         </is>
       </c>
@@ -2526,6 +2747,11 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
           <t>prior (&gt;0 reappears) stands; today's probe inert — parts-only WO computes shop supplies on labor, stayed $0 | WORDING+VIU 2026-07-13: Shop-Supplies-reappears carried from prior VIU.</t>
         </is>
       </c>
@@ -2568,6 +2794,11 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
           <t>prior batch-4 declined-line $0-render stands; decline flip blocked today (staged-parts lock) | WORDING+VIU 2026-07-13: Declined-line $0-but-shows carried.</t>
         </is>
       </c>
@@ -2610,6 +2841,11 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-1 NOT REPRODUCED (3rd consecutive pass): document bottom block reads Subtotal $202.68 / GST (5%) $9.14 / Total $211.82 = EXACTLY the API values incl. all adjustments; block sits before Subtotal. Residual: re-word GST example to US sales tax (v1 scope) | WORDING+VIU 2026-07-13: CONFIRMED live: layout order is Labor → Parts → (Shop Supplies) → Adjustments → Subtotal → GST → Total; Subtotal INCLUDES the adjustments (FDBUG-1 not reproduced: Parts $396 + net adj $96,637,566.11 = Subtotal $96,637,962.11).</t>
         </is>
       </c>
@@ -2652,6 +2888,11 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
           <t>change accepts name/amount/maxCap/taxable only; kind/calc unchanged after edit (200) | WORDING+VIU 2026-07-13: Edit dialog confirmed live (shot edit-01): title 'Edit Fee / Discount'; Type + Calculation Type greyed/locked; Name/Amount/Taxable editable; opened from sidebar 'WO Fees &amp; Discounts' ⋮ &gt; Edit. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -2694,6 +2935,11 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
           <t>edit 10%-&gt;20% re-resolved 34.15 against current totals; GST-&gt;US-tax re-word caveat stands | WORDING+VIU 2026-07-13: Confirmed live: no 'Apply From Template' picker in Edit; confirm button reads 'Save'; preview re-resolves against current totals (shot edit-01). | V1_3 (2026-07-17): Δ2 — Story 10 renamed 'history log' -&gt; 'audit log' (terminology only; gates/behavior/status unchanged). Notes-only touch: the reader-facing text of this case already uses the exact build labels ('Audit Log' ⋮ menu / 'Work Order Log' page) and carries no generic history-log prose. The internal `area`/section name is left as-is (TestRail section rename not authorized).</t>
         </is>
       </c>
@@ -2736,6 +2982,11 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
           <t>invalid edit (empty name + amount 0) -&gt; 400, original left intact | WORDING+VIU 2026-07-13: Behavior (dialog stays open on save error + error message) carried from prior VIU — not force-failed this run.</t>
         </is>
       </c>
@@ -2778,6 +3029,11 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
           <t>'Fees &amp; Discounts (5)' collapsed row seen in Financial Info with net total | WORDING+VIU 2026-07-13: Financial Info card confirmed live: 'Fees &amp; Discounts (N)' row shows net in grey (shot fin-03). | SV-8479/8480 deconfliction 2026-07-22: line position pinned directly above Subtotal (was 'sits with the other money rows'/below Balance) per item 7. Absorbs dropped new case FD-WO-022. Hidden-when-zero stays in FD-FIN-003 (no change). | VIU 2026-07-22 LIVE: Financial Info order = Parts $40.00, Labor $509.90, Shop Supplies $53.54, Fees &amp; Discounts (10) $273.31, Subtotal $876.75, GST, Total, Balance — F&amp;D line renders directly above Subtotal. Ev: wo/FD-FIN-004-FD-WO-021-card-financialinfo.png, wo/lines-bodytext.txt.</t>
         </is>
       </c>
@@ -2820,6 +3076,11 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
           <t>creation order re-proven on the document block (Flat fee &lt; WFee &lt; WDisc indices); read-only listing per batch-3 | WORDING+VIU 2026-07-13: Confirmed the Financial Info F&amp;D row is read-only (no add/edit/remove in this card).</t>
         </is>
       </c>
@@ -2862,6 +3123,11 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
           <t>tech (no SFD): WO view masks money (sub_total/total '0.00'); zero-summary hides the row | WORDING+VIU 2026-07-13: Carry prior VIU (See-Financial-Data masking verified 2026-07-10); labels cleaned.</t>
         </is>
       </c>
@@ -2904,6 +3170,11 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
           <t>card renders 'WO Fees &amp; Discounts / Flat fee $12.00 +$12.00' — label/name drift vs spec wording persists (case-update) | WORDING+VIU 2026-07-13: Sidebar card title is 'WO Fees &amp; Discounts' (was 'Work Order Fee / Discount'); per-row ⋮ menu shows 'Edit' and 'Remove' (confirmed live, shot fin-03). Now build-accurate. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: card entries reworded from 'signed rate badge' to plain text with bracketed percent + sign rule (item 5). Absorbs dropped new case FD-WO-020. Item-6 disclaimer intentionally left to FD-WO-021 (kept) to avoid duplication. | VIU 2026-07-22 LIVE: card titled 'Work Order Fees &amp; Discounts', lists only whole-WO entries as plain text with bracketed percent — fee 'Customer Fee (10%) +$65.88', discount 'WO Disc (−5%) −$32.94', flat 'Flat Fee 2 +$32.00'/'Flat Fee +$11.00' (name+amount, no brackets); each entry has a ⋮ menu; card renders above Financial Info. Ev: wo/FD-FIN-004-FD-WO-021-card-financialinfo.png, wo/lines-bodytext.txt. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -2946,6 +3217,11 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
           <t>sidebar card present with entries + no Add control (re-observed); hidden-when-none per batch-3 | WORDING+VIU 2026-07-13: Card title corrected to 'WO Fees &amp; Discounts'. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -2988,6 +3264,11 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-3 CONFIRMED AGAIN: auto-applied adjustments (auto template + auto pfees) write NO history entry (fresh WO: 1 auto adjustment, 0 adjustment events); manual add/edit/remove ARE logged (added=15/updated=1/removed=15 in today's battery) | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: CONFIRMED live: the 'Work Order Log' renders the bold event label 'Fee added' (columns Event/User/Line/Details/Date/Time; shot hist-01). Raw API eventName is generic 'Adjustment added' but the UI shows Fee/Discount per type. | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -3030,6 +3311,11 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-11 (details omit 'Type:' line) per batch-1; entry payload captured today (eventType/eventName/user fields); UI detail block not re-driven | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: CONFIRMED live: the Details column shows 'Name: &lt;name&gt;  Amount: &lt;set rate&gt;  Applied to: &lt;target&gt;' (shot hist-01; a flat fee showed 'Amount: $50,000,000.00' = the set rate). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -3072,6 +3358,11 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
           <t>adjustment entries carry lineId=null -&gt; Line column '−'; saved-state icon empty per batch | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: DEVIATION: the Line column shows the line number/name for a line-level entry (saw '43434'), not '−' for every entry as the old expected claimed. Confirmed live (shot hist-01). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -3114,6 +3405,11 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
           <t>tech (no SFD): history GET 200 incl. F&amp;D entries with SET rate — history independent of SFD | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no See Financial Data, view_mode:tech, financials masked) still gets the Work Order Log with fee/discount entries (history endpoint 200 with entries). The log shows the SET rate, so SFD does not gate it. | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -3156,6 +3452,11 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
           <t>View History Logs is an FE display gate (tech got 200 + 56 adjustment entries); documented enforcement model | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: Positive confirmed live (Tech has Work Orders/Work Order Lines: Create &amp; Edit → sees the log, 200). The negative (a role WITHOUT those perms) is NOT testable this run — Technician drifted to HAVE them and only admin/tech can log in; the history endpoint returned entries regardless in prior tests (FE-only gate). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -3198,6 +3499,11 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
           <t>extends FDBUG-3: auto-added pfee NOT logged on add; REMOVAL logged; no 'updated' entries (manual base fee logged correctly) | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: Processing-Fee logging carried (no live pfee on the sample WO); Applied to 'Full invoice' + no 'updated' entry. | V1_3 (2026-07-17): Δ2 — Story 10 renamed 'history log' -&gt; 'audit log' (terminology only; gates/behavior/status unchanged). Notes-only touch: the reader-facing text of this case already uses the exact build labels ('Audit Log' ⋮ menu / 'Work Order Log' page) and carries no generic history-log prose. The internal `area`/section name is left as-is (TestRail section rename not authorized).</t>
         </is>
       </c>
@@ -3240,6 +3546,11 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
           <t>work_order.adjustment.updated entry written on edit (set rate carried) | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: Set-rate-on-edit carried (Details Amount = set rate, confirmed for add; edit shows the new set rate). | V1_3 (2026-07-17): Δ2 — Story 10 renamed 'history log' -&gt; 'audit log' (terminology only; gates/behavior/status unchanged). Notes-only touch: the reader-facing text of this case already uses the exact build labels ('Audit Log' ⋮ menu / 'Work Order Log' page) and carries no generic history-log prose. The internal `area`/section name is left as-is (TestRail section rename not authorized).</t>
         </is>
       </c>
@@ -3282,6 +3593,11 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
           <t>batch UI evidence stands; today's headless text capture did not surface inline rows (grid render timing) — API line adjustment placement re-proven (adjustments under lines/{wo}) | WORDING+VIU 2026-07-13: Inline row labelled 'Fees/Discounts' with ↳, name, rate badge, grey amount confirmed live (shot fin-03). | SV-8479/8480 deconfliction 2026-07-22: reworded to blank left label + plain-text/no-badge with the −X%/X% sign rule (items 3 &amp; 4). Absorbs dropped new case FD-WO-019 (labor half). | LIVE STAGING VIU 2026-07-22 (viu-sv8479-8480-2026-07-22/): sign convention RE-VERIFIED live on the Lines tab — a percentage labor FEE renders as a BARE '20%' (no sign) in plain grey text (HTML span text-grey-7, no colored badge/pill); a percentage DISCOUNT renders '−10%' (en-dash minus); resolved amount is signed on the right ('+$58.00' / '−$4.00'); '↳' arrow, blank left label. Wording accurate — no change. Ev: 018/019-lines-expanded-full.png. | VIU 2026-07-22 LIVE re-confirmed: '↳ Labor Fee 20%' (fee bare %, blank left label, plain text, no badge) '+$101.98'; '↳ Labor Disc −10% −$50.99' (discount minus). Ev: wo/inline-expanded-text.txt, wo/inline-expanded.png.</t>
         </is>
       </c>
@@ -3324,6 +3640,11 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
           <t>as FD-INLINE-001; part-line adjustment lives under the part in lines payload (re-proven) | WORDING+VIU 2026-07-13: Inline part-line row confirmed live (↳ yiy [badge] +amount ⋮, shot wo-01/fin-03). | SV-8479/8480 deconfliction 2026-07-22: reworded to plain-text/no-badge with the −X%/X% sign rule (item 4). Absorbs dropped new case FD-WO-019 (part half). | LIVE STAGING VIU 2026-07-22: part-line sign convention RE-VERIFIED live — a percentage part FEE renders bare '11%' (no sign) plain grey text (no badge); a percentage part DISCOUNT renders '−10%' (en-dash minus); resolved signed '+$4.40' / '−$4.00'. Wording accurate — no change. Ev: 018/019-lines-expanded-full.png. | VIU 2026-07-22 LIVE re-confirmed: '↳ Part Fee 11% +$4.40' plain text, no badge. Ev: wo/inline-expanded-text.txt.</t>
         </is>
       </c>
@@ -3366,6 +3687,11 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
           <t>batch evidence stands (Total column incl own adjustments); not re-driven | WORDING+VIU 2026-07-13: Per-line Total stacks base + each adjustment; display-only. Labels cleaned. | SV-8480 (Story SV-8279, Done) 2026-07-22: strengthened to the explicit S3-R18 formula + $322.20 worked example + no-fee-line-unchanged sub-check. Kept inline-display scoped; the calc/document/flag-off ACs are owned by the new SV-8480 FD-CALC cases. viu_status unchanged (VIU-Verified) — re-observe at VIU. | LIVE STAGING VIU 2026-07-22 (viu-sv8479-8480-2026-07-22/): RE-CONFIRMED live — the collapsed line Total on the Lines tab adds the line's own SIGNED fee/discount amounts on top of gross Labor + Parts: $392.40 with a labor fee +20% ($58.00) + part fee +11% ($4.40) on a $290 labor / $40 parts line; $330.00 gross when the line has no fees; display-only, no stored value changes. Ev: 018-lines-collapsed-full.png, 020-lines-nofee-line.png, api-FD-CALC-018-024-total_cost-392.40.json.</t>
         </is>
       </c>
@@ -3408,6 +3734,11 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
           <t>3-dot Edit|Remove menu on adjustment entries re-observed (card menu 'Edit | Remove') | WORDING+VIU 2026-07-13: Inline line ⋮ menu shows 'Edit' and 'Remove' (was 'Edit'/'Delete') — confirmed live (shot inline-01).</t>
         </is>
       </c>
@@ -3450,6 +3781,11 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
           <t>label drift (subtitle 'Applying to: {line}' without 'Line {N} Labor —' prefix) per batch-1; not re-driven today | WORDING+VIU 2026-07-13: Menu item is 'Add Fee/Discount'; dialog subtitle 'Applying to: &lt;line name&gt;' (no 'Line N Labor —' prefix) — matches build. Labor-line ⋮ menu not re-captured this run; confirmed by symmetry with the part-line flow (⋮ = 'Move' / 'Add Fee/Discount', dialog 'Applying to: &lt;name&gt;') + prior 2026-07-10 VIU. | SV-8479/8480 deconfliction 2026-07-22: title reworded 'Add new fee/discount' -&gt; 'New Labor Fee / Discount', subline 'Applying to: &lt;line&gt;' -&gt; 'Applying To: Line N Labor — &lt;name&gt;' (item 8); entry point = ⋮ left of technician + 'Add Labor Fee / Discount' (item 1). Absorbs dropped new case FD-WO-023. | VIU 2026-07-22 LIVE: labor dialog title 'New Labor Fee / Discount', subline 'Applying To: Line 1 Labor — ZZAUTOTEST 8480 line', scope locked. Ev: wo/FD-LABOR-001-labor-dialog.png, wo/labor-dialog-text.txt.</t>
         </is>
       </c>
@@ -3492,6 +3828,11 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
           <t>pct_labor resolves against the line's LABOR total: on a 0-labor (parts-only) line 10% -&gt; $0.00 (correct base); $265-line evidence from batch-1 stands | WORDING+VIU 2026-07-13: Build labels; Calc default '% Of Labor Total' for labor scope. Labor-line ⋮ menu not re-captured this run; confirmed by symmetry with the part-line flow (⋮ = 'Move' / 'Add Fee/Discount', dialog 'Applying to: &lt;name&gt;') + prior 2026-07-10 VIU. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Labor Fee / Discount' / 'New Labor Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Labor Fee / Discount' confirmed present in the labor row ⋮ menu; case behavior unchanged. Ev: wo/FD-WO-017-labor-menu-open.png.</t>
         </is>
       </c>
@@ -3534,6 +3875,11 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
           <t>labor-line flat 9.99 -&gt; resolved 9.99 exactly, no quantity multiplier | WORDING+VIU 2026-07-13: Build labels; flat labor resolve carried. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Labor Fee / Discount' / 'New Labor Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Labor Fee / Discount' confirmed present in the labor row ⋮ menu; case behavior unchanged. Ev: wo/FD-WO-017-labor-menu-open.png.</t>
         </is>
       </c>
@@ -3576,6 +3922,11 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
           <t>prior decline-&gt;$0 evidence stands; today's decline flip blocked ('Can`t change status while there are staged parts' on S-15895's completed line; no fresh WO possible — line-create 500) | WORDING+VIU 2026-07-13: Declined-line $0 carried.</t>
         </is>
       </c>
@@ -3618,6 +3969,11 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
           <t>prior (line delete removes its adjustment); not re-seedable today (line-create 500 env-wide) | WORDING+VIU 2026-07-13: Delete-line cascades; carried; build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -3660,6 +4016,11 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
           <t>FE gate per roles-matrix derivation; CAVEAT: shared-env Technician role drifted (now has more perms) — re-derive matrix before relying on per-role negatives | WORDING+VIU 2026-07-13: Line-add gated by Work Order Lines: Create &amp; Edit. NOTE: re-check the negative after the roles matrix is re-derived. | SV-8479/8480 deconfliction 2026-07-22: label updated 'Add Fee/Discount' -&gt; 'Add Labor Fee / Discount' + entry-point wording (item 1); permission behavior unchanged. | VIU 2026-07-22 LIVE: menu label 'Add Labor Fee / Discount' confirmed present; permission-negative behavior (hidden without Work Order Lines: Create &amp; Edit) unchanged from prior verification — role-negative not re-driven this UI batch.</t>
         </is>
       </c>
@@ -3702,6 +4063,11 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-14 label defects (missing 'Line {N} Part —' prefix, raw enum 'Pct_parts', part-% option mislabeled '% of Labor Total') per batch-4; part dialog not re-driven today | WORDING+VIU 2026-07-13: CONFIRMED live: part ⋮ = 'Move' / 'Add Fee/Discount'; dialog 'Add new fee/discount' with subtitle 'Applying to: &lt;part name&gt;' (NO 'Line N Part —' prefix — build differs from the old spec text); Calc default '% Of Parts Total' (shots line-01/02). Now build-accurate. | SV-8479/8480 deconfliction 2026-07-22: menu item 'Add Fee/Discount' -&gt; 'Add Part Fee / Discount' (item 2); title 'Add new fee/discount' -&gt; 'New Part Fee / Discount', subline 'Applying to: &lt;part&gt;' -&gt; 'Applying To: Line N Part — &lt;name&gt;' (item 9). Absorbs dropped new case FD-WO-024. | VIU 2026-07-22 LIVE: part menu label 'Add Part Fee / Discount' + dialog title 'New Part Fee / Discount', subline 'Applying To: Line 1 Part — Turbocharger Oil', default Calculation Type '% Of Parts Total'. Ev: wo/FD-PART-001-part-dialog.png, wo/part-dialog-text.txt.</t>
         </is>
       </c>
@@ -3744,6 +4110,11 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
           <t>per-item flat re-proven: $2.00 x qty 4 -&gt; $8.00 on S-15895's received part (estimate row 'ZZAUTOTEST PartFlat $8.00') | WORDING+VIU 2026-07-13: Per-item flat carried; build labels. | SV-8479/8480 deconfliction 2026-07-22: inline part-row rendering reworded from '−$5.00 flat rate badge' to plain text (item 4); per-item flat calc unchanged. | VIU 2026-07-22 LIVE: inline part fee renders plain text ('Part Fee 11% +$4.40'), no colored badge; per-item flat calc unchanged (verified prior passes). Ev: wo/inline-expanded-text.txt.</t>
         </is>
       </c>
@@ -3786,6 +4157,11 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
           <t>prior batch-4 requested-state evidence stands; not re-seedable today (make-request -&gt; 400 'Part requests can`t be modified on completed line', line-create 500) | WORDING+VIU 2026-07-13: Add-to-requested-part carried; build labels. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Part Fee / Discount' / 'New Part Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Part Fee / Discount' confirmed present in the part row ⋮ menu; case behavior unchanged. Ev: wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
@@ -3828,6 +4204,11 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
           <t>pct_parts re-proven: 10% of qty4 x 42.69 = 170.76 -&gt; $17.08 | WORDING+VIU 2026-07-13: %-of-parts base carried; build labels. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Part Fee / Discount' / 'New Part Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Part Fee / Discount' confirmed present in the part row ⋮ menu; case behavior unchanged. Ev: wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
@@ -3870,6 +4251,11 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
           <t>prior decline-&gt;$0 (batch-4) stands; decline flip blocked today (staged-parts lock) | WORDING+VIU 2026-07-13: Declined/returned part $0 carried.</t>
         </is>
       </c>
@@ -3912,6 +4298,11 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
           <t>prior delete-cascade (batch-4) stands; not re-seedable today | WORDING+VIU 2026-07-13: Delete-part cascades; carried; build labels.</t>
         </is>
       </c>
@@ -3954,6 +4345,11 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
           <t>qty-1 flat = base amount (batch); per-item semantics re-proven today at qty 4 | WORDING+VIU 2026-07-13: Per-item edge carried; build labels.</t>
         </is>
       </c>
@@ -3996,6 +4392,11 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
           <t>RE-CHECKED TODAY on a freshly created part sale (P3-127): NO 'Fees &amp; Discounts' column on the part-sale page; API add against a part-sale id -&gt; 400 needs-target (no part-sale adjustment surface). Story 11 still NOT BUILT (shot 12-part-sale) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Column shows single fee/discount name+rate (Fee $6.00 / Discount -11%). Live staging (ps-scrolled).</t>
         </is>
       </c>
@@ -4038,6 +4439,11 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
           <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: +N badge on multi-fee part (Fee $6.00 +1). Live staging (psB4-badge.png). | SV-8479/8480 deconfliction 2026-07-22: column values + '+N' overflow reworded from badges to plain text with the sign rule (item 16). Absorbs dropped new case FD-PSALE-005. (FD-PCOL-001 already plain text — no change.) | SV-8479 Batch-3 STAGING LIVE VIU 2026-07-22 (part-sale surface): seeded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: NEXUS cell = 'Part Fee 11% +1' plain text, no badge, fee no sign.</t>
         </is>
       </c>
@@ -4080,6 +4486,11 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
           <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Filled cell opens viewer with Name/Type/Calculation/Amount/Max Amount columns. Live staging (psC-viewer2rows.png).</t>
         </is>
       </c>
@@ -4122,6 +4533,11 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
           <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Viewer Net adjustment = signed sum (+$12.00 + $2.00 = +$14.00). Live staging (psC-viewer2rows.png).</t>
         </is>
       </c>
@@ -4164,6 +4580,11 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
           <t>Story 11 surface absent (re-checked today) | WORDING+VIU 2026-07-13:  NOT BUILT: Story 11 (Part Sales fees/discounts) has not shipped — the Parts page has no 'Fees &amp; Discounts' column and there is no part-sale F&amp;D surface. Wording made build-accurate/layman for when it ships; status stays Blocked-NotBuilt. | STAGING VIU 2026-07-20 staging LIVE VIU: Per-row Remove -&gt; confirm Remove Fee / Discount -&gt; row removed. Live staging (psE-confirm/afterremove). | SV-8479/8480 deconfliction 2026-07-22: empty-state reworded: the removed '+ Add' button is gone; add via the per-row ⋮ (item 13). | SV-8479 Batch-3 STAGING LIVE VIU 2026-07-22 (part-sale surface): seeded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: breakdown viewer per-row delete -&gt; confirm 'Remove Fee / Discount' -&gt; removed -&gt; empty state, no '+ Add'.</t>
         </is>
       </c>
@@ -4206,6 +4627,11 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
           <t>tech (no SFD): WO view masks all money (sub_total/total '0.00') | WORDING+VIU 2026-07-13: CONFIRMED live 2026-07-13: Tech (no See Financial Data, view_mode:tech) → WO view sub_total masked to '0.00' (amounts hidden).</t>
         </is>
       </c>
@@ -4248,6 +4674,11 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
           <t>positive half fresh (tech WITH lines-C&amp;E: line add 201/remove 204); negative half via roles-matrix FE derivation (role-drift caveat) | WORDING+VIU 2026-07-13: Positive: Tech HAS Work Order Lines: Create &amp; Edit. Negative not testable (Tech drifted to have it). Line-level gate carried from prior derivation.</t>
         </is>
       </c>
@@ -4290,6 +4721,11 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
           <t>Part Sales adjustment surface absent (Story 11 re-checked today) | WORDING+VIU 2026-07-13: NOT BUILT: Story 11 Part Sales fees/discounts not shipped; cannot test the Part Sales permission gate. | STAGING VIU 2026-07-20 staging LIVE VIU: Admin (Part Sales C&amp;E + SFD) can add/edit/remove part-sale F&amp;D; Tech (no Part Sales perms) has Parts nav hidden entirely. Live staging.</t>
         </is>
       </c>
@@ -4332,6 +4768,11 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
           <t>SFD prerequisite: controls live on SFD-masked surfaces (tech masked view re-confirmed) | WORDING+VIU 2026-07-13: See-Financial-Data masking confirmed live (Tech financials masked). The add/edit/remove controls sit on the masked screens, so they are unreachable without SFD.</t>
         </is>
       </c>
@@ -4374,6 +4815,11 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
           <t>removal uses the same Create&amp;Edit gate (tech remove 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove via Create &amp; Edit (not a separate Delete) carried.</t>
         </is>
       </c>
@@ -4416,6 +4862,11 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
           <t>templates admin BE-enforced: tech GET/POST 403 | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no Settings → Finance) → GET templates 403 'Access denied.' | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -4458,6 +4909,11 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
           <t>customer defaults BE-enforced: tech GET 403 + POST 403 | WORDING+VIU 2026-07-13: CONFIRMED live: Tech (no Manage AP/AR, no Customer Mgmt C&amp;E) → customer default-adjustments GET 403 AND POST 403 'Access denied.'</t>
         </is>
       </c>
@@ -4500,6 +4956,11 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
           <t>history entries: BE serves them regardless (tech 200) — FE display gate per enforcement model; entries carry set rate | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: Positive confirmed live (Tech has Work Orders/Work Order Lines: Create &amp; Edit → Work Order Log 200 with fee/discount entries; the log shows the set rate so See Financial Data does not gate it — Tech's financials are masked yet history shows). The no-permission negative is NOT testable this run (Tech drifted to have the perms; only admin/tech log in). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -4542,6 +5003,11 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
           <t>flag ON + permission still required (tech 403 on templates/defaults with flag ON) | WORDING+VIU 2026-07-13: Permission gating confirmed live (templates/customer-defaults 403; SFD masking). Feature is ON. Both-gates model holds. | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -4584,6 +5050,11 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
           <t>Invoiced WO: add 409 + edit 409 (BE-enforced lock) | WORDING+VIU 2026-07-13: Invoiced/Paid block is back-end enforced (409) — established; carried. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -4626,6 +5097,11 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
           <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -4668,6 +5144,11 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
           <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -4710,6 +5191,11 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
           <t>RE-CHECKED TODAY: template-builder Type options are exactly [Fee, Discount] — Processing Fee STILL MISSING from the builder UI (PO Q3=B says in-scope; FDBUG-8; shot 02-template-dialog) | WORDING+VIU 2026-07-13: Confirmed live: Type dropdown = Fee/Discount only. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Type dropdown offers Fee, Discount, Processing Fee (admin template dialog). Live-observed staging (proc-type-open).</t>
         </is>
       </c>
@@ -4752,6 +5238,11 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
           <t>builder UI absent (re-checked today); BE method constraint re-proven separately (pct_labor rejected for processing_fee) | WORDING+VIU 2026-07-13: Builder not shipped. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Processing Fee Calc Type = Flat Amount + % of Grand Total only. Live staging (proc-fee-calc-open.png).</t>
         </is>
       </c>
@@ -4794,6 +5285,11 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
           <t>builder UI absent (re-checked today); BE rejects pfee maxCap (400) | WORDING+VIU 2026-07-13: Builder not shipped. NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: No Max Amount field for Processing Fee (both methods). Live staging (proc-fee-full.png).</t>
         </is>
       </c>
@@ -4836,6 +5332,11 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
           <t>builder UI absent (re-checked today) | WORDING+VIU 2026-07-13: Builder not shipped; when it ships, also check the §5-R15 note (currently absent in the whole-WO dialog per FD-WO-016). NOT BUILT: the template Type dropdown offers only Fee/Discount (no 'Processing Fee'); the Story-8 Processing-Fee builder UI has not shipped. The back-end DOES accept kind=processing_fee via API (201). Re-test when the builder ships. | V1_3 (2026-07-17): Δ1 — §5-R15 gains one appended sentence (spec verbatim): 'The note is shown only to users with See Financial Data.' Expected gains the gate qualifier. This dialog is the one place the gate is independently observable (Story-7 admin access needs no See Financial Data, while the WO Add/Edit dialog already requires it — spec-diff §H.b). Status stays Blocked-NotBuilt (Story-8 builder UI absent); check the note + gate when the builder ships. | STAGING VIU 2026-07-20 staging LIVE VIU: Processing Fee Taxable defaults Yes + jurisdiction note present; note gated on See Financial Data (Tech w/o SFD sees toggle, not note). Live staging (proc-fee-full.png / tech-tmpl-dialog.png).</t>
         </is>
       </c>
@@ -4878,6 +5379,11 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
           <t>manual pfee add -&gt; 400 'A processing fee cannot be added manually.'; manual pct_grand_total fee also rejected for scope | WORDING+VIU 2026-07-13: Confirmed: WO Add Type dropdown = Fee/Discord only (no Processing Fee); build labels ('Add Fee/Discount', 'Apply From Template'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -4920,6 +5426,11 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
           <t>auto-apply pfee template landed on a fresh WO (kind=processing_fee, appliedBy=auto) | WORDING+VIU 2026-07-13: Reaches WO via auto-apply (pfee accepted by BE); build labels. Menu option is 'Remove' (Edit inert for a pfee). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -4962,6 +5473,11 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
           <t>customer-default pfee landed on a fresh WO (kind=processing_fee, appliedBy=customer_default, amount 2.5) | WORDING+VIU 2026-07-13: Reaches WO via customer default; build labels. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -5004,6 +5520,11 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
           <t>pfee template with maxCap -&gt; 400; pfee with pct_labor -&gt; 400 'not allowed for a processing_fee' | WORDING+VIU 2026-07-13: Confirmed live 2026-07-13 via API: Max cap → 400 'A processing fee cannot have a minimum or maximum cap.'; disallowed method → 400 'Calculation type "pct_subtotal" is not allowed for a processing_fee.' Lives in an API-titled section.</t>
         </is>
       </c>
@@ -5046,6 +5567,11 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
           <t>pfees resolve as positive fees only (kind=processing_fee, amounts &gt;= 0) | WORDING+VIU 2026-07-13: Always a plus; carried.</t>
         </is>
       </c>
@@ -5088,6 +5614,11 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
           <t>template amount 3-&gt;9 (200) left the existing WO pfee at 3 (values copied at apply time) | WORDING+VIU 2026-07-13: Template edit independence; carried.</t>
         </is>
       </c>
@@ -5130,6 +5661,11 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
           <t>two auto pfees (3%+2%) resolved 0.63/0.42 = exact 3:2 ratio -&gt; same base, pfees exclude each other | WORDING+VIU 2026-07-13: Multiple pfees share the same base; carried.</t>
         </is>
       </c>
@@ -5172,6 +5708,11 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
           <t>pfee minimum silently STRIPPED on create (201, no min field persisted) — §8 invariant holds; silent-ignore wording note stands | WORDING+VIU 2026-07-13: Confirmed live 2026-07-13: BE rejects a min/max cap on a Processing Fee (400 'A processing fee cannot have a minimum or maximum cap.'). PO Q4 (whether pfee minimums should be supported at all) still pending. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q4=B): PO ruled Processing Fees do NOT support a minimum and the app must make that clear (do not silently drop). Premise confirmed WAD: no minimum field in the UI and the API rejects a pfee minimum with an explicit error (matches the live 2026-07-13 finding: 400 'A processing fee cannot have a minimum or maximum cap.'). Older 2026-07-10 'silent strip' reading superseded (last-update-wins). Expected reworded to the explicit-reject + no-field behavior. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md).</t>
         </is>
       </c>
@@ -5214,6 +5755,11 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
           <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -5256,6 +5802,11 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve"> NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. F&amp;D column has no '+ Add' (grep '+Add'=0); per-row ⋮ 'Add Part Fee / Discount' + top-right ⋮ 'Add Parts Sale Fee / Discount' both present.</t>
         </is>
       </c>
@@ -5298,6 +5849,11 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
           <t>TEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Per-part ⋮ menu text = 'Add Part Fee / Discount' exactly; opens 'New Part Fee / Discount' dialog.</t>
         </is>
       </c>
@@ -5340,6 +5896,11 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
           <t>/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Whole-sale card 'Parts Sale Fees &amp; Discounts' live: 'Customer Fee (10%) +$82.12', 'Sale Disc (−5%) −$41.06', 'Flat Fee +$50.00' (flat name-only), 'Processing Fee (6%) +$51.73' — plain text, no badge, bracket %/sign convention matches WO card item 5.</t>
         </is>
       </c>
@@ -5382,6 +5943,11 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
           <t>ded ZZAUTOTEST part sale P3-1118 (2 fee-less rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Live: 'Fees &amp; Discounts (6) $189.27' directly above Subtotal $963.95 in Financial Info.</t>
         </is>
       </c>
@@ -5424,6 +5990,11 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
           <t>). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. VIU-CONFIRM RESOLVED (Picture 26 was missing): top-right ⋮ label CONFIRMED LIVE = 'Add Parts Sale Fee / Discount'; dialog title 'New Parts Sale Fee / Discount'; subline 'Applying To: Entire Parts Sale'. Case wording already matched.</t>
         </is>
       </c>
@@ -5466,6 +6037,11 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
           <t>ss rows + NEXUS 2-adj) + whole-sale percent/flat/discount; observed live as admin (Part Sales C&amp;E + SFD). Evidence build/fees-discounts/viu-sv8479-8480-2026-07-22/psale/. Statistics F&amp;D (6) section live headings '% Amount'; flat fee blank %; rows +11%/+6%/+10% fees + −5% discounts; 'Total +$189.27'.</t>
         </is>
       </c>
@@ -5508,6 +6084,11 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
           <t>floor worked-example halves re-proven at WO level: non-taxable over-discount -&gt; sub 0.00, tax UNCHANGED (9.14), total=tax, excess 117.24; taxable variant -&gt; tax 0.00, total 0.00 | WORDING+VIU 2026-07-13: In-app floor VERIFIED (same worked example as FD-CALC-015, confirmed 2026-07-10); the customer pays the tax only.</t>
         </is>
       </c>
@@ -5550,6 +6131,11 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-15 CONFIRMED AGAIN (API half): over-discount saves 201 with NO warning payload; excess carried silently (117.24). Batch-6 UI shots show no warn/confirm dialog. Violates S6-R12 | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-15 / PO Q1 pending): an over-discount currently saves SILENTLY — no mandatory warn/confirm before saving. Expected kept as the spec requirement. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q1=A): PO ruled the warn/confirm is required AND already exists per spec (S6-R12) — it fires before invoicing and before marking the WO reviewed/complete, NOT when the adjustment is merely added (add is uncommitted; the Add dialog preview shows the resulting totals). Our FDBUG-15 'silent save' was observed at ADD time = the wrong trigger point; PO says that is intentional. FDBUG-15 reclassified NOT-A-DEFECT (no dev ticket released). Expected reworded to the commit-point warning. Status -&gt; VIU-Pending: the invoice/mark-reviewed/complete warning has not yet been observed live and needs a commit-time re-VIU. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). COMMIT-TIME RE-VIU 2026-07-14: attempted but BOTH qb cookie sets (cookies-viu.env 2026-07-13, cookies-fresh.env 2026-07-10) return 401 sso_required on quick-login (env woken, API root 200) — cookies EXPIRED. Left VIU-Pending: needs fresh qb cookies for the commit-time (invoice / mark-reviewed / complete) re-VIU. | COMMIT-TIME RE-VIU SETTLED 2026-07-14 (fresh qb cookies): VERIFIED. Live FE source + live data-condition confirm Chris's Q1=A exactly. (1) ADD-TIME SILENT: the Add/Edit dialog component (AdjustmentDialog) has NO over-discount warning and does not import the warning dialog -- adding an over-sized discount is silent (only an unrelated 'A percentage discount cannot exceed 100%' field check). (2) COMMIT-TIME WARN/CONFIRM BUILT: a dedicated component OverDiscountWarningDialog exists (title 'Discount exceeds subtotal'; body "The total discount exceeds this work order's subtotal. The subtotal will be reduced to $0.00, but any tax on the taxable base is still owed. The remaining $&lt;excess&gt; will be carried as a customer credit. Continue?"; buttons Continue / Cancel). It is imported and wired in the Invoice component: the Create-Invoice handler (Lt-&gt;_a) AND the mark-reviewed/Complete handler (Vt-&gt;ga, posts status:'complete') BOTH intercept when the excess-credit gate is true (FeesAndDiscounts flag ON &amp;&amp; not partSale &amp;&amp; adjustmentsSummary.excessCreditAmount&gt;0), open the dialog, and only run the commit on Continue (confirm) / abort on Cancel. So the mandatory warn/confirm fires at BOTH commit points, never silently. (3) LIVE DATA CONDITION: on WO S-15970 added a $9,999 whole-WO flat discount (reversible ZZAUTOTEST, removed after) -&gt; sub_total floored to $0.00, adjustmentsSummary.excessCreditAmount=9522.26 (&gt;0) =&gt; the FE gate evaluates TRUE, so the dialog would fire at Create Invoice / Mark-Reviewed / Complete. WO restored byte-identical to baseline afterward. Evidence: FE chunks OverDiscountWarningDialog.BCmTBE33.js + Invoice.Ny62BJnd.js + AdjustmentDialog.S8gN6cAn.js (captured live from qb.qa.shopview.com 2026-07-14); live API view before/after. Verdict: VIU-Verified. FDBUG-15 stays NOT-A-DEFECT (add-time silence is intentional). Expected wording already build-accurate (floor $0.00 + tax on taxable base still owed + exact excess as customer credit + must confirm) -&gt; no TestRail wording change needed; status flip local only. Exact on-screen labels now captured for the record: dialog 'Discount exceeds subtotal', buttons 'Continue'/'Cancel'.</t>
         </is>
       </c>
@@ -5592,6 +6178,11 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
           <t>remove-confirm wording drift per batch-1 (case-update); not re-driven today | WORDING+VIU 2026-07-13: Confirm dialog matched EXACTLY live: title 'Remove Fee / Discount', message 'Are you sure you want to remove this fee?', buttons 'Remove'/'Cancel' (shot inline-02; cancelled — no shared data deleted). Toast not re-observed this run. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -5634,6 +6225,11 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
           <t>removal governed by Create&amp;Edit (tech WITH lines-C&amp;E removed line-level 204; no Delete-perm dependency) | WORDING+VIU 2026-07-13: Remove uses Create &amp; Edit not a separate Delete permission; carry prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -5676,6 +6272,11 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
           <t>line-level remove 204 and gone from the line | WORDING+VIU 2026-07-13: Inline menu option is 'Remove' (was 'Delete'); confirm dialog 'Remove Fee / Discount' confirmed live.</t>
         </is>
       </c>
@@ -5718,6 +6319,11 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
           <t>part flat + part pct resolved independently on the part's own gross (fresh: $8.00 and $17.08 coexist, no compounding) | WORDING+VIU 2026-07-13: Netting carried; build labels. Display half (only first shows + 'Show N more') is the FD-INLINE-003 deviation (no Show-N-more in this build).</t>
         </is>
       </c>
@@ -5760,6 +6366,11 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
           <t>two 10% whole-WO fees resolve 17.08 each (same base, no compounding) | WORDING+VIU 2026-07-13: Same-base netting carried; build labels.</t>
         </is>
       </c>
@@ -5802,6 +6413,11 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
           <t>'Flat fee' template applied twice by hand -&gt; 201/201, two distinct adjustments | WORDING+VIU 2026-07-13: Same-template-twice carried; build labels ('Add Fee/Discount', 'Apply From Template', 'WO Fees &amp; Discounts'). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -5844,6 +6460,11 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
           <t>CONFIRMED AGAIN: Stats shows aggregate 'Fees &amp; Discounts (5) $25.00' style block, NOT the per-row Value/%+Amount table — PO Q1=B design regression persists (shot 07-stats) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-2): the Stats 'Fees &amp; Discounts (N)' section lists rows (name, a value/% for percentages, and an amount) but has NO 'Value'/'Amount' column headers like the other Stats sections. Confirmed live (shot fin-01). | SV-8479/8480 deconfliction 2026-07-22: added the right-side '%' and 'Amount' column headings + blank-% for flat fees (item 12). Absorbs dropped new case FD-WO-027. viu_status unchanged (VIU-Deviation) — re-observe at VIU. | VIU 2026-07-22 LIVE: prior 'no headers' deviation RESOLVED — Stats tab 'Fees &amp; Discounts (10)' section now shows the '% Amount' column headings. Rows show percent under % (blank for flat: 'Flat Fee 2 +$32.00', 'Flat Fee +$11.00') and signed amount under Amount ('Labor Fee +20% +$101.98', 'Labor Disc −10% −$50.99', 'Customer Fee +10% +$65.88', 'WO Disc −5% −$32.94'), with 'Total +$273.31'. Ev: wo/FD-STATS-001-stats-tab.png, wo/stats-bodytext.txt.</t>
         </is>
       </c>
@@ -5886,6 +6507,11 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
           <t>net = signed sum re-consistent (adjustmentsSummary netAmount matches card); full UI table from batch-2 | WORDING+VIU 2026-07-13: Total = signed sum; carry prior VIU. Minus-sign jargon removed.</t>
         </is>
       </c>
@@ -5928,6 +6554,11 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
           <t>no-adjustments WO -&gt; adjustments=[] + all-zero summary -&gt; section hidden | WORDING+VIU 2026-07-13: Section hidden with no adjustments; carry prior VIU.</t>
         </is>
       </c>
@@ -5970,6 +6601,11 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
           <t>admin library lives under Administration -&gt; FINANCE (route /administration/adjustment-templates), not Service-below-Canned-Lines; page re-loaded today (case-update per S13-R8 target) | WORDING+VIU 2026-07-13: CORRECTED location: templates live under Administration → FINANCE → 'Fees &amp; Discounts' (below 'Payment Methods'), NOT 'Service, below Canned Lines' (Canned Lines is under SERVICE). Confirmed live (shot tmpl-02-create-dialog). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6012,6 +6648,11 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
           <t>list + delete action per batch-1; page renders today; columns not re-verified individually | WORDING+VIU 2026-07-13: List columns confirmed live (shot tmpl-02). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6054,6 +6695,11 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
           <t>PARTIAL IMPROVEMENT: create-dialog title NOW 'New Fee / Discount' (matches spec; was 'Add new fee/discount'); confirm button still 'Create' (spec 'Add Fee / Discount') and toast 'Template created' per batch-1 — drift remains | WORDING+VIU 2026-07-13: Create dialog confirmed live: title 'New Fee / Discount', fields Name/Type/Calculation Type/'$ Default Amount'/Taxable toggle/'Auto-apply to new work orders' toggle/'Description (Optional)', 'Create' button. Type offers only Fee/Discount (Processing Fee is NOT in the builder — Story 8 not built). Create API 201 live. Toast text carried from prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6096,6 +6742,11 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
           <t>generic 'Template created' toast vs spec 'Discount added' per batch-1; not re-driven | WORDING+VIU 2026-07-13: CORRECTED title: the toast is generic (not a per-type 'Discount added'). Create dialog + list confirmed live. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6138,6 +6789,11 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
           <t>auto-apply template ('Capped discount' + test pfees) landed on every fresh WO as appliedBy=auto | WORDING+VIU 2026-07-13: CORRECTED auto-apply label: dialog toggle is 'Auto-apply to new work orders'; list column 'Auto-Apply To Work Orders'. Confirmed live (shot tmpl-02). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6180,6 +6836,11 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
           <t>edit locks Type+Calc on template edit (spec locks only in WO dialog) per batch-1; not re-driven | WORDING+VIU 2026-07-13: Edit dialog title 'Edit Fee / Discount' + 'Save' button confirmed on the fee/discount Edit dialog (shot edit-01). Edit opens from the row's pencil button. Toast text carried.</t>
         </is>
       </c>
@@ -6222,6 +6883,11 @@
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
           <t>delete-confirm dialog + affectedCustomerCount warning per batch-1; delete-precondition endpoint intact | WORDING+VIU 2026-07-13: Delete confirm confirmed live: standardized 'Delete Template' dialog with 'Cancel' + red 'Delete' (shot tmpl-03). The plain (no-customer) body wording was not captured this run — the sample template had a customer default (see FD-TMPL-008).</t>
         </is>
       </c>
@@ -6264,6 +6930,11 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
           <t>standardized 'Delete Template' dialog wording = intended per epic; case-update to adopt live wording still pending | WORDING+VIU 2026-07-13: Customer-default warning confirmed live EXACTLY: 'This template is set as a default for N customer(s). Deleting it will remove it from them.' (saw '1 customer', shot tmpl-03).</t>
         </is>
       </c>
@@ -6306,6 +6977,11 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
           <t>template deleted (204) -&gt; WO adjustment made from it survives unchanged (resolved 6 intact) | WORDING+VIU 2026-07-13: Delete leaves WO adjustments unchanged; carried. Nav corrected to Finance. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6348,6 +7024,11 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
           <t>maxCap 0 accepted and STORED as 0 on the template (201) and WO resolve treats 0 as NO cap (34.15) — FDBUG-9 persists | WORDING+VIU 2026-07-13: Max Amount only for % confirmed (WO+template dialogs). DEVIATION (PO Q2): a Max Amount of 0 is treated as 'no cap'. Labels cleaned. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount = 'no limit' (WAD, S2-R25). 0-handling no longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md).</t>
         </is>
       </c>
@@ -6390,6 +7071,11 @@
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
           <t>discount template 150% -&gt; 400; fee template 150% -&gt; 201 | WORDING+VIU 2026-07-13: %&gt;100 discount rejected (confirmed via API 2026-07-13: 'A percentage discount cannot exceed 100%').</t>
         </is>
       </c>
@@ -6432,6 +7118,11 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
           <t>builder offers exactly 4 whole-WO methods (Flat, % Labor, % Parts, % Subtotal), no scope field, no legacy '% Labor+Parts' | WORDING+VIU 2026-07-13: Calc Type options confirmed (same 4 whole-WO methods as the WO dialog); no scope field.</t>
         </is>
       </c>
@@ -6474,6 +7165,11 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
           <t>template empty name -&gt; 400; amount 0 -&gt; 400 (save-failure surfaced) | WORDING+VIU 2026-07-13: Save-failure toast text carried from prior VIU (not force-failed this run).</t>
         </is>
       </c>
@@ -6516,6 +7212,11 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
           <t>BE-enforced: tech templates GET/POST -&gt; 403; page FE-gated settingsFinance | WORDING+VIU 2026-07-13: Templates admin is back-end gated by Settings → Finance (Tech → 403), established batch-2. Nav corrected to Finance. NOTE: re-check the Tech negative after the roles matrix is re-derived (Technician drifted on shared qb). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6558,6 +7259,11 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
           <t>name 100ch -&gt; 201; 101ch -&gt; 400 | WORDING+VIU 2026-07-13: Name 100-char limit carried.</t>
         </is>
       </c>
@@ -6600,6 +7306,11 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
           <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6642,6 +7353,11 @@
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
           <t>CONFIRMED AGAIN: Add button enabled on empty form (validates on submit) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: DEVIATION re-confirmed 2026-07-13 (BUG-FD-4): the 'Add Fee' button is ENABLED on an empty form (validates on submit). Labels build-accurate (Add Fee/Add Discount, Calculation Type, Max Amount). | STAGING VIU 2026-07-20 staging LIVE VIU: BUG-FD-4 FIXED on staging: confirm button disabled until Name+Type+Calc+Amount&gt;0 set. Live-observed (dev-wo-emptyform + part-sale Add Fee disabled-until-valid). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -6684,6 +7400,11 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
           <t>amount 0 -&gt; 400 (API); UI inline error on submit | WORDING+VIU 2026-07-13: Blank/0 amount blocked; carry prior VIU. Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -6726,6 +7447,11 @@
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
           <t>UI blocks empty name (inline required error). NEW FDBUG-16: raw API now ACCEPTS empty-name adds (201; regression vs batch-3 400) — FE-only guard; name 101ch -&gt; 400, 100ch -&gt; 201 | WORDING+VIU 2026-07-13: Empty name blocked in UI; 100-char limit. (Raw back-end accepts empty name — FDBUG-16 — but the dialog blocks it.) | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -6768,6 +7494,11 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
           <t>discount &gt;100% invalid (400), fee uncapped (201) | WORDING+VIU 2026-07-13: %&gt;100 discount invalid, fee uncapped; carry prior VIU. Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -6810,6 +7541,11 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
           <t>negative amount -&gt; 400 | WORDING+VIU 2026-07-13: Negatives rejected; carry prior VIU. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -6852,6 +7588,11 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-9: maxCap 0 behaves as NO cap (not 'no maximum' spec reading matches build for empty, but 0 disagrees w/ §5-R6 $0-forces-$0) — persists | WORDING+VIU 2026-07-13: Confirmed live: '$ Max Amount (Optional)' appears only for percentage methods (hidden for Flat Amount, shots wo-03/wo-05). DEVIATION (FDBUG-9 / PO Q2 pending): whether a Max Amount of 0 means 'no cap' or 'cap at $0.00' is a pending product decision — expected kept as current build behavior. | CHRIS WARD ROUND-2 ANSWER APPLIED 2026-07-14(Q2=A): PO ruled a typed 0 in Max Amount = 'no limit' (WAD, S2-R25). 0-handling no longer a deviation; FDBUG-9 closed as accepted; jira draft TICKET 4 DROPPED. Expected reworded to affirm 0=no-cap. PUSHED TO TESTRAIL 2026-07-14 via update_case (QA-lead one-day authorization; update 200 / re-verify 200 MATCH; audit: testrail-round2-push-log.md). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -6894,6 +7635,11 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
           <t>auto+default template -&gt; exactly ONE adjustment on the new WO | WORDING+VIU 2026-07-13: Double-add does not stack (one adjustment); carry prior VIU. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -6936,6 +7682,11 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
           <t>dialog title still 'Add new fee/discount' (spec 'New Fee / Discount'), menu item 'Add Fee/Discount' — label drift persists (UI re-driven, shot 10-wo-add-dialog) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Now build-accurate (was VIU-Deviation only because the case used the older spec wording). Dialog shows no work-order-number subtitle in this build (old expected claim dropped). | SV-8479/8480 deconfliction 2026-07-22: menu item 'Add Fee/Discount' -&gt; 'Add Work Order Fee / Discount' (item 10); title 'Add new fee/discount' -&gt; 'New Work Order Fee / Discount' + new subline 'Applying To: Entire Work Order' (item 11, reverses the old 'no Applying-to line' claim). Absorbs dropped new case FD-WO-026. | VIU 2026-07-22 LIVE: whole-WO dialog opens from toolbar menu; title 'New Work Order Fee / Discount', subline 'Applying To: Entire Work Order', no scope dropdown. Ev: wo/FD-WO-001-wo-dialog.png, wo/wo-dialog-text.txt.</t>
         </is>
       </c>
@@ -6978,6 +7729,11 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
           <t>whole-WO flat fee add 201 + visible in WO view (flat 7.77 resolved exactly) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Sidebar card is 'WO Fees &amp; Discounts' (was 'Work Order Fee / Discount'). Exact success-toast text not re-captured this pass (worded as 'a success message'). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. Re-confirmed on current staging build — 8 UI corrections intact (Taxable Yes/No dropdown; Auto-apply checkbox+caption; modal field order Type/CalcType&gt;Name&gt;Amount&gt;Taxable+jur.note&gt;Auto-apply&gt;Description; Settings table plain-text left-aligned no badges; F&amp;D nav under SERVICE below Canned Lines; WO &amp; Part-Sale cards above Financial Info [Batch 2/3]; Customer 'Fees &amp; Discounts' tab mirrors Settings styling minus convenience toggle) AND Settings-&gt;Service permission pivot CONFIRMED live per role (seeded ServiceRole vs FinanceRole, assigned to Tech, Tech restored to Technician 50bf6a0d + verified, both ZZAUTOTEST roles deleted 204): Service-user sees+manages F&amp;D nav + convenience toggle, direct /administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -7020,6 +7776,11 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
           <t>dialog live preview re-driven ($5 flat -&gt; '+$5.00 / New work-order subtotal $187.76'); pct preview math not re-driven, API pct resolution re-proven (10%-&gt;17.08) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calc type corrected from generic 'Percentage' to the real whole-WO option '% of Subtotal'. Exact preview row labels not re-captured this pass (behavior verified 2026-07-10). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7062,6 +7823,11 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
           <t>not re-driven today (Apply-From-Template combobox present in dialog); templateId add path re-proven via API (FD-STACK-003) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Dropdown label is exactly 'Apply From Template' (was 'Apply from template (optional)'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7104,6 +7870,11 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
           <t>CONFIRMED AGAIN: 'Add Fee' button ENABLED on an empty form (disabled-on-empty=false) — PO Q4=B defect persists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION re-confirmed live 2026-07-13: the 'Add Fee' button is ENABLED on an empty form (validation happens on submit, not by disabling) — BUG-FD-4. Expected kept as the intended behavior; tester will see the button enabled. | STAGING VIU 2026-07-20 staging LIVE VIU: BUG-FD-4 FIXED on staging: Add Fee button is DISABLED on an empty form (was enabled on qb). Live-observed (dev-wo-emptyform, disabled=true). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7146,6 +7917,11 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
           <t>20% of 170.76 (=34.15) capped at Max 15 -&gt; resolved exactly 15 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). The '$ Max Amount (Optional)' field appears only after a percentage method is chosen (confirmed live). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7188,6 +7964,11 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
           <t>confirm label 'Add Fee' observed; Type-flip re-observed in batch-1 (not re-driven) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7230,6 +8011,11 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
           <t>UI BLOCKS empty name (inline 'Name' required, dialog stays open, nothing saved). NOTE NEW FDBUG-16: the RAW API now ACCEPTS an empty-name adjustment (201; was 400 in batch-3) — BE validation regression, FE still guards | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). (Note: the raw back-end will accept an empty name — FDBUG-16 — but the on-screen dialog blocks it, which is what a manual tester sees.) | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7272,6 +8058,11 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
           <t>amount 0 -&gt; 400 at API; UI validates on submit | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7314,6 +8105,11 @@
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
           <t>discount 150% -&gt; 400 'A percentage discount cannot exceed 100%.'; fee 150% -&gt; 201 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7356,6 +8152,11 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
           <t>pct_subtotal resolves on the WO subtotal EXCLUDING whole-WO adjustments (10% of 182.76-sub -&gt; 17.08 = 10% of 170.76 line total) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Calculation Type options confirmed live (exactly the 4 listed; no '% of Grand Total'). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7398,6 +8199,11 @@
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
           <t>add on Invoiced WO -&gt; 409 'Adjustments cannot be changed on an invoiced or paid work order.'; edit also 409 | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7440,6 +8246,11 @@
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
           <t>'Enter an amount to see the impact.' prompt present in the re-driven dialog | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Exact prompt text 'Enter an amount to see the impact.' confirmed live (shot wo-03). | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7482,6 +8293,11 @@
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
           <t>preview row '+$5.00' with new-subtotal line re-observed; color/sign convention from batch-1 (not re-checked) | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). Kept to sign only; the exact fee/discount colours were not re-captured this pass. | SV-8479/8480 deconfliction 2026-07-22: label sweep: navigation labels -&gt; 'Add Work Order Fee / Discount' / 'New Work Order Fee / Discount' (behavior/expected unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav label 'Add Work Order Fee / Discount' confirmed present in the WO toolbar ⋯ menu; case behavior unchanged. Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7524,6 +8340,11 @@
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
           <t>administration/adjustment-templates loads; Finance-only user has NO F&amp;D nav, FINANCE=Payment Methods only, direct route bounces to /workorders. viu_status VIU-Verified re-confirmed. Ev build/fees-discounts/viu-sv8456-2026-07-22/ (01-settings-landing, 02-new-dialog, 03-customer-fd-tab, SVC-*, FIN-*).</t>
         </is>
       </c>
@@ -7566,6 +8387,11 @@
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
           <t>. | VIU 2026-07-22 LIVE: part-row ⋮ menu = 'Move', 'Add Part Fee / Discount' (label correct; opens part fee/discount dialog). 'Return' state-gated — the seeded part was 'Auth To Order' (not received) so Return was not offered; Return appears only for returnable parts. Ev: wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
@@ -7608,6 +8434,11 @@
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
           <t>s a mockup. QA passed on staging 2026-07-22 (✅). | VIU 2026-07-22 LIVE: Work Order Fees &amp; Discounts card shows disclaimer exactly 'Applies to the whole work order, after all other fees &amp; discounts.' below the adjustment list. Ev: wo/FD-FIN-004-FD-WO-021-card-financialinfo.png, wo/lines-bodytext.txt.</t>
         </is>
       </c>
@@ -7650,6 +8481,11 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
           <t>6-07-22 LIVE: toolbar ⋯ menu label 'Add Work Order Fee / Discount' correct; opens whole-WO fee/discount dialog. WORDING CORRECTED — observed order is 'Audit Log' -&gt; 'Timesheets (N)' -&gt; 'Add Work Order Fee / Discount' -&gt; 'Delete Work Order' (Add is 3rd, NOT at top). Ev: wo/FD-WO-025-toolbar-menu.png.</t>
         </is>
       </c>
@@ -7691,6 +8527,11 @@
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>No action needed — passed.</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr">
         <is>
           <t>&amp; Discounts Settings page (Settings -&gt; Service -&gt; Fees &amp; Discounts / adjustment-templates) — it is NOT rendered inside the WO fee/discount dialogs. Ev: wo/labor-dialog-text.txt, wo/part-dialog-text.txt, wo/wo-dialog-text.txt, wo/FD-WO-028-settings-convenience-banner.png, wo/settings-fd-bodytext.txt.</t>
         </is>
@@ -7876,7 +8717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7886,7 +8727,8 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7927,6 +8769,11 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Fresh Evidence / Note</t>
         </is>
       </c>
@@ -7969,6 +8816,11 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>Same Processing Fee amount problem — the base wrongly includes the whole-work-order fees/discounts. A developer needs to fix it; re-test the amount once fixed.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-2 CONFIRMED AGAIN (clean discriminator): pfee base INCLUDES whole-WO adjustments + their tax (3% -&gt; 0.63 where spec expects 0.00). Structural defect is tax-model independent | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-2): the Processing Fee base wrongly includes whole-work-order fees/discounts (should exclude them). Build labels applied. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. The SV-8456 UI-correction wording + Settings-&gt;Service permission pivot were re-confirmed live on the current staging build (Service-user sees+manages F&amp;D; Finance-only user no F&amp;D nav, direct route bounces to /workorders; Tech restored to Technician 50bf6a0d + verified; ZZAUTOTEST roles deleted). This case retains its prior VIU-Deviation for its OWN (non-SV-8456) reason — that specific behavior was NOT re-driven this pass. Ev build/fees-discounts/viu-sv8456-2026-07-22/.</t>
         </is>
       </c>
@@ -8011,6 +8863,11 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Re-check on staging how a Processing Fee template's type is shown in the customer picker, and confirm with the team whether showing it as 'Fee' is acceptable or needs fixing.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>accepted deviation (PO Q6=A); list assertions hold; case-update pending | WORDING+VIU 2026-07-13: DEVIATION carried: a Processing Fee template appears in the customer picker with its Type shown as 'Fee' (display quirk). Picker label 'Fee / Discount Templates' confirmed live; the Processing-Fee-as-Fee display not re-captured this run.</t>
         </is>
       </c>
@@ -8053,6 +8910,11 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>Accepted as-is by the team — the picker shows 'No results' when there is nothing left to add. Update the test case wording to expect 'No results'; no developer fix needed.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>'No results' empty picker message per batch-1 (spec wording differs); case-update pending; not re-driven | WORDING+VIU 2026-07-13: Empty-picker state carried from prior VIU (not re-captured — the shared env has templates available).</t>
         </is>
       </c>
@@ -8095,6 +8957,11 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>A developer needs to add the 'Show N more' collapse so a line with two or more fees/discounts no longer shows them all at once. Re-test once fixed.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>CONFIRMED AGAIN: 2 adjustments on one part render with NO 'Show N more' collapse — PO Q5=B defect persists | WORDING+VIU 2026-07-13: DEVIATION carried (BUG-FD-5): no 'Show N more' collapse — a line/part with 2+ fees/discounts shows all of them. Not re-driven with a 3-adjustment line this run.</t>
         </is>
       </c>
@@ -8137,6 +9004,11 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>The system only hides the option on the screen — it still allows the change in the background. Ask the team whether the system should also block it in the background, then re-test.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
           <t>BUG-FD-3 stands on batch evidence; NOT re-testable today — Technician role drifted on the shared env (now HAS workOrdersCreateAndEdit, so its 201 is legitimate); enforcement-depth question unchanged (dev decision) | WORDING+VIU 2026-07-13: DEVIATION (BUG-FD-3): the whole-work-order add/edit/remove hide is front-end only — the back-end does not block the write. NOT re-testable this run: Technician drifted to HAVE Work Orders: Create &amp; Edit, and only admin/tech can log in.</t>
         </is>
       </c>
@@ -8179,6 +9051,11 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>The menu still offers an 'Edit' option for a Processing Fee even though editing does nothing (only 'Remove' works). A developer needs to make it remove-only. Re-test once fixed.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>BE re-proven: pfee change -&gt; 409 'cannot be edited through this endpoint', remove -&gt; 204; card still offers Edit per batch-1 (S8-N5 UI drift) | WORDING+VIU 2026-07-13: DEVIATION carried: the ⋮ menu still shows 'Edit' for a Processing Fee but it is inert (cannot edit a pfee on the WO); 'Remove' works. Build labels ('Remove Fee / Discount' confirm). | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. The SV-8456 UI-correction wording + Settings-&gt;Service permission pivot were re-confirmed live on the current staging build (Service-user sees+manages F&amp;D; Finance-only user no F&amp;D nav, direct route bounces to /workorders; Tech restored to Technician 50bf6a0d + verified; ZZAUTOTEST roles deleted). This case retains its prior VIU-Deviation for its OWN (non-SV-8456) reason — that specific behavior was NOT re-driven this pass. Ev build/fees-discounts/viu-sv8456-2026-07-22/.</t>
         </is>
       </c>
@@ -8221,6 +9098,11 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>A developer needs to fix the Processing Fee amount — its base should NOT include the whole-work-order fees/discounts (or their tax). Re-test the amount once fixed.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-2 CONFIRMED AGAIN with a clean discriminator: on a WO whose ONLY money is a whole-WO $20 taxable fee, 3% pfee resolved 0.63 (=3% of 21.00 incl the whole-WO fee + its tax); spec base must EXCLUDE whole-WO adjustments -&gt; expected 0.00 | WORDING+VIU 2026-07-13: DEVIATION carried (FDBUG-2): the Processing Fee base wrongly includes whole-WO fees/discounts + their tax (should exclude them).</t>
         </is>
       </c>
@@ -8263,6 +9145,11 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>A developer needs to change the Statistics tab to show one row per fee/discount that names its target. Re-test once that per-row layout is built.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>per-row scope hyperlink impossible while the layout is aggregate (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: Stats F&amp;D rows show the name only — no scope hyperlink to the target. Confirmed live (rows read plain names, shot fin-01).</t>
         </is>
       </c>
@@ -8305,6 +9192,11 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>Once the Statistics tab shows one row per fee/discount, check they are listed oldest first. Re-test after the per-row layout is built by the developer.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
           <t>creation-order rows blocked by aggregate layout (dep. FD-STATS-001) | WORDING+VIU 2026-07-13: DEVIATION carried: creation-order ruling pending (BUG-FD-2 group). Labels cleaned.</t>
         </is>
       </c>
@@ -8347,6 +9239,11 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>The line-level dialog currently has no 'Apply From Template' picker, so template scoping can't be checked there. Re-check on staging whether that picker now exists; if it is still missing, confirm with the team whether that is intended.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
           <t>FDBUG-13 (line-scope Add dialog has no template picker) per batch-1/4; not re-driven today | WORDING+VIU 2026-07-13: DEVIATION carried: template scoping in the line 'Apply From Template' picker + the compatibility hint not re-captured this run (needs the line-level picker). Labels cleaned. | SV-8479/8480 deconfliction 2026-07-22: mixed label sweep: labor step -&gt; 'Add Labor Fee / Discount', part step -&gt; 'Add Part Fee / Discount' (behavior unchanged). | VIU 2026-07-22 LIVE: SV-8479 nav labels 'Add Labor Fee / Discount' (step 1) and 'Add Part Fee / Discount' (step 3) both confirmed present; case status unchanged (existing Deviation for its own reason). Ev: wo/FD-WO-017-labor-menu-open.png, wo/FD-WO-018-part-menu.png.</t>
         </is>
       </c>
@@ -8389,6 +9286,11 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>The option is only hidden on the screen — the system still lets the change go through behind the scenes. Ask the team whether the system should also block it in the background, not just hide the button, then re-test.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>BUG-FD-3 stands on prior evidence; NOT re-testable today: the shared-env Technician role was CHANGED (now includes workOrdersCreateAndEdit+workOrdersDelete, 8 perms vs matrix 6) so tech's 201 is now legitimate; no login lacking the perm exists | WORDING+VIU 2026-07-13: rewritten to exact build labels (⋮ menu item 'Add Fee/Discount'; dialog 'Add new fee/discount'; fields 'Apply From Template'/'Name'/'Type'/'Calculation Type'/'$ Amount' or 'Percent %'/'$ Max Amount (Optional)'/'Taxable' toggle; whole-WO Calculation Type options = Flat Amount, % of Labor Total, % of Parts Total, % of Subtotal; buttons 'Add Fee'/'Add Discount'; sidebar card 'WO Fees &amp; Discounts'; preview empty prompt 'Enter an amount to see the impact.'). Captured live on WO S3-15960 (shots wo-01..wo-05). DEVIATION (BUG-FD-3: the hide is front-end only; the back-end does not block the write). NOT re-testable this run — the Technician role has drifted on the shared qb env; re-derive the roles matrix before re-checking. | SV-8479/8480 deconfliction 2026-07-22: label updated 'Add Fee/Discount' -&gt; 'Add Work Order Fee / Discount' (item 10); permission behavior unchanged. | VIU 2026-07-22 LIVE: toolbar label 'Add Work Order Fee / Discount' confirmed present (admin); permission-negative status unchanged — role-negative not re-driven this UI batch.</t>
         </is>
       </c>
@@ -8430,6 +9332,11 @@
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>A developer needs to move the three-dot menu to the LEFT of 'Unassigned' (it currently sits on the right); the label is already correct. Re-test the left placement once the fix is in.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>me row y=282); spec requires LEFT. Label 'Add Labor Fee / Discount' is correct and opens the labor fee/discount dialog. Menu contained only 'Add Labor Fee / Discount' (no separate 'Edit labor' item observed). Ev: wo/FD-WO-017-labor-row-menu-RIGHT.png, wo/FD-WO-017-labor-menu-open.png, obs2 geometry.</t>
         </is>
@@ -8460,7 +9367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8470,7 +9377,8 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8510,6 +9418,11 @@
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Fresh Evidence / Note</t>
         </is>
@@ -8526,7 +9439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8536,7 +9449,8 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8577,6 +9491,11 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Fresh Evidence / Note</t>
         </is>
       </c>
@@ -8619,6 +9538,11 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company to check the penny-rounding on discount lines. Test once QuickBooks is connected.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>floor half RE-PROVEN (stacked 120+100 on 182.76 -&gt; sub 0.00, excess 37.24 exact); QB penny-cap half needs QB-side line view | WORDING+VIU 2026-07-13: BLOCKED-ENV: the QuickBooks penny-cap (largest-remainder) allocation on discount lines is only observable inside QuickBooks (no QB read API; export currently fails on duplicate document numbers). The in-app $0.00 floor half is verified. Build labels applied.</t>
         </is>
       </c>
@@ -8661,6 +9585,11 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Needs an environment with the Fees &amp; Discounts feature turned OFF (it can't be toggled on the shared one). Test when that is available.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>re flag is ON at the org level on the SHARED staging org (d55bc308); toggling it OFF org-wide during an unattended run would strip F&amp;D from all users and break concurrent/later VIU batches, and no separate flag-off org is available. Not inferred — needs a dedicated flag-off org/state to verify live.</t>
         </is>
       </c>
@@ -8703,6 +9632,11 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>Needs a window where the Fees &amp; Discounts feature can be turned off. Test when that is available.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>org flag toggling deliberately NOT done: shared env, manual tester active today | WORDING+VIU 2026-07-13: BLOCKED-ENV: cannot take a feature-off window on the shared qb env while a manual tester is active. Wording made layman. | V1_3 (2026-07-17): Δ2 — Story 10 renamed 'history log' -&gt; 'audit log' (terminology only; gates/behavior/status unchanged). Notes-only touch: the reader-facing text of this case already uses the exact build labels ('Audit Log' ⋮ menu / 'Work Order Log' page) and carries no generic history-log prose. The internal `area`/section name is left as-is (TestRail section rename not authorized).</t>
         </is>
       </c>
@@ -8745,6 +9679,11 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>Needs a window where the Fees &amp; Discounts feature can be turned off. Test when that is available.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>as FD-FLAG-001 | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: BLOCKED-ENV + V1_2 re-VIU pending: needs a feature-off window (not takeable on the shared env) to confirm history entries stay visible. Wording made layman. | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -8787,6 +9726,11 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>Needs a window where the Fees &amp; Discounts feature can be turned off. Test when that is available.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
           <t>as FD-FLAG-001; the flag-ON half of the AND-gate is fresh-proven (FD-PERM-010) | WORDING+VIU 2026-07-13: BLOCKED-ENV (permission half): the See-Financial-Data masking half is established, but the full both-gates check needs a restricted-role login — re-run after the roles matrix is re-derived. Wording made layman.</t>
         </is>
       </c>
@@ -8829,6 +9773,11 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>Needs a window where the Fees &amp; Discounts feature can be turned off (it can't be toggled on the shared environment). Test when that is available.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>feature-flag OFF window deliberately not taken on the shared env (manual tester active today) | V1_2 (2026-07-13): history-log gate updated per S13-R10 — WO-level history requires Work Orders: Create and Edit; line-level history requires Work Order Lines: Create and Edit (was View History Logs). Expected/preconditions updated; needs live re-VIU. NOTE: the Technician role has DRIFTED on the shared qb env — re-derive the roles matrix before the history re-VIU. | WORDING+VIU 2026-07-13: BLOCKED-ENV: needs a feature-off window (not takeable on the shared env with a live tester). | V1_3 (2026-07-17): Δ2 terminology sweep — Story 10 renamed 'history log' -&gt; 'audit log' throughout (terminology only; gates/behavior/status unchanged). Generic 'history log / history entry / work-order history' prose replaced with 'audit log / audit-log entry'; the exact build labels 'Audit Log' (⋮ menu) and 'Work Order Log' (page) kept per Standing Rule 9. TestRail section name left as-is (rename not authorized).</t>
         </is>
       </c>
@@ -8871,6 +9820,11 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>QB invoice line internals unobservable (no read API; export of re-invoiced WOs fails on duplicate doc numbers) — needs QB-UI eyeball of a cleanly synced invoice | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the QuickBooks invoice line-item internals are only visible inside QuickBooks (no QB read API; and re-invoiced work orders currently fail to export on duplicate document numbers) — a human logged into QuickBooks is needed to confirm. Observable today: adjustment-item-mapping-status = QuickBooks connected + Fee item mapped + Discount item mapped (checked live).</t>
         </is>
       </c>
@@ -8913,6 +9867,11 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>as FD-QB-001 — needs QB UI (generic Fee/Discount item + description=name) | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the QuickBooks invoice line-item internals are only visible inside QuickBooks (no QB read API; and re-invoiced work orders currently fail to export on duplicate document numbers) — a human logged into QuickBooks is needed to confirm. Observable today: adjustment-item-mapping-status = QuickBooks connected + Fee item mapped + Discount item mapped (checked live).</t>
         </is>
       </c>
@@ -8955,6 +9914,11 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
           <t>as FD-QB-001 — $0-line skip only visible QB-side | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the QuickBooks invoice line-item internals are only visible inside QuickBooks (no QB read API; and re-invoiced work orders currently fail to export on duplicate document numbers) — a human logged into QuickBooks is needed to confirm. Observable today: adjustment-item-mapping-status = QuickBooks connected + Fee item mapped + Discount item mapped (checked live).</t>
         </is>
       </c>
@@ -8997,6 +9961,11 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
           <t>unmap not achievable today: PUT bookkeeping/settings {settings:{feeItemId:null}} -&gt; 500 (requestId 4bd14847); flat payload -&gt; 400 'settings missing'. Mapping stayed connected+mapped (verified). Guard cycle needs a working unmap (dev/QB-side) | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the mapping-guard block cannot be driven — the two items are currently mapped and the unmap call (PUT /api/bookkeeping/settings) 500s on this env, so an unmapped state can't be created. The guard's data source (connected/feeItemMapped/discountItemMapped) is observable and all true.</t>
         </is>
       </c>
@@ -9039,6 +10008,11 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>as FD-QB-004 (unmap 500) | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the mapping-guard block cannot be driven — the two items are currently mapped and the unmap call (PUT /api/bookkeeping/settings) 500s on this env, so an unmapped state can't be created. The guard's data source (connected/feeItemMapped/discountItemMapped) is observable and all true.</t>
         </is>
       </c>
@@ -9081,6 +10055,11 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
           <t>as FD-QB-004 (unmap 500) | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the mapping-guard block cannot be driven — the two items are currently mapped and the unmap call (PUT /api/bookkeeping/settings) 500s on this env, so an unmapped state can't be created. The guard's data source (connected/feeItemMapped/discountItemMapped) is observable and all true.</t>
         </is>
       </c>
@@ -9123,6 +10102,11 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
           <t>as FD-QB-004 (unmap 500) | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the mapping-guard block cannot be driven — the two items are currently mapped and the unmap call (PUT /api/bookkeeping/settings) 500s on this env, so an unmapped state can't be created. The guard's data source (connected/feeItemMapped/discountItemMapped) is observable and all true.</t>
         </is>
       </c>
@@ -9165,6 +10149,11 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
           <t>as FD-QB-004; positive half (template create while MAPPED) works throughout | WORDING+VIU 2026-07-13: Observable half CONFIRMED live: creating a non-auto-apply template is always allowed (template create 201). The 'no block when QuickBooks not connected' half is Blocked-Env — QuickBooks is connected here and cannot be disconnected on the shared env.</t>
         </is>
       </c>
@@ -9207,6 +10196,11 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company; the unmap action also currently errors on this environment. Test once QuickBooks is connected and that is working.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>unexported-items list + retry + mark-done endpoints re-exercised (mark-done 200 on my entries); the unmap-in-flight repro blocked by the unmap 500 | WORDING+VIU 2026-07-13:  BLOCKED-ENV: cannot unmap an in-use item — the unmap call 500s on this env — so the route-to-Unexported-Items behavior can't be driven. (The Unexported Items list itself is reachable and returns data.)</t>
         </is>
       </c>
@@ -9249,6 +10243,11 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>Class application only visible QB-side | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the QuickBooks invoice line-item internals are only visible inside QuickBooks (no QB read API; and re-invoiced work orders currently fail to export on duplicate document numbers) — a human logged into QuickBooks is needed to confirm. Observable today: adjustment-item-mapping-status = QuickBooks connected + Fee item mapped + Discount item mapped (checked live).</t>
         </is>
       </c>
@@ -9291,6 +10290,11 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
           <t>stale-Class abort only reproducible QB-side | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the QuickBooks invoice line-item internals are only visible inside QuickBooks (no QB read API; and re-invoiced work orders currently fail to export on duplicate document numbers) — a human logged into QuickBooks is needed to confirm. Observable today: adjustment-item-mapping-status = QuickBooks connected + Fee item mapped + Discount item mapped (checked live).</t>
         </is>
       </c>
@@ -9333,6 +10337,11 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
           <t>penny-cap allocation of discount LINES only visible on QB invoice lines | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the largest-remainder penny allocation on the QuickBooks discount lines is only visible inside QuickBooks (same as FD-CALC-017). The in-app $0.00 floor half is verified.</t>
         </is>
       </c>
@@ -9375,6 +10384,11 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
           <t>IN-APP HALF VERIFIED TODAY: invoicing the over-discounted WO recorded a CUSTOMER CREDIT (unpaid-transactions 2-&gt;4; 'current' bucket -11.63 -&gt; -119.73 = +9.14 invoice &amp; -117.24 credit exactly). QB goodwill-memo half unobservable: invoice export fails on the duplicate-doc-number env bug, no credit_memo export fired, no QB read API — needs QB UI on a cleanly synced org | WORDING+VIU 2026-07-13: In-app customer-credit half VERIFIED 2026-07-10 (invoicing an over-discounted WO recorded a customer credit of exactly the excess). BLOCKED-ENV: the QuickBooks tax-exempt goodwill credit-memo half needs a human in QuickBooks (export fails on duplicate document numbers; no QB read API).</t>
         </is>
       </c>
@@ -9417,6 +10431,11 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
+          <t>Needs a QuickBooks-connected company. Test this in QuickBooks once that is available.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
           <t>tax code on the QB line unobservable in-app; in-app taxable base shifts re-proven (FD-CALC-011) | WORDING+VIU 2026-07-13:  BLOCKED-ENV: the QuickBooks invoice line-item internals are only visible inside QuickBooks (no QB read API; and re-invoiced work orders currently fail to export on duplicate document numbers) — a human logged into QuickBooks is needed to confirm. Observable today: adjustment-item-mapping-status = QuickBooks connected + Fee item mapped + Discount item mapped (checked live).</t>
         </is>
       </c>
@@ -9458,6 +10477,11 @@
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Needs an environment where the template library can be emptied (the shared one always has templates). Test the empty-state message when that is available.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>empty-state needs deleting ALL location templates — not acceptable on the shared env (3 real templates present; manual tester active) | WORDING+VIU 2026-07-13: BLOCKED-ENV: the empty-state message cannot be seen — the shared env's template list is never empty (needs a location with zero templates). Nav corrected to Finance. | SV-8456 (2026-07-21 staging LIVE VIU): F&amp;D moved to SETTINGS→SERVICE (below Canned Lines); template/WO/Part-sale/customer dialogs now show Taxable as a Yes/No DROPDOWN (was toggle); Auto-apply is a CHECKBOX with a 'When on…' caption; settings &amp; customer tables are plain-text/left-aligned (no badges); WO sidebar card retitled 'Work Order Fees &amp; Discounts' and renders ABOVE Financial Info; Part-sale card 'Parts Sale Fees &amp; Discounts' above Financial Info. Permission gate pivoted Settings→Finance → Settings→Service (verified live: Service-user sees+manages F&amp;D &amp; convenience toggle; Finance-only user has no F&amp;D nav item and /administration/adjustment-templates bounces to /workorders). Frontend-only; functionality + calc INTACT. | RE-VIU 2026-07-22 LIVE (Batch 4, SV-8456 re-verify): access-check quick-login {admin} HTTP 200. The SV-8456 UI-correction wording + Settings-&gt;Service permission pivot were re-confirmed live on the current staging build (Service-user sees+manages F&amp;D; Finance-only user no F&amp;D nav, direct route bounces to /workorders; Tech restored to Technician 50bf6a0d + verified; ZZAUTOTEST roles deleted). This case retains its prior VIU-Blocked-Env for its OWN (non-SV-8456) reason — that specific behavior was NOT re-driven this pass. Ev build/fees-discounts/viu-sv8456-2026-07-22/.</t>
         </is>
@@ -9497,7 +10521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9507,7 +10531,8 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9548,6 +10573,11 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
+          <t>What needs to be done (plain)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Fresh Evidence / Note</t>
         </is>
       </c>
@@ -9589,6 +10619,11 @@
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Re-test on staging once a part can be moved from requested to received (this was blocked by an environment error before). Check the fee/discount stays attached after the part is received.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>STILL PENDING: requested-&gt;received transition unreachable — line-create 500s env-wide, make-request rejected on completed lines, receiving subsystem needs a fresh order | WORDING+VIU 2026-07-13: BLOCKED/PENDING: requested→received transition blocked by the env-wide WO line-create 500 + completed-line part-request lock — cannot drive the transition. Build labels applied.</t>
         </is>

</xml_diff>